<commit_message>
Conclui charter científico FT-001
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R3ce7794f69024b05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Racc1e375121645a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rd8874763e8584d9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Red02bcbb023a49e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -501,7 +501,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -512,7 +512,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -523,7 +523,7 @@
         <x:color rgb="FF17365D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAF7"/>
         </x:patternFill>
       </x:fill>
@@ -534,7 +534,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -724,7 +724,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2c6ff1346c2f4d25"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R83a32998c0f044c1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1016,7 +1016,7 @@
       </x:c>
       <x:c r="E5" s="9" t="n">
         <x:f>COUNTIF(Atividades!$G$5:$G$52,"Concluído")</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F5" s="50"/>
       <x:c r="G5" s="8" t="str">
@@ -1024,7 +1024,7 @@
       </x:c>
       <x:c r="H5" s="10" t="n">
         <x:f>E5/B5</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.2708333333333333</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -1067,7 +1067,7 @@
       </x:c>
       <x:c r="B9" s="53" t="n">
         <x:f>COUNTIF(Atividades!$G$5:$G$52,A9)</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C9" s="50"/>
       <x:c r="D9" s="50"/>
@@ -1082,7 +1082,7 @@
       </x:c>
       <x:c r="B10" s="55" t="n">
         <x:f>COUNTIF(Atividades!$G$5:$G$52,A10)</x:f>
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C10" s="50"/>
       <x:c r="D10" s="50"/>
@@ -1352,7 +1352,7 @@
     <x:mergeCell ref="A29:H30"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49ef37620c3e458e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9b80d901b8b4be1"/>
 </x:worksheet>
 </file>
 
@@ -1449,13 +1449,13 @@
         <x:v>Revisar e aprovar o charter; registrar o que a plataforma pode e não pode afirmar; nomear responsáveis pelas portas científicas.</x:v>
       </x:c>
       <x:c r="G5" s="84" t="str">
-        <x:v>Parcial</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
       <x:c r="H5" s="81" t="str">
-        <x:v>PLANEJAMENTO_MESTRE.md e limites científicos já documentados; não há registro de aprovação formal nem responsáveis nomeados.</x:v>
+        <x:v>docs/CHARTER_FT_001.md v1.0: propósito, independência, escopo LTFT/HTFT, fronteiras de evidência, exclusões e matriz de decisão aprovados por Allan Maia em 2026-10-12.</x:v>
       </x:c>
       <x:c r="I5" s="81" t="str">
-        <x:v>Aprovar o charter e registrar responsáveis por produto, ciência, dados e operação.</x:v>
+        <x:v>Controlar alterações por nova versão, análise de impacto e aprovação explícita; concluir os demais requisitos da porta G0 separadamente.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
@@ -2839,7 +2839,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15f9855b4d6e430d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c643abeb9174130"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Implementa unidades canônicas FT-003
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rd8874763e8584d9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Red02bcbb023a49e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R58109e1bbfa54cec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rddfea38bfd9d447b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -724,7 +724,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R83a32998c0f044c1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R995d5f6803554bf2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1016,7 +1016,7 @@
       </x:c>
       <x:c r="E5" s="9" t="n">
         <x:f>COUNTIF(Atividades!$G$5:$G$52,"Concluído")</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F5" s="50"/>
       <x:c r="G5" s="8" t="str">
@@ -1024,7 +1024,7 @@
       </x:c>
       <x:c r="H5" s="10" t="n">
         <x:f>E5/B5</x:f>
-        <x:v>0.2708333333333333</x:v>
+        <x:v>0.2916666666666667</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -1067,7 +1067,7 @@
       </x:c>
       <x:c r="B9" s="53" t="n">
         <x:f>COUNTIF(Atividades!$G$5:$G$52,A9)</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C9" s="50"/>
       <x:c r="D9" s="50"/>
@@ -1082,7 +1082,7 @@
       </x:c>
       <x:c r="B10" s="55" t="n">
         <x:f>COUNTIF(Atividades!$G$5:$G$52,A10)</x:f>
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C10" s="50"/>
       <x:c r="D10" s="50"/>
@@ -1352,7 +1352,7 @@
     <x:mergeCell ref="A29:H30"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9b80d901b8b4be1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a8c74811cd34474"/>
 </x:worksheet>
 </file>
 
@@ -1507,13 +1507,13 @@
         <x:v>Definir catálogo de unidades, conversões, precisão, validações dimensionais e conservação das unidades originais.</x:v>
       </x:c>
       <x:c r="G7" s="85" t="str">
-        <x:v>Parcial</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
       <x:c r="H7" s="82" t="str">
-        <x:v>CONTRATO_V1.md e campos com sufixos canônicos; validações numéricas existem, mas não há catálogo/conversor completo.</x:v>
+        <x:v>src/plataforma_ltft/units.py e docs/UNIDADES_CANONICAS.md: catálogo 1.0.0, 10 grandezas, preservação da unidade original e 9 testes específicos; suíte completa com 41 testes aprovada.</x:v>
       </x:c>
       <x:c r="I7" s="82" t="str">
-        <x:v>Criar módulo de unidades e testes de conversão para todas as grandezas do contrato v2.</x:v>
+        <x:v>Versionar qualquer mudança de definição; integrar normalização em novos fluxos de ingestão sem reinterpretar silenciosamente dados legados.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
@@ -2839,7 +2839,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c643abeb9174130"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Race8ff57e9ed4164"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Conclui contrato de catalisador FT-005
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R58109e1bbfa54cec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rddfea38bfd9d447b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Re78d9125f9584352"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R4fa52351d1ca4871"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -724,7 +724,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R995d5f6803554bf2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7f5362f5d7cc45fa"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1016,7 +1016,7 @@
       </x:c>
       <x:c r="E5" s="9" t="n">
         <x:f>COUNTIF(Atividades!$G$5:$G$52,"Concluído")</x:f>
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F5" s="50"/>
       <x:c r="G5" s="8" t="str">
@@ -1024,7 +1024,7 @@
       </x:c>
       <x:c r="H5" s="10" t="n">
         <x:f>E5/B5</x:f>
-        <x:v>0.2916666666666667</x:v>
+        <x:v>0.3125</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -1067,7 +1067,7 @@
       </x:c>
       <x:c r="B9" s="53" t="n">
         <x:f>COUNTIF(Atividades!$G$5:$G$52,A9)</x:f>
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C9" s="50"/>
       <x:c r="D9" s="50"/>
@@ -1082,7 +1082,7 @@
       </x:c>
       <x:c r="B10" s="55" t="n">
         <x:f>COUNTIF(Atividades!$G$5:$G$52,A10)</x:f>
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C10" s="50"/>
       <x:c r="D10" s="50"/>
@@ -1352,7 +1352,7 @@
     <x:mergeCell ref="A29:H30"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a8c74811cd34474"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe49ce20bd82419c"/>
 </x:worksheet>
 </file>
 
@@ -1565,13 +1565,13 @@
         <x:v>Criar entidade/schema próprio para lote, precursor, suporte, promotor, carga, preparação, ativação e caracterização.</x:v>
       </x:c>
       <x:c r="G9" s="85" t="str">
-        <x:v>Parcial</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
       <x:c r="H9" s="82" t="str">
-        <x:v>LTFTCase já contém família, fase hipotética, suporte, carga, promotor, precursor e ativação; falta contrato dedicado e lote/caracterização.</x:v>
+        <x:v>ft-catalyst-v1.schema.json, catalyst.py, CONTRATO_CATALISADOR_V1.md e exemplos Co/Fe/Co-Fe: lote, preparação, ativação, fase e proveniência validados; suíte completa com 49 testes aprovada.</x:v>
       </x:c>
       <x:c r="I9" s="82" t="str">
-        <x:v>Criar catalyst-v1.schema.json e exemplos de Co, Fe e sistema exploratório.</x:v>
+        <x:v>Integrar o catalyst_id/batch_id aos futuros registros experimentais e manter caracterizações como evidências referenciadas, sem promover hipóteses a medições.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -2839,7 +2839,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Race8ff57e9ed4164"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ae28640bfa0466a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Prioriza modernizacao UX no planejamento
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Re78d9125f9584352"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R4fa52351d1ca4871"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Ree40c1513e614d37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Ra2975cc19fcc4dfa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,11 +14,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
+    <x:numFmt numFmtId="202" formatCode="General"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="24">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -77,8 +78,84 @@
       <x:color rgb="FF222222"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF17312A"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF4B625B"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF17312A"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF245C2C"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF2C4C72"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF735A00"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF8A2424"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF17312A"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17312A"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17312A"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FF17312A"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="13"/>
+      <x:color rgb="FF17312A"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF6B5200"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="55">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -100,8 +177,258 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF176B55"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4F0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE5F0FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEFD8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7EEF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7D7D7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF176B55"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F1ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF245D78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF176B55"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F1ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF245D78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF176B55"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F1ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF245D78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF176B55"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F1ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF245D78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF176B55"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F1ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF245D78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF176B55"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F1ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF245D78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF176B55"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F1ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF245D78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1C7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="18">
+  <x:borders count="24">
     <x:border>
       <x:left/>
       <x:right/>
@@ -292,11 +619,93 @@
       <x:bottom/>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFFFFFFF"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFFFFFFF"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFFFFFFF"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFFFFFFF"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD8E4DF"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD8E4DF"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD8E4DF"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E4DF"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB8CEC5"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB8CEC5"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB8CEC5"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB8CEC5"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9B95B"/>
+      </x:left>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFD9B95B"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9B95B"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFD9B95B"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9B95B"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFD9B95B"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9B95B"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9B95B"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="87">
+  <x:cellXfs count="422">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -489,6 +898,807 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="8" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="11" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="11" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="11" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="11" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="12" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="12" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="12" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="12" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="19" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="13" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="13" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="15" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="15" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="19" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="22" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="22" fillId="15" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="22" fillId="15" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="13" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="17" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="17" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="17" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="17" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="17" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="18" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="18" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="18" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="18" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="18" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="18" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="18" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="18" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="18" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="19" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="22" fillId="19" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="19" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="19" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="19" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="19" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="19" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="19" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="19" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="19" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="19" fillId="19" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="19" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="19" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="19" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="21" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="21" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="19" fillId="21" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="22" fillId="21" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="23" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="23" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="23" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="23" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="24" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="24" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="24" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="24" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="24" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="24" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="27" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="27" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="27" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="22" fillId="27" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="25" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="29" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="29" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="30" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="30" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="30" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="30" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="30" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="30" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="30" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="30" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="30" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="29" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="21" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="12" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="22" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="22" fillId="33" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="22" fillId="33" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="22" fillId="33" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="22" fillId="33" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="31" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="35" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="35" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="36" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="36" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="36" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="36" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="36" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="36" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="35" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="21" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="12" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="22" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="22" fillId="39" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="22" fillId="39" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="22" fillId="39" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="22" fillId="39" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="37" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="41" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="41" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="42" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="42" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="42" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="42" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="42" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="42" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="42" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="42" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="42" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="41" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="21" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="12" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="22" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="22" fillId="45" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="22" fillId="45" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="22" fillId="45" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="22" fillId="45" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="43" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="47" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="47" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="48" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="48" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="48" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="48" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="48" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="48" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="48" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="48" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="48" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="47" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="21" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="12" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="22" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="22" fillId="51" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="22" fillId="51" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="22" fillId="51" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="22" fillId="51" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="49" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="53" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="53" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="18" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="54" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="54" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="54" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="23" fillId="54" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="54" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="54" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="54" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="54" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="23" fillId="54" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="53" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="9" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -543,199 +1753,8 @@
 </x:styleSheet>
 </file>
 
-<file path=xl/drawings/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:r>
-              <a:rPr sz="900">
-                <a:latin typeface="Arial"/>
-                <a:ea typeface="Arial"/>
-                <a:cs typeface="Arial"/>
-              </a:rPr>
-              <a:t>Atividades por status</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-      <c:txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr>
-            <a:defRPr sz="900">
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:defRPr>
-          </a:pPr>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:plotArea>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>Quantidade</c:v>
-          </c:tx>
-          <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Resumo'!$A$9:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="0"/>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Resumo'!$B$9:$B$12</c:f>
-              <c:numCache>
-                <c:formatCode>0</c:formatCode>
-                <c:ptCount val="0"/>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:axId val="48650112"/>
-        <c:axId val="48672768"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="48650112"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="CCCCCC"/>
-              </a:solidFill>
-              <a:prstDash val="dash"/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr sz="750">
-                <a:latin typeface="Arial"/>
-                <a:ea typeface="Arial"/>
-                <a:cs typeface="Arial"/>
-              </a:defRPr>
-            </a:pPr>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="48672768"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="48672768"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="CCCCCC"/>
-              </a:solidFill>
-              <a:prstDash val="dash"/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="0" sourceLinked="0"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr sz="750">
-                <a:latin typeface="Arial"/>
-                <a:ea typeface="Arial"/>
-                <a:cs typeface="Arial"/>
-              </a:defRPr>
-            </a:pPr>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="48650112"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-  </c:chart>
-  <c:spPr>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-      <a:solidFill>
-        <a:srgbClr val="D9D9D9"/>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-    </a:ln>
-  </c:spPr>
-</c:chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="1" name="Chart"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
-        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7f5362f5d7cc45fa"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ActivitiesTable" displayName="ActivitiesTable" ref="A4:I52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:I52"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogFT" displayName="BacklogFT" ref="A4:I60" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Prioridade"/>
@@ -949,389 +1968,383 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="3" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="3" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="66" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="4" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="20" customHeight="1">
-      <x:c r="A1" s="50"/>
-      <x:c r="B1" s="50"/>
-      <x:c r="C1" s="50"/>
-      <x:c r="D1" s="50"/>
-      <x:c r="E1" s="50"/>
-      <x:c r="F1" s="50"/>
-      <x:c r="G1" s="50"/>
-      <x:c r="H1" s="50"/>
+      <x:c r="A1" s="387"/>
+      <x:c r="B1" s="387"/>
+      <x:c r="C1" s="387"/>
+      <x:c r="D1" s="387"/>
+      <x:c r="E1" s="387"/>
+      <x:c r="F1" s="387"/>
+      <x:c r="G1" s="387"/>
+      <x:c r="H1" s="387"/>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
-      <x:c r="A2" s="2" t="str">
+      <x:c r="A2" s="388" t="str">
         <x:v>Atividades da Plataforma Reação Fischer–Tropsch</x:v>
       </x:c>
-      <x:c r="B2" s="2"/>
-      <x:c r="C2" s="2"/>
-      <x:c r="D2" s="2"/>
-      <x:c r="E2" s="2"/>
-      <x:c r="F2" s="2"/>
-      <x:c r="G2" s="2"/>
-      <x:c r="H2" s="2"/>
+      <x:c r="B2" s="388"/>
+      <x:c r="C2" s="388"/>
+      <x:c r="D2" s="388"/>
+      <x:c r="E2" s="388"/>
+      <x:c r="F2" s="388"/>
+      <x:c r="G2" s="388"/>
+      <x:c r="H2" s="388"/>
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
-      <x:c r="A3" s="51" t="str">
-        <x:v>Situação verificada no repositório principal em 2026-10-12</x:v>
-      </x:c>
-      <x:c r="B3" s="51"/>
-      <x:c r="C3" s="51"/>
-      <x:c r="D3" s="51"/>
-      <x:c r="E3" s="51"/>
-      <x:c r="F3" s="51"/>
-      <x:c r="G3" s="51"/>
-      <x:c r="H3" s="51"/>
+      <x:c r="A3" s="389" t="str">
+        <x:v>Situação verificada no repositório principal em 2026-10-13</x:v>
+      </x:c>
+      <x:c r="B3" s="389"/>
+      <x:c r="C3" s="389"/>
+      <x:c r="D3" s="389"/>
+      <x:c r="E3" s="389"/>
+      <x:c r="F3" s="389"/>
+      <x:c r="G3" s="389"/>
+      <x:c r="H3" s="389"/>
     </x:row>
     <x:row r="4" ht="20" customHeight="1">
-      <x:c r="A4" s="50"/>
-      <x:c r="B4" s="50"/>
-      <x:c r="C4" s="50"/>
-      <x:c r="D4" s="50"/>
-      <x:c r="E4" s="50"/>
-      <x:c r="F4" s="50"/>
-      <x:c r="G4" s="50"/>
-      <x:c r="H4" s="50"/>
+      <x:c r="A4" s="387"/>
+      <x:c r="B4" s="387"/>
+      <x:c r="C4" s="387"/>
+      <x:c r="D4" s="387"/>
+      <x:c r="E4" s="387"/>
+      <x:c r="F4" s="387"/>
+      <x:c r="G4" s="387"/>
+      <x:c r="H4" s="387"/>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
-      <x:c r="A5" s="8" t="str">
+      <x:c r="A5" s="393" t="str">
         <x:v>Total de atividades</x:v>
       </x:c>
-      <x:c r="B5" s="9" t="n">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="C5" s="50"/>
-      <x:c r="D5" s="8" t="str">
+      <x:c r="B5" s="398" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="C5" s="387"/>
+      <x:c r="D5" s="393" t="str">
         <x:v>Concluídas</x:v>
       </x:c>
-      <x:c r="E5" s="9" t="n">
-        <x:f>COUNTIF(Atividades!$G$5:$G$52,"Concluído")</x:f>
+      <x:c r="E5" s="398" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F5" s="50"/>
-      <x:c r="G5" s="8" t="str">
+      <x:c r="F5" s="387"/>
+      <x:c r="G5" s="393" t="str">
         <x:v>Progresso concluído</x:v>
       </x:c>
-      <x:c r="H5" s="10" t="n">
-        <x:f>E5/B5</x:f>
-        <x:v>0.3125</x:v>
+      <x:c r="H5" s="399" t="n">
+        <x:v>0.26785714285714285</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
-      <x:c r="A6" s="50"/>
-      <x:c r="B6" s="50"/>
-      <x:c r="C6" s="50"/>
-      <x:c r="D6" s="50"/>
-      <x:c r="E6" s="50"/>
-      <x:c r="F6" s="50"/>
-      <x:c r="G6" s="50"/>
-      <x:c r="H6" s="50"/>
+      <x:c r="A6" s="387"/>
+      <x:c r="B6" s="387"/>
+      <x:c r="C6" s="387"/>
+      <x:c r="D6" s="387"/>
+      <x:c r="E6" s="387"/>
+      <x:c r="F6" s="387"/>
+      <x:c r="G6" s="387"/>
+      <x:c r="H6" s="387"/>
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
-      <x:c r="A7" s="50"/>
-      <x:c r="B7" s="50"/>
-      <x:c r="C7" s="50"/>
-      <x:c r="D7" s="50"/>
-      <x:c r="E7" s="50"/>
-      <x:c r="F7" s="50"/>
-      <x:c r="G7" s="50"/>
-      <x:c r="H7" s="50"/>
+      <x:c r="A7" s="387"/>
+      <x:c r="B7" s="387"/>
+      <x:c r="C7" s="387"/>
+      <x:c r="D7" s="387"/>
+      <x:c r="E7" s="387"/>
+      <x:c r="F7" s="387"/>
+      <x:c r="G7" s="387"/>
+      <x:c r="H7" s="387"/>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
-      <x:c r="A8" s="14" t="str">
+      <x:c r="A8" s="403" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B8" s="14" t="str">
+      <x:c r="B8" s="403" t="str">
         <x:v>Quantidade</x:v>
       </x:c>
-      <x:c r="C8" s="50"/>
-      <x:c r="D8" s="50"/>
-      <x:c r="E8" s="50"/>
-      <x:c r="F8" s="50"/>
-      <x:c r="G8" s="50"/>
-      <x:c r="H8" s="50"/>
+      <x:c r="C8" s="387"/>
+      <x:c r="D8" s="387"/>
+      <x:c r="E8" s="387"/>
+      <x:c r="F8" s="387"/>
+      <x:c r="G8" s="387"/>
+      <x:c r="H8" s="387"/>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
-      <x:c r="A9" s="52" t="str">
+      <x:c r="A9" s="405" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="B9" s="53" t="n">
-        <x:f>COUNTIF(Atividades!$G$5:$G$52,A9)</x:f>
+      <x:c r="B9" s="406" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C9" s="50"/>
-      <x:c r="D9" s="50"/>
-      <x:c r="E9" s="50"/>
-      <x:c r="F9" s="50"/>
-      <x:c r="G9" s="50"/>
-      <x:c r="H9" s="50"/>
+      <x:c r="C9" s="387"/>
+      <x:c r="D9" s="387"/>
+      <x:c r="E9" s="387"/>
+      <x:c r="F9" s="387"/>
+      <x:c r="G9" s="387"/>
+      <x:c r="H9" s="387"/>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
-      <x:c r="A10" s="54" t="str">
+      <x:c r="A10" s="405" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="B10" s="55" t="n">
-        <x:f>COUNTIF(Atividades!$G$5:$G$52,A10)</x:f>
+      <x:c r="B10" s="406" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C10" s="50"/>
-      <x:c r="D10" s="50"/>
-      <x:c r="E10" s="50"/>
-      <x:c r="F10" s="50"/>
-      <x:c r="G10" s="50"/>
-      <x:c r="H10" s="50"/>
+      <x:c r="C10" s="387"/>
+      <x:c r="D10" s="387"/>
+      <x:c r="E10" s="387"/>
+      <x:c r="F10" s="387"/>
+      <x:c r="G10" s="387"/>
+      <x:c r="H10" s="387"/>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
-      <x:c r="A11" s="54" t="str">
+      <x:c r="A11" s="405" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="B11" s="55" t="n">
-        <x:f>COUNTIF(Atividades!$G$5:$G$52,A11)</x:f>
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C11" s="50"/>
-      <x:c r="D11" s="50"/>
-      <x:c r="E11" s="50"/>
-      <x:c r="F11" s="50"/>
-      <x:c r="G11" s="50"/>
-      <x:c r="H11" s="50"/>
+      <x:c r="B11" s="406" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C11" s="387"/>
+      <x:c r="D11" s="387"/>
+      <x:c r="E11" s="387"/>
+      <x:c r="F11" s="387"/>
+      <x:c r="G11" s="387"/>
+      <x:c r="H11" s="387"/>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
-      <x:c r="A12" s="56" t="str">
+      <x:c r="A12" s="405" t="str">
         <x:v>Bloqueado</x:v>
       </x:c>
-      <x:c r="B12" s="57" t="n">
-        <x:f>COUNTIF(Atividades!$G$5:$G$52,A12)</x:f>
+      <x:c r="B12" s="406" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C12" s="50"/>
-      <x:c r="D12" s="50"/>
-      <x:c r="E12" s="50"/>
-      <x:c r="F12" s="50"/>
-      <x:c r="G12" s="50"/>
-      <x:c r="H12" s="50"/>
+      <x:c r="C12" s="387"/>
+      <x:c r="D12" s="387"/>
+      <x:c r="E12" s="387"/>
+      <x:c r="F12" s="387"/>
+      <x:c r="G12" s="387"/>
+      <x:c r="H12" s="387"/>
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
-      <x:c r="A13" s="50"/>
-      <x:c r="B13" s="50"/>
-      <x:c r="C13" s="50"/>
-      <x:c r="D13" s="50"/>
-      <x:c r="E13" s="50"/>
-      <x:c r="F13" s="50"/>
-      <x:c r="G13" s="50"/>
-      <x:c r="H13" s="50"/>
+      <x:c r="A13" s="387"/>
+      <x:c r="B13" s="387"/>
+      <x:c r="C13" s="387"/>
+      <x:c r="D13" s="387"/>
+      <x:c r="E13" s="387"/>
+      <x:c r="F13" s="387"/>
+      <x:c r="G13" s="387"/>
+      <x:c r="H13" s="387"/>
     </x:row>
     <x:row r="14" ht="20" customHeight="1">
-      <x:c r="A14" s="50"/>
-      <x:c r="B14" s="50"/>
-      <x:c r="C14" s="50"/>
-      <x:c r="D14" s="50"/>
-      <x:c r="E14" s="50"/>
-      <x:c r="F14" s="50"/>
-      <x:c r="G14" s="50"/>
-      <x:c r="H14" s="50"/>
-    </x:row>
-    <x:row r="15" ht="20" customHeight="1">
-      <x:c r="A15" s="58" t="str">
+      <x:c r="A14" s="387"/>
+      <x:c r="B14" s="387"/>
+      <x:c r="C14" s="387"/>
+      <x:c r="D14" s="387"/>
+      <x:c r="E14" s="387"/>
+      <x:c r="F14" s="387"/>
+      <x:c r="G14" s="387"/>
+      <x:c r="H14" s="387"/>
+    </x:row>
+    <x:row r="15" ht="26" customHeight="1">
+      <x:c r="A15" s="391" t="str">
         <x:v>Leitura do status</x:v>
       </x:c>
-      <x:c r="B15" s="58"/>
-      <x:c r="C15" s="58"/>
-      <x:c r="D15" s="58"/>
-      <x:c r="E15" s="58"/>
-      <x:c r="F15" s="58"/>
-      <x:c r="G15" s="58"/>
-      <x:c r="H15" s="58"/>
-    </x:row>
-    <x:row r="16" ht="20" customHeight="1">
-      <x:c r="A16" s="59" t="str">
+      <x:c r="B15" s="391"/>
+      <x:c r="C15" s="387"/>
+      <x:c r="D15" s="387"/>
+      <x:c r="E15" s="387"/>
+      <x:c r="F15" s="387"/>
+      <x:c r="G15" s="387"/>
+      <x:c r="H15" s="387"/>
+    </x:row>
+    <x:row r="16" ht="28" customHeight="1">
+      <x:c r="A16" s="419" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="B16" s="60" t="str">
+      <x:c r="B16" s="419" t="str">
         <x:v>Existe implementação e evidência verificável no repositório.</x:v>
       </x:c>
-      <x:c r="C16" s="50"/>
-      <x:c r="D16" s="50"/>
-      <x:c r="E16" s="50"/>
-      <x:c r="F16" s="50"/>
-      <x:c r="G16" s="50"/>
-      <x:c r="H16" s="50"/>
-    </x:row>
-    <x:row r="17" ht="20" customHeight="1">
-      <x:c r="A17" s="59" t="str">
+      <x:c r="C16" s="387"/>
+      <x:c r="D16" s="387"/>
+      <x:c r="E16" s="387"/>
+      <x:c r="F16" s="387"/>
+      <x:c r="G16" s="387"/>
+      <x:c r="H16" s="387"/>
+    </x:row>
+    <x:row r="17" ht="28" customHeight="1">
+      <x:c r="A17" s="419" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="B17" s="60" t="str">
+      <x:c r="B17" s="419" t="str">
         <x:v>Há base implementada, mas faltam entregáveis ou critérios de aceite.</x:v>
       </x:c>
-      <x:c r="C17" s="50"/>
-      <x:c r="D17" s="50"/>
-      <x:c r="E17" s="50"/>
-      <x:c r="F17" s="50"/>
-      <x:c r="G17" s="50"/>
-      <x:c r="H17" s="50"/>
-    </x:row>
-    <x:row r="18" ht="20" customHeight="1">
-      <x:c r="A18" s="59" t="str">
+      <x:c r="C17" s="387"/>
+      <x:c r="D17" s="387"/>
+      <x:c r="E17" s="387"/>
+      <x:c r="F17" s="387"/>
+      <x:c r="G17" s="387"/>
+      <x:c r="H17" s="387"/>
+    </x:row>
+    <x:row r="18" ht="28" customHeight="1">
+      <x:c r="A18" s="419" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="B18" s="60" t="str">
+      <x:c r="B18" s="419" t="str">
         <x:v>A atividade está documentada, sem implementação verificável.</x:v>
       </x:c>
-      <x:c r="C18" s="50"/>
-      <x:c r="D18" s="50"/>
-      <x:c r="E18" s="50"/>
-      <x:c r="F18" s="50"/>
-      <x:c r="G18" s="50"/>
-      <x:c r="H18" s="50"/>
-    </x:row>
-    <x:row r="19" ht="20" customHeight="1">
-      <x:c r="A19" s="59" t="str">
+      <x:c r="C18" s="387"/>
+      <x:c r="D18" s="387"/>
+      <x:c r="E18" s="387"/>
+      <x:c r="F18" s="387"/>
+      <x:c r="G18" s="387"/>
+      <x:c r="H18" s="387"/>
+    </x:row>
+    <x:row r="19" ht="28" customHeight="1">
+      <x:c r="A19" s="419" t="str">
         <x:v>Bloqueado</x:v>
       </x:c>
-      <x:c r="B19" s="60" t="str">
+      <x:c r="B19" s="419" t="str">
         <x:v>Depende de evidência, aprovação, infraestrutura ou etapa anterior.</x:v>
       </x:c>
-      <x:c r="C19" s="50"/>
-      <x:c r="D19" s="50"/>
-      <x:c r="E19" s="50"/>
-      <x:c r="F19" s="50"/>
-      <x:c r="G19" s="50"/>
-      <x:c r="H19" s="50"/>
+      <x:c r="C19" s="387"/>
+      <x:c r="D19" s="387"/>
+      <x:c r="E19" s="387"/>
+      <x:c r="F19" s="387"/>
+      <x:c r="G19" s="387"/>
+      <x:c r="H19" s="387"/>
     </x:row>
     <x:row r="20" ht="20" customHeight="1">
-      <x:c r="A20" s="50"/>
-      <x:c r="B20" s="50"/>
-      <x:c r="C20" s="50"/>
-      <x:c r="D20" s="50"/>
-      <x:c r="E20" s="50"/>
-      <x:c r="F20" s="50"/>
-      <x:c r="G20" s="50"/>
-      <x:c r="H20" s="50"/>
+      <x:c r="A20" s="420"/>
+      <x:c r="B20" s="420"/>
+      <x:c r="C20" s="387"/>
+      <x:c r="D20" s="387"/>
+      <x:c r="E20" s="387"/>
+      <x:c r="F20" s="387"/>
+      <x:c r="G20" s="387"/>
+      <x:c r="H20" s="387"/>
     </x:row>
     <x:row r="21" ht="20" customHeight="1">
-      <x:c r="A21" s="50"/>
-      <x:c r="B21" s="50"/>
-      <x:c r="C21" s="50"/>
-      <x:c r="D21" s="50"/>
-      <x:c r="E21" s="50"/>
-      <x:c r="F21" s="50"/>
-      <x:c r="G21" s="50"/>
-      <x:c r="H21" s="50"/>
-    </x:row>
-    <x:row r="22" ht="20" customHeight="1">
-      <x:c r="A22" s="58" t="str">
+      <x:c r="A21" s="420"/>
+      <x:c r="B21" s="420"/>
+      <x:c r="C21" s="387"/>
+      <x:c r="D21" s="387"/>
+      <x:c r="E21" s="387"/>
+      <x:c r="F21" s="387"/>
+      <x:c r="G21" s="387"/>
+      <x:c r="H21" s="387"/>
+    </x:row>
+    <x:row r="22" ht="26" customHeight="1">
+      <x:c r="A22" s="421" t="str">
         <x:v>Fontes usadas na classificação</x:v>
       </x:c>
-      <x:c r="B22" s="58"/>
-      <x:c r="C22" s="58"/>
-      <x:c r="D22" s="58"/>
-      <x:c r="E22" s="58"/>
-      <x:c r="F22" s="58"/>
-      <x:c r="G22" s="58"/>
-      <x:c r="H22" s="58"/>
-    </x:row>
-    <x:row r="23" ht="20" customHeight="1">
-      <x:c r="A23" s="59" t="str">
+      <x:c r="B22" s="421"/>
+      <x:c r="C22" s="387"/>
+      <x:c r="D22" s="387"/>
+      <x:c r="E22" s="387"/>
+      <x:c r="F22" s="387"/>
+      <x:c r="G22" s="387"/>
+      <x:c r="H22" s="387"/>
+    </x:row>
+    <x:row r="23" ht="28" customHeight="1">
+      <x:c r="A23" s="419" t="str">
         <x:v>Planejamento</x:v>
       </x:c>
-      <x:c r="B23" s="60" t="str">
-        <x:v>PLANEJAMENTO_MESTRE.md e docs/BACKLOG_INICIAL.md</x:v>
-      </x:c>
-      <x:c r="C23" s="50"/>
-      <x:c r="D23" s="50"/>
-      <x:c r="E23" s="50"/>
-      <x:c r="F23" s="50"/>
-      <x:c r="G23" s="50"/>
-      <x:c r="H23" s="50"/>
-    </x:row>
-    <x:row r="24" ht="20" customHeight="1">
-      <x:c r="A24" s="59" t="str">
+      <x:c r="B23" s="419" t="str">
+        <x:v>PLANEJAMENTO_MESTRE.md, PLANEJAMENTO.md e docs/BACKLOG_INICIAL.md</x:v>
+      </x:c>
+      <x:c r="C23" s="387"/>
+      <x:c r="D23" s="387"/>
+      <x:c r="E23" s="387"/>
+      <x:c r="F23" s="387"/>
+      <x:c r="G23" s="387"/>
+      <x:c r="H23" s="387"/>
+    </x:row>
+    <x:row r="24" ht="28" customHeight="1">
+      <x:c r="A24" s="419" t="str">
         <x:v>Contratos</x:v>
       </x:c>
-      <x:c r="B24" s="60" t="str">
+      <x:c r="B24" s="419" t="str">
         <x:v>schemas/, docs/CONTRATO_V1.md e docs/CONTRATO_V2.md</x:v>
       </x:c>
-      <x:c r="C24" s="50"/>
-      <x:c r="D24" s="50"/>
-      <x:c r="E24" s="50"/>
-      <x:c r="F24" s="50"/>
-      <x:c r="G24" s="50"/>
-      <x:c r="H24" s="50"/>
-    </x:row>
-    <x:row r="25" ht="20" customHeight="1">
-      <x:c r="A25" s="59" t="str">
+      <x:c r="C24" s="387"/>
+      <x:c r="D24" s="387"/>
+      <x:c r="E24" s="387"/>
+      <x:c r="F24" s="387"/>
+      <x:c r="G24" s="387"/>
+      <x:c r="H24" s="387"/>
+    </x:row>
+    <x:row r="25" ht="28" customHeight="1">
+      <x:c r="A25" s="419" t="str">
         <x:v>Implementação</x:v>
       </x:c>
-      <x:c r="B25" s="60" t="str">
+      <x:c r="B25" s="419" t="str">
         <x:v>src/plataforma_ltft/, app.py, tools/ e examples/</x:v>
       </x:c>
-      <x:c r="C25" s="50"/>
-      <x:c r="D25" s="50"/>
-      <x:c r="E25" s="50"/>
-      <x:c r="F25" s="50"/>
-      <x:c r="G25" s="50"/>
-      <x:c r="H25" s="50"/>
-    </x:row>
-    <x:row r="26" ht="20" customHeight="1">
-      <x:c r="A26" s="59" t="str">
+      <x:c r="C25" s="387"/>
+      <x:c r="D25" s="387"/>
+      <x:c r="E25" s="387"/>
+      <x:c r="F25" s="387"/>
+      <x:c r="G25" s="387"/>
+      <x:c r="H25" s="387"/>
+    </x:row>
+    <x:row r="26" ht="28" customHeight="1">
+      <x:c r="A26" s="419" t="str">
         <x:v>Validação</x:v>
       </x:c>
-      <x:c r="B26" s="60" t="str">
-        <x:v>tests/ — 32 testes aprovados na auditoria</x:v>
-      </x:c>
-      <x:c r="C26" s="50"/>
-      <x:c r="D26" s="50"/>
-      <x:c r="E26" s="50"/>
-      <x:c r="F26" s="50"/>
-      <x:c r="G26" s="50"/>
-      <x:c r="H26" s="50"/>
-    </x:row>
-    <x:row r="27" ht="20" customHeight="1">
-      <x:c r="A27" s="59" t="str">
+      <x:c r="B26" s="419" t="str">
+        <x:v>tests/ — 53 testes aprovados na verificação de 2026-10-13</x:v>
+      </x:c>
+      <x:c r="C26" s="387"/>
+      <x:c r="D26" s="387"/>
+      <x:c r="E26" s="387"/>
+      <x:c r="F26" s="387"/>
+      <x:c r="G26" s="387"/>
+      <x:c r="H26" s="387"/>
+    </x:row>
+    <x:row r="27" ht="28" customHeight="1">
+      <x:c r="A27" s="419" t="str">
         <x:v>Publicação</x:v>
       </x:c>
-      <x:c r="B27" s="60" t="str">
+      <x:c r="B27" s="419" t="str">
         <x:v>GitHub reacao-fischer-tropsch e protótipo Streamlit público</x:v>
       </x:c>
-      <x:c r="C27" s="50"/>
-      <x:c r="D27" s="50"/>
-      <x:c r="E27" s="50"/>
-      <x:c r="F27" s="50"/>
-      <x:c r="G27" s="50"/>
-      <x:c r="H27" s="50"/>
+      <x:c r="C27" s="387"/>
+      <x:c r="D27" s="387"/>
+      <x:c r="E27" s="387"/>
+      <x:c r="F27" s="387"/>
+      <x:c r="G27" s="387"/>
+      <x:c r="H27" s="387"/>
     </x:row>
     <x:row r="28" ht="20" customHeight="1">
-      <x:c r="A28" s="50"/>
-      <x:c r="B28" s="50"/>
-      <x:c r="C28" s="50"/>
-      <x:c r="D28" s="50"/>
-      <x:c r="E28" s="50"/>
-      <x:c r="F28" s="50"/>
-      <x:c r="G28" s="50"/>
-      <x:c r="H28" s="50"/>
-    </x:row>
-    <x:row r="29" ht="26" customHeight="1">
-      <x:c r="A29" s="41" t="str">
-        <x:v>Observação: o status descreve o estado verificado dos artefatos. Planejamento ou publicação isolados não equivalem a validação científica, homologação ou produção.</x:v>
-      </x:c>
-      <x:c r="B29" s="42"/>
-      <x:c r="C29" s="42"/>
-      <x:c r="D29" s="42"/>
-      <x:c r="E29" s="42"/>
-      <x:c r="F29" s="42"/>
-      <x:c r="G29" s="42"/>
-      <x:c r="H29" s="43"/>
+      <x:c r="A28" s="387"/>
+      <x:c r="B28" s="387"/>
+      <x:c r="C28" s="387"/>
+      <x:c r="D28" s="387"/>
+      <x:c r="E28" s="387"/>
+      <x:c r="F28" s="387"/>
+      <x:c r="G28" s="387"/>
+      <x:c r="H28" s="387"/>
+    </x:row>
+    <x:row r="29" ht="42" customHeight="1">
+      <x:c r="A29" s="416" t="str">
+        <x:v>Observação: FT-049 a FT-056 formam a fase prioritária de modernização UX/UI. O backlog científico anterior é retomado após o aceite de FT-056. Planejamento ou publicação isolados não equivalem a validação científica, homologação ou produção.</x:v>
+      </x:c>
+      <x:c r="B29" s="417"/>
+      <x:c r="C29" s="417"/>
+      <x:c r="D29" s="417"/>
+      <x:c r="E29" s="417"/>
+      <x:c r="F29" s="417"/>
+      <x:c r="G29" s="417"/>
+      <x:c r="H29" s="418"/>
     </x:row>
     <x:row r="30" ht="26" customHeight="1">
       <x:c r="A30" s="44"/>
@@ -1345,14 +2358,11 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A3:H3"/>
-    <x:mergeCell ref="A15:H15"/>
-    <x:mergeCell ref="A22:H22"/>
-    <x:mergeCell ref="A29:H30"/>
+    <x:mergeCell ref="A15:B15"/>
+    <x:mergeCell ref="A22:B22"/>
+    <x:mergeCell ref="A29:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe49ce20bd82419c"/>
 </x:worksheet>
 </file>
 
@@ -1363,1461 +2373,1693 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="27" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="43" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="56" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="29" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="52" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="55" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="50" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="62" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="54" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2">
-      <x:c r="A2" s="1" t="str">
+      <x:c r="A2" s="87" t="str">
         <x:v>Backlog auditado da Plataforma Reação Fischer–Tropsch</x:v>
       </x:c>
-      <x:c r="B2" s="1"/>
-      <x:c r="C2" s="1"/>
-      <x:c r="D2" s="1"/>
-      <x:c r="E2" s="1"/>
-      <x:c r="F2" s="1"/>
-      <x:c r="G2" s="1"/>
-      <x:c r="H2" s="1"/>
-      <x:c r="I2" s="1"/>
+      <x:c r="B2" s="87"/>
+      <x:c r="C2" s="87"/>
+      <x:c r="D2" s="87"/>
+      <x:c r="E2" s="87"/>
+      <x:c r="F2" s="87"/>
+      <x:c r="G2" s="87"/>
+      <x:c r="H2" s="87"/>
+      <x:c r="I2" s="87"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="3" t="str">
+      <x:c r="A3" s="88" t="str">
         <x:v>Status baseado em artefatos existentes no repositório; atualize a coluna Status após cada entrega e registre a nova evidência.</x:v>
       </x:c>
-      <x:c r="B3" s="3"/>
-      <x:c r="C3" s="3"/>
-      <x:c r="D3" s="3"/>
-      <x:c r="E3" s="3"/>
-      <x:c r="F3" s="3"/>
-      <x:c r="G3" s="3"/>
-      <x:c r="H3" s="3"/>
-      <x:c r="I3" s="3"/>
+      <x:c r="B3" s="88"/>
+      <x:c r="C3" s="88"/>
+      <x:c r="D3" s="88"/>
+      <x:c r="E3" s="88"/>
+      <x:c r="F3" s="88"/>
+      <x:c r="G3" s="88"/>
+      <x:c r="H3" s="88"/>
+      <x:c r="I3" s="88"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
-      <x:c r="A4" s="71" t="str">
+      <x:c r="A4" s="92" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B4" s="72" t="str">
+      <x:c r="B4" s="92" t="str">
         <x:v>Prioridade</x:v>
       </x:c>
-      <x:c r="C4" s="72" t="str">
+      <x:c r="C4" s="92" t="str">
         <x:v>Fase</x:v>
       </x:c>
-      <x:c r="D4" s="72" t="str">
+      <x:c r="D4" s="92" t="str">
         <x:v>Atividade</x:v>
       </x:c>
-      <x:c r="E4" s="72" t="str">
+      <x:c r="E4" s="92" t="str">
         <x:v>Objetivo</x:v>
       </x:c>
-      <x:c r="F4" s="72" t="str">
+      <x:c r="F4" s="92" t="str">
         <x:v>O que se faz</x:v>
       </x:c>
-      <x:c r="G4" s="72" t="str">
+      <x:c r="G4" s="92" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H4" s="72" t="str">
+      <x:c r="H4" s="92" t="str">
         <x:v>Evidência verificada</x:v>
       </x:c>
-      <x:c r="I4" s="73" t="str">
+      <x:c r="I4" s="92" t="str">
         <x:v>Próxima ação</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="54" customHeight="1">
-      <x:c r="A5" s="84" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>FT-001</x:v>
       </x:c>
-      <x:c r="B5" s="84" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="C5" s="84" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Fundação</x:v>
       </x:c>
-      <x:c r="D5" s="81" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>Charter e fronteira científica</x:v>
       </x:c>
-      <x:c r="E5" s="81" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>Formalizar propósito, escopo, exclusões, responsáveis e critérios de decisão.</x:v>
       </x:c>
-      <x:c r="F5" s="81" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>Revisar e aprovar o charter; registrar o que a plataforma pode e não pode afirmar; nomear responsáveis pelas portas científicas.</x:v>
       </x:c>
-      <x:c r="G5" s="84" t="str">
+      <x:c r="G5" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H5" s="81" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>docs/CHARTER_FT_001.md v1.0: propósito, independência, escopo LTFT/HTFT, fronteiras de evidência, exclusões e matriz de decisão aprovados por Allan Maia em 2026-10-12.</x:v>
       </x:c>
-      <x:c r="I5" s="81" t="str">
+      <x:c r="I5" s="97" t="str">
         <x:v>Controlar alterações por nova versão, análise de impacto e aprovação explícita; concluir os demais requisitos da porta G0 separadamente.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
-      <x:c r="A6" s="85" t="str">
+      <x:c r="A6" s="98" t="str">
         <x:v>FT-002</x:v>
       </x:c>
-      <x:c r="B6" s="85" t="str">
+      <x:c r="B6" s="98" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="C6" s="85" t="str">
+      <x:c r="C6" s="98" t="str">
         <x:v>Fundação</x:v>
       </x:c>
-      <x:c r="D6" s="82" t="str">
+      <x:c r="D6" s="98" t="str">
         <x:v>Taxonomia LTFT/HTFT</x:v>
       </x:c>
-      <x:c r="E6" s="82" t="str">
+      <x:c r="E6" s="98" t="str">
         <x:v>Separar regimes para evitar transferência indevida de modelos e evidências.</x:v>
       </x:c>
-      <x:c r="F6" s="82" t="str">
+      <x:c r="F6" s="98" t="str">
         <x:v>Versionar envelopes LTFT, transição e HTFT; exigir justificativa na transição; testar as fronteiras de temperatura.</x:v>
       </x:c>
-      <x:c r="G6" s="85" t="str">
+      <x:c r="G6" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H6" s="82" t="str">
+      <x:c r="H6" s="98" t="str">
         <x:v>Contrato v2, ESCOPO_LTFT_HTFT.md, classify_ft_regime e testes em 260/280 °C.</x:v>
       </x:c>
-      <x:c r="I6" s="82" t="str">
+      <x:c r="I6" s="98" t="str">
         <x:v>Manter versionamento do envelope e revisar quando houver evidência aprovada.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
-      <x:c r="A7" s="85" t="str">
+      <x:c r="A7" s="97" t="str">
         <x:v>FT-003</x:v>
       </x:c>
-      <x:c r="B7" s="85" t="str">
+      <x:c r="B7" s="97" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="C7" s="85" t="str">
+      <x:c r="C7" s="97" t="str">
         <x:v>Fundação</x:v>
       </x:c>
-      <x:c r="D7" s="82" t="str">
+      <x:c r="D7" s="97" t="str">
         <x:v>Unidades canônicas</x:v>
       </x:c>
-      <x:c r="E7" s="82" t="str">
+      <x:c r="E7" s="97" t="str">
         <x:v>Padronizar entrada, armazenamento e comparação de grandezas.</x:v>
       </x:c>
-      <x:c r="F7" s="82" t="str">
+      <x:c r="F7" s="97" t="str">
         <x:v>Definir catálogo de unidades, conversões, precisão, validações dimensionais e conservação das unidades originais.</x:v>
       </x:c>
-      <x:c r="G7" s="85" t="str">
+      <x:c r="G7" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H7" s="82" t="str">
+      <x:c r="H7" s="97" t="str">
         <x:v>src/plataforma_ltft/units.py e docs/UNIDADES_CANONICAS.md: catálogo 1.0.0, 10 grandezas, preservação da unidade original e 9 testes específicos; suíte completa com 41 testes aprovada.</x:v>
       </x:c>
-      <x:c r="I7" s="82" t="str">
+      <x:c r="I7" s="97" t="str">
         <x:v>Versionar qualquer mudança de definição; integrar normalização em novos fluxos de ingestão sem reinterpretar silenciosamente dados legados.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
-      <x:c r="A8" s="85" t="str">
+      <x:c r="A8" s="98" t="str">
         <x:v>FT-004</x:v>
       </x:c>
-      <x:c r="B8" s="85" t="str">
+      <x:c r="B8" s="98" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="C8" s="85" t="str">
+      <x:c r="C8" s="98" t="str">
         <x:v>Fundação</x:v>
       </x:c>
-      <x:c r="D8" s="82" t="str">
+      <x:c r="D8" s="98" t="str">
         <x:v>Contrato de caso</x:v>
       </x:c>
-      <x:c r="E8" s="82" t="str">
+      <x:c r="E8" s="98" t="str">
         <x:v>Garantir casos completos, versionados e reproduzíveis.</x:v>
       </x:c>
-      <x:c r="F8" s="82" t="str">
+      <x:c r="F8" s="98" t="str">
         <x:v>Definir schemas, campos obrigatórios e condicionais, exemplos válidos/inválidos e migração v1→v2.</x:v>
       </x:c>
-      <x:c r="G8" s="85" t="str">
+      <x:c r="G8" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H8" s="82" t="str">
+      <x:c r="H8" s="98" t="str">
         <x:v>ltft-case-v1.schema.json, ft-case-v2.schema.json, exemplos, migração explícita e testes.</x:v>
       </x:c>
-      <x:c r="I8" s="82" t="str">
+      <x:c r="I8" s="98" t="str">
         <x:v>Evoluir o v2 somente por migração versionada e ampliar campos experimentais.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
-      <x:c r="A9" s="85" t="str">
+      <x:c r="A9" s="97" t="str">
         <x:v>FT-005</x:v>
       </x:c>
-      <x:c r="B9" s="85" t="str">
+      <x:c r="B9" s="97" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="C9" s="85" t="str">
+      <x:c r="C9" s="97" t="str">
         <x:v>Fundação</x:v>
       </x:c>
-      <x:c r="D9" s="82" t="str">
+      <x:c r="D9" s="97" t="str">
         <x:v>Contrato de catalisador</x:v>
       </x:c>
-      <x:c r="E9" s="82" t="str">
+      <x:c r="E9" s="97" t="str">
         <x:v>Representar composição, preparação, fase e proveniência sem confundir hipótese com medição.</x:v>
       </x:c>
-      <x:c r="F9" s="82" t="str">
+      <x:c r="F9" s="97" t="str">
         <x:v>Criar entidade/schema próprio para lote, precursor, suporte, promotor, carga, preparação, ativação e caracterização.</x:v>
       </x:c>
-      <x:c r="G9" s="85" t="str">
+      <x:c r="G9" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H9" s="82" t="str">
+      <x:c r="H9" s="97" t="str">
         <x:v>ft-catalyst-v1.schema.json, catalyst.py, CONTRATO_CATALISADOR_V1.md e exemplos Co/Fe/Co-Fe: lote, preparação, ativação, fase e proveniência validados; suíte completa com 49 testes aprovada.</x:v>
       </x:c>
-      <x:c r="I9" s="82" t="str">
+      <x:c r="I9" s="97" t="str">
         <x:v>Integrar o catalyst_id/batch_id aos futuros registros experimentais e manter caracterizações como evidências referenciadas, sem promover hipóteses a medições.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
-      <x:c r="A10" s="85" t="str">
+      <x:c r="A10" s="98" t="str">
         <x:v>FT-006</x:v>
       </x:c>
-      <x:c r="B10" s="85" t="str">
+      <x:c r="B10" s="98" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="C10" s="85" t="str">
+      <x:c r="C10" s="98" t="str">
         <x:v>Fundação</x:v>
       </x:c>
-      <x:c r="D10" s="82" t="str">
+      <x:c r="D10" s="98" t="str">
         <x:v>Contrato de evidência</x:v>
       </x:c>
-      <x:c r="E10" s="82" t="str">
+      <x:c r="E10" s="98" t="str">
         <x:v>Tornar cada dado rastreável e governado por licença e revisão.</x:v>
       </x:c>
-      <x:c r="F10" s="82" t="str">
+      <x:c r="F10" s="98" t="str">
         <x:v>Registrar origem, licença, método, unidade, condição, incerteza, status de revisão e hash do artefato.</x:v>
       </x:c>
-      <x:c r="G10" s="85" t="str">
+      <x:c r="G10" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H10" s="82" t="str">
+      <x:c r="H10" s="98" t="str">
         <x:v>ltft-evidence-v1.schema.json, evidence-csv-specs-v1.json, manifesto/auditoria e testes estruturais.</x:v>
       </x:c>
-      <x:c r="I10" s="82" t="str">
+      <x:c r="I10" s="98" t="str">
         <x:v>Adicionar fluxos de promoção de extraído para verificado/aprovado e responsáveis.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
-      <x:c r="A11" s="85" t="str">
+      <x:c r="A11" s="97" t="str">
         <x:v>FT-007</x:v>
       </x:c>
-      <x:c r="B11" s="85" t="str">
+      <x:c r="B11" s="97" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="C11" s="85" t="str">
+      <x:c r="C11" s="97" t="str">
         <x:v>Fundação</x:v>
       </x:c>
-      <x:c r="D11" s="82" t="str">
+      <x:c r="D11" s="97" t="str">
         <x:v>Contrato de resultado</x:v>
       </x:c>
-      <x:c r="E11" s="82" t="str">
+      <x:c r="E11" s="97" t="str">
         <x:v>Evitar que saídas sejam interpretadas além da evidência disponível.</x:v>
       </x:c>
-      <x:c r="F11" s="82" t="str">
+      <x:c r="F11" s="97" t="str">
         <x:v>Versionar resultado, regime, origem de alpha, prontidão, bloqueios e avisos científicos.</x:v>
       </x:c>
-      <x:c r="G11" s="85" t="str">
+      <x:c r="G11" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H11" s="82" t="str">
+      <x:c r="H11" s="97" t="str">
         <x:v>ltft-result-v1.schema.json, ft-result-v2.schema.json e saídas com recommendation_blocked.</x:v>
       </x:c>
-      <x:c r="I11" s="82" t="str">
+      <x:c r="I11" s="97" t="str">
         <x:v>Adicionar identificadores de dados, código e configuração usados em cada execução.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
-      <x:c r="A12" s="85" t="str">
+      <x:c r="A12" s="98" t="str">
         <x:v>FT-008</x:v>
       </x:c>
-      <x:c r="B12" s="85" t="str">
+      <x:c r="B12" s="98" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="C12" s="85" t="str">
+      <x:c r="C12" s="98" t="str">
         <x:v>Fundação</x:v>
       </x:c>
-      <x:c r="D12" s="82" t="str">
+      <x:c r="D12" s="98" t="str">
         <x:v>Worker determinístico</x:v>
       </x:c>
-      <x:c r="E12" s="82" t="str">
+      <x:c r="E12" s="98" t="str">
         <x:v>Executar casos por JSON de forma repetível e auditável.</x:v>
       </x:c>
-      <x:c r="F12" s="82" t="str">
+      <x:c r="F12" s="98" t="str">
         <x:v>Validar configuração, migrar contrato quando permitido, executar motor e gravar resultado versionado.</x:v>
       </x:c>
-      <x:c r="G12" s="85" t="str">
+      <x:c r="G12" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H12" s="82" t="str">
+      <x:c r="H12" s="98" t="str">
         <x:v>src/plataforma_ltft/worker.py, exemplos e testes ponta a ponta para LTFT, produto e HTFT.</x:v>
       </x:c>
-      <x:c r="I12" s="82" t="str">
+      <x:c r="I12" s="98" t="str">
         <x:v>Adicionar identificador de execução, hash de entrada e idempotência persistida.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
-      <x:c r="A13" s="85" t="str">
+      <x:c r="A13" s="97" t="str">
         <x:v>FT-009</x:v>
       </x:c>
-      <x:c r="B13" s="85" t="str">
+      <x:c r="B13" s="97" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="C13" s="85" t="str">
+      <x:c r="C13" s="97" t="str">
         <x:v>Fundação</x:v>
       </x:c>
-      <x:c r="D13" s="82" t="str">
+      <x:c r="D13" s="97" t="str">
         <x:v>Testes de limites</x:v>
       </x:c>
-      <x:c r="E13" s="82" t="str">
+      <x:c r="E13" s="97" t="str">
         <x:v>Prevenir regressões em regras, unidades e fronteiras científicas.</x:v>
       </x:c>
-      <x:c r="F13" s="82" t="str">
+      <x:c r="F13" s="97" t="str">
         <x:v>Cobrir casos positivos, negativos, condicionais, fronteiras de regime, schemas e bloqueios cruzados.</x:v>
       </x:c>
-      <x:c r="G13" s="85" t="str">
+      <x:c r="G13" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H13" s="82" t="str">
-        <x:v>32 testes aprovados, incluindo 260/280 °C, migração, HTFT, ASF, evidências e Streamlit.</x:v>
-      </x:c>
-      <x:c r="I13" s="82" t="str">
+      <x:c r="H13" s="97" t="str">
+        <x:v>53 testes aprovados, incluindo notebooks modulares, limites 260/280 °C, migração, HTFT, ASF, evidências e Streamlit.</x:v>
+      </x:c>
+      <x:c r="I13" s="97" t="str">
         <x:v>Adicionar CI para executar automaticamente a suíte em cada mudança.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="54" customHeight="1">
-      <x:c r="A14" s="85" t="str">
+      <x:c r="A14" s="99" t="str">
+        <x:v>FT-049</x:v>
+      </x:c>
+      <x:c r="B14" s="99" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C14" s="99" t="str">
+        <x:v>Modernização UX/UI</x:v>
+      </x:c>
+      <x:c r="D14" s="99" t="str">
+        <x:v>Fluxo guiado e navegação lateral</x:v>
+      </x:c>
+      <x:c r="E14" s="99" t="str">
+        <x:v>Orientar o usuário do produto desejado até evidências e resultados sem perder o contexto científico.</x:v>
+      </x:c>
+      <x:c r="F14" s="99" t="str">
+        <x:v>Separar a interface em etapas produto, regime, catalisador, condições, resultados e evidências; exibir progresso, pendências e estado persistente da sessão.</x:v>
+      </x:c>
+      <x:c r="G14" s="107" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="H14" s="99" t="str">
+        <x:v>Recomendação de design aprovada pelo responsável do projeto em 2026-10-13; ainda sem implementação no app.py.</x:v>
+      </x:c>
+      <x:c r="I14" s="99" t="str">
+        <x:v>Refatorar a navegação do Streamlit em componentes, mantendo src/plataforma_ltft como fonte única das regras.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="54" customHeight="1">
+      <x:c r="A15" s="99" t="str">
+        <x:v>FT-050</x:v>
+      </x:c>
+      <x:c r="B15" s="99" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C15" s="99" t="str">
+        <x:v>Modernização UX/UI</x:v>
+      </x:c>
+      <x:c r="D15" s="99" t="str">
+        <x:v>Página inicial e estado da plataforma</x:v>
+      </x:c>
+      <x:c r="E15" s="99" t="str">
+        <x:v>Apresentar finalidade, ações principais e maturidade científica antes do preenchimento do caso.</x:v>
+      </x:c>
+      <x:c r="F15" s="99" t="str">
+        <x:v>Criar abertura com Iniciar planejamento e Avaliar caso; mostrar LTFT disponível, HTFT em preparação e recomendação calibrada bloqueada.</x:v>
+      </x:c>
+      <x:c r="G15" s="107" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="H15" s="99" t="str">
+        <x:v>A interface atual abre diretamente nas abas e usa apenas título, legenda e alerta geral.</x:v>
+      </x:c>
+      <x:c r="I15" s="99" t="str">
+        <x:v>Executar após FT-049 e testar rotas de entrada sem duplicar estado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="54" customHeight="1">
+      <x:c r="A16" s="99" t="str">
+        <x:v>FT-051</x:v>
+      </x:c>
+      <x:c r="B16" s="99" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C16" s="99" t="str">
+        <x:v>Modernização UX/UI</x:v>
+      </x:c>
+      <x:c r="D16" s="99" t="str">
+        <x:v>Sistema visual, responsividade e acessibilidade</x:v>
+      </x:c>
+      <x:c r="E16" s="99" t="str">
+        <x:v>Dar identidade própria e tornar a plataforma legível em desktop e celular.</x:v>
+      </x:c>
+      <x:c r="F16" s="99" t="str">
+        <x:v>Definir cores semânticas, tipografia, espaçamento, cartões e componentes; validar contraste, teclado, textos alternativos e pontos de quebra responsivos.</x:v>
+      </x:c>
+      <x:c r="G16" s="107" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="H16" s="99" t="str">
+        <x:v>Existe tema Streamlit básico em .streamlit/config.toml, sem sistema de componentes ou verificação formal de acessibilidade.</x:v>
+      </x:c>
+      <x:c r="I16" s="99" t="str">
+        <x:v>Criar tokens visuais e componentes reutilizáveis; executar auditoria visual em desktop e celular.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="54" customHeight="1">
+      <x:c r="A17" s="99" t="str">
+        <x:v>FT-052</x:v>
+      </x:c>
+      <x:c r="B17" s="99" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C17" s="99" t="str">
+        <x:v>Modernização UX/UI</x:v>
+      </x:c>
+      <x:c r="D17" s="99" t="str">
+        <x:v>Formulário modular e validação imediata</x:v>
+      </x:c>
+      <x:c r="E17" s="99" t="str">
+        <x:v>Reduzir carga cognitiva e tornar campos, unidades e pendências compreensíveis.</x:v>
+      </x:c>
+      <x:c r="F17" s="99" t="str">
+        <x:v>Organizar produto, catalisador, reator, alimentação, condições e proveniência em blocos; incluir ajuda contextual, unidades e validação próxima do campo.</x:v>
+      </x:c>
+      <x:c r="G17" s="107" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="H17" s="99" t="str">
+        <x:v>O formulário atual reúne campos em uma única seção e valida principalmente após o envio.</x:v>
+      </x:c>
+      <x:c r="I17" s="99" t="str">
+        <x:v>Implementar depois de FT-049/FT-051 e preservar as validações do domínio.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="54" customHeight="1">
+      <x:c r="A18" s="99" t="str">
+        <x:v>FT-053</x:v>
+      </x:c>
+      <x:c r="B18" s="99" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C18" s="99" t="str">
+        <x:v>Modernização UX/UI</x:v>
+      </x:c>
+      <x:c r="D18" s="99" t="str">
+        <x:v>Painel científico de resultados</x:v>
+      </x:c>
+      <x:c r="E18" s="99" t="str">
+        <x:v>Apresentar cálculos, condições e limites em uma leitura científica integrada.</x:v>
+      </x:c>
+      <x:c r="F18" s="99" t="str">
+        <x:v>Exibir curva ASF por Cn, faixa-alvo destacada, cortes de produtos, alpha, fração-alvo, condições usadas, prontidão, avisos e limitações em áreas distintas.</x:v>
+      </x:c>
+      <x:c r="G18" s="107" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="H18" s="99" t="str">
+        <x:v>A interface atual usa gráfico de barras por faixa, uma métrica e JSON bruto de prontidão.</x:v>
+      </x:c>
+      <x:c r="I18" s="99" t="str">
+        <x:v>Criar visualização interativa sem alterar o cálculo ASF e adicionar testes de consistência dos valores exibidos.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="54" customHeight="1">
+      <x:c r="A19" s="99" t="str">
+        <x:v>FT-054</x:v>
+      </x:c>
+      <x:c r="B19" s="99" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C19" s="99" t="str">
+        <x:v>Modernização UX/UI</x:v>
+      </x:c>
+      <x:c r="D19" s="99" t="str">
+        <x:v>Maturidade visual da evidência</x:v>
+      </x:c>
+      <x:c r="E19" s="99" t="str">
+        <x:v>Impedir que resultados de naturezas diferentes pareçam equivalentes.</x:v>
+      </x:c>
+      <x:c r="F19" s="99" t="str">
+        <x:v>Exibir categorias matemático, heurístico, literatura, experimental, calibrado e bloqueado, vinculadas à proveniência e aos bloqueios já existentes.</x:v>
+      </x:c>
+      <x:c r="G19" s="107" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="H19" s="99" t="str">
+        <x:v>Os limites aparecem como texto e recommendation_blocked, mas não há componente visual uniforme de maturidade.</x:v>
+      </x:c>
+      <x:c r="I19" s="99" t="str">
+        <x:v>Mapear cada selo para estados contratuais verificáveis; não inferir maturidade pela aparência.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="54" customHeight="1">
+      <x:c r="A20" s="99" t="str">
+        <x:v>FT-055</x:v>
+      </x:c>
+      <x:c r="B20" s="99" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C20" s="99" t="str">
+        <x:v>Modernização UX/UI</x:v>
+      </x:c>
+      <x:c r="D20" s="99" t="str">
+        <x:v>Comparação de cenários</x:v>
+      </x:c>
+      <x:c r="E20" s="99" t="str">
+        <x:v>Permitir avaliar sensibilidade qualitativa sem apresentar otimização experimental indevida.</x:v>
+      </x:c>
+      <x:c r="F20" s="99" t="str">
+        <x:v>Comparar dois ou três valores de alpha, catalisadores ou condições; sobrepor curvas e mostrar diferenças, entradas, unidades, evidência e bloqueios.</x:v>
+      </x:c>
+      <x:c r="G20" s="107" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="H20" s="99" t="str">
+        <x:v>A plataforma executa um caso por vez e não mantém comparação visual entre cenários.</x:v>
+      </x:c>
+      <x:c r="I20" s="99" t="str">
+        <x:v>Executar após FT-052 a FT-054; limitar comparações às regras e evidências compatíveis.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="54" customHeight="1">
+      <x:c r="A21" s="99" t="str">
+        <x:v>FT-056</x:v>
+      </x:c>
+      <x:c r="B21" s="99" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C21" s="99" t="str">
+        <x:v>Modernização UX/UI</x:v>
+      </x:c>
+      <x:c r="D21" s="99" t="str">
+        <x:v>Aceite UX e publicação</x:v>
+      </x:c>
+      <x:c r="E21" s="99" t="str">
+        <x:v>Confirmar que a modernização funciona sem regressão científica ou operacional.</x:v>
+      </x:c>
+      <x:c r="F21" s="99" t="str">
+        <x:v>Testar fluxos, responsividade, acessibilidade, estados vazios e erros, regressão do worker, Streamlit e contratos; publicar revisão e executar teste de fumaça.</x:v>
+      </x:c>
+      <x:c r="G21" s="107" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="H21" s="99" t="str">
+        <x:v>A suíte atual tem 53 testes, mas ainda não cobre o novo fluxo de UX nem seus pontos de quebra.</x:v>
+      </x:c>
+      <x:c r="I21" s="99" t="str">
+        <x:v>Executar após FT-049 a FT-055; só então liberar a retomada do backlog científico anterior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="54" customHeight="1">
+      <x:c r="A22" s="98" t="str">
         <x:v>FT-010</x:v>
       </x:c>
-      <x:c r="B14" s="85" t="str">
+      <x:c r="B22" s="98" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="C14" s="85" t="str">
+      <x:c r="C22" s="98" t="str">
         <x:v>Fundação</x:v>
       </x:c>
-      <x:c r="D14" s="82" t="str">
+      <x:c r="D22" s="98" t="str">
         <x:v>CI mínima</x:v>
       </x:c>
-      <x:c r="E14" s="82" t="str">
+      <x:c r="E22" s="98" t="str">
         <x:v>Validar automaticamente código e schemas antes da integração.</x:v>
       </x:c>
-      <x:c r="F14" s="82" t="str">
+      <x:c r="F22" s="98" t="str">
         <x:v>Configurar workflow GitHub para testes, validação de schemas e verificação de estilo/artefatos.</x:v>
       </x:c>
-      <x:c r="G14" s="85" t="str">
+      <x:c r="G22" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H14" s="82" t="str">
+      <x:c r="H22" s="98" t="str">
         <x:v>Não existe diretório .github/workflows no repositório.</x:v>
       </x:c>
-      <x:c r="I14" s="82" t="str">
+      <x:c r="I22" s="98" t="str">
         <x:v>Criar workflow de CI para Python suportado e proteger a branch principal.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="54" customHeight="1">
-      <x:c r="A15" s="85" t="str">
+    <x:row r="23" ht="54" customHeight="1">
+      <x:c r="A23" s="97" t="str">
         <x:v>FT-011</x:v>
       </x:c>
-      <x:c r="B15" s="85" t="str">
+      <x:c r="B23" s="97" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="C15" s="85" t="str">
+      <x:c r="C23" s="97" t="str">
         <x:v>LTFT mínimo</x:v>
       </x:c>
-      <x:c r="D15" s="82" t="str">
+      <x:c r="D23" s="97" t="str">
         <x:v>Seleção de produto</x:v>
       </x:c>
-      <x:c r="E15" s="82" t="str">
+      <x:c r="E23" s="97" t="str">
         <x:v>Iniciar o planejamento pelo hidrocarboneto ou corte desejado.</x:v>
       </x:c>
-      <x:c r="F15" s="82" t="str">
+      <x:c r="F23" s="97" t="str">
         <x:v>Aceitar C1–C60, cortes padronizados e aliases; normalizar o alvo e informar limitações.</x:v>
       </x:c>
-      <x:c r="G15" s="85" t="str">
+      <x:c r="G23" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H15" s="82" t="str">
+      <x:c r="H23" s="97" t="str">
         <x:v>product_targets.py, exemplos, interface e testes de aliases, faixas e hidrocarboneto individual.</x:v>
       </x:c>
-      <x:c r="I15" s="82" t="str">
+      <x:c r="I23" s="97" t="str">
         <x:v>Adicionar base de seletividade e requisitos de upgrading por alvo.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="54" customHeight="1">
-      <x:c r="A16" s="85" t="str">
+    <x:row r="24" ht="54" customHeight="1">
+      <x:c r="A24" s="98" t="str">
         <x:v>FT-012</x:v>
       </x:c>
-      <x:c r="B16" s="85" t="str">
+      <x:c r="B24" s="98" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="C16" s="85" t="str">
+      <x:c r="C24" s="98" t="str">
         <x:v>LTFT mínimo</x:v>
       </x:c>
-      <x:c r="D16" s="82" t="str">
+      <x:c r="D24" s="98" t="str">
         <x:v>ASF em base de carbono</x:v>
       </x:c>
-      <x:c r="E16" s="82" t="str">
+      <x:c r="E24" s="98" t="str">
         <x:v>Oferecer referência matemática transparente para distribuição de produtos.</x:v>
       </x:c>
-      <x:c r="F16" s="82" t="str">
+      <x:c r="F24" s="98" t="str">
         <x:v>Calcular frações exclusivas por faixa, fechamento, cauda e alpha ótimo matemático para o alvo.</x:v>
       </x:c>
-      <x:c r="G16" s="85" t="str">
+      <x:c r="G24" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H16" s="82" t="str">
+      <x:c r="H24" s="98" t="str">
         <x:v>asf.py, screening.py e testes de fechamento e máximos matemáticos.</x:v>
       </x:c>
-      <x:c r="I16" s="82" t="str">
+      <x:c r="I24" s="98" t="str">
         <x:v>Adicionar comparação com dados medidos e propagação de incerteza.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="54" customHeight="1">
-      <x:c r="A17" s="85" t="str">
+    <x:row r="25" ht="54" customHeight="1">
+      <x:c r="A25" s="97" t="str">
         <x:v>FT-013</x:v>
       </x:c>
-      <x:c r="B17" s="85" t="str">
+      <x:c r="B25" s="97" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="C17" s="85" t="str">
+      <x:c r="C25" s="97" t="str">
         <x:v>LTFT mínimo</x:v>
       </x:c>
-      <x:c r="D17" s="82" t="str">
+      <x:c r="D25" s="97" t="str">
         <x:v>Caso experimental completo</x:v>
       </x:c>
-      <x:c r="E17" s="82" t="str">
+      <x:c r="E25" s="97" t="str">
         <x:v>Registrar condições necessárias para interpretar e reproduzir um ensaio.</x:v>
       </x:c>
-      <x:c r="F17" s="82" t="str">
+      <x:c r="F25" s="97" t="str">
         <x:v>Capturar reator, alimentação, ativação, vazão, GHSV/WHSV, leito, massa, tempo e condições.</x:v>
       </x:c>
-      <x:c r="G17" s="85" t="str">
+      <x:c r="G25" s="111" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="H17" s="82" t="str">
+      <x:c r="H25" s="97" t="str">
         <x:v>Contrato inclui vários campos e exemplo experimental completo; faltam gradiente térmico, método analítico, replicatas e estado estacionário.</x:v>
       </x:c>
-      <x:c r="I17" s="82" t="str">
+      <x:c r="I25" s="97" t="str">
         <x:v>Ampliar contrato v2 com qualidade analítica, temperaturas múltiplas e replicatas.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="54" customHeight="1">
-      <x:c r="A18" s="85" t="str">
+    <x:row r="26" ht="54" customHeight="1">
+      <x:c r="A26" s="98" t="str">
         <x:v>FT-014</x:v>
       </x:c>
-      <x:c r="B18" s="85" t="str">
+      <x:c r="B26" s="98" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="C18" s="85" t="str">
+      <x:c r="C26" s="98" t="str">
         <x:v>LTFT mínimo</x:v>
       </x:c>
-      <x:c r="D18" s="82" t="str">
+      <x:c r="D26" s="98" t="str">
         <x:v>Balanço de carbono</x:v>
       </x:c>
-      <x:c r="E18" s="82" t="str">
+      <x:c r="E26" s="98" t="str">
         <x:v>Verificar consistência material antes de usar dados em modelos.</x:v>
       </x:c>
-      <x:c r="F18" s="82" t="str">
+      <x:c r="F26" s="98" t="str">
         <x:v>Calcular entrada/saída de carbono, incluir CO2 e espécies não identificadas, aplicar tolerância versionada e emitir relatório.</x:v>
       </x:c>
-      <x:c r="G18" s="85" t="str">
+      <x:c r="G26" s="111" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="H18" s="82" t="str">
+      <x:c r="H26" s="98" t="str">
         <x:v>Auditoria verifica fechamento de seletividades; ainda não calcula balanço material completo de carbono.</x:v>
       </x:c>
-      <x:c r="I18" s="82" t="str">
+      <x:c r="I26" s="98" t="str">
         <x:v>Definir tolerância e implementar módulo de balanço com casos sintéticos.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="54" customHeight="1">
-      <x:c r="A19" s="85" t="str">
+    <x:row r="27" ht="54" customHeight="1">
+      <x:c r="A27" s="97" t="str">
         <x:v>FT-015</x:v>
       </x:c>
-      <x:c r="B19" s="85" t="str">
+      <x:c r="B27" s="97" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="C19" s="85" t="str">
+      <x:c r="C27" s="97" t="str">
         <x:v>LTFT mínimo</x:v>
       </x:c>
-      <x:c r="D19" s="82" t="str">
+      <x:c r="D27" s="97" t="str">
         <x:v>Balanços de H/O</x:v>
       </x:c>
-      <x:c r="E19" s="82" t="str">
+      <x:c r="E27" s="97" t="str">
         <x:v>Avaliar consistência de hidrogênio, oxigênio, água e CO2.</x:v>
       </x:c>
-      <x:c r="F19" s="82" t="str">
+      <x:c r="F27" s="97" t="str">
         <x:v>Definir espécies/bases, calcular fechamentos H e O e propagar incerteza.</x:v>
       </x:c>
-      <x:c r="G19" s="85" t="str">
+      <x:c r="G27" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H19" s="82" t="str">
+      <x:c r="H27" s="97" t="str">
         <x:v>Não há módulo nem campos suficientes para balanços completos de H/O.</x:v>
       </x:c>
-      <x:c r="I19" s="82" t="str">
+      <x:c r="I27" s="97" t="str">
         <x:v>Aprovar contrato analítico e implementar após o balanço de carbono.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="54" customHeight="1">
-      <x:c r="A20" s="85" t="str">
+    <x:row r="28" ht="54" customHeight="1">
+      <x:c r="A28" s="98" t="str">
         <x:v>FT-016</x:v>
       </x:c>
-      <x:c r="B20" s="85" t="str">
+      <x:c r="B28" s="98" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="C20" s="85" t="str">
+      <x:c r="C28" s="98" t="str">
         <x:v>LTFT mínimo</x:v>
       </x:c>
-      <x:c r="D20" s="82" t="str">
+      <x:c r="D28" s="98" t="str">
         <x:v>Auditor de evidência</x:v>
       </x:c>
-      <x:c r="E20" s="82" t="str">
+      <x:c r="E28" s="98" t="str">
         <x:v>Impedir uso automático de dados incompletos ou incompatíveis.</x:v>
       </x:c>
-      <x:c r="F20" s="82" t="str">
+      <x:c r="F28" s="98" t="str">
         <x:v>Validar cabeçalhos, tipos, duplicatas, limites, fechamento, manifesto, hash e compatibilidade contextual.</x:v>
       </x:c>
-      <x:c r="G20" s="85" t="str">
+      <x:c r="G28" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H20" s="82" t="str">
+      <x:c r="H28" s="98" t="str">
         <x:v>evidence_validation.py, audit_evidence.py, VALIDACAO_EVIDENCIAS.md e testes.</x:v>
       </x:c>
-      <x:c r="I20" s="82" t="str">
+      <x:c r="I28" s="98" t="str">
         <x:v>Integrar o auditor à interface e registrar revisão humana por evidência.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="54" customHeight="1">
-      <x:c r="A21" s="85" t="str">
+    <x:row r="29" ht="54" customHeight="1">
+      <x:c r="A29" s="97" t="str">
         <x:v>FT-017</x:v>
       </x:c>
-      <x:c r="B21" s="85" t="str">
+      <x:c r="B29" s="97" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="C21" s="85" t="str">
+      <x:c r="C29" s="97" t="str">
         <x:v>LTFT mínimo</x:v>
       </x:c>
-      <x:c r="D21" s="82" t="str">
+      <x:c r="D29" s="97" t="str">
         <x:v>Comparação ASF/medição</x:v>
       </x:c>
-      <x:c r="E21" s="82" t="str">
+      <x:c r="E29" s="97" t="str">
         <x:v>Quantificar onde a ASF descreve ou falha em descrever os produtos observados.</x:v>
       </x:c>
-      <x:c r="F21" s="82" t="str">
+      <x:c r="F29" s="97" t="str">
         <x:v>Alinhar base de seletividade, calcular resíduos por Cn/faixa e mostrar incerteza e desvios C1/C2/cauda.</x:v>
       </x:c>
-      <x:c r="G21" s="85" t="str">
+      <x:c r="G29" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H21" s="82" t="str">
+      <x:c r="H29" s="97" t="str">
         <x:v>A plataforma calcula ASF, mas não ingere medições aprovadas para comparação quantitativa.</x:v>
       </x:c>
-      <x:c r="I21" s="82" t="str">
+      <x:c r="I29" s="97" t="str">
         <x:v>Definir formato de medição e implementar relatório de resíduos.</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="54" customHeight="1">
-      <x:c r="A22" s="85" t="str">
+    <x:row r="30" ht="54" customHeight="1">
+      <x:c r="A30" s="98" t="str">
         <x:v>FT-018</x:v>
       </x:c>
-      <x:c r="B22" s="85" t="str">
+      <x:c r="B30" s="98" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="C22" s="85" t="str">
+      <x:c r="C30" s="98" t="str">
         <x:v>LTFT mínimo</x:v>
       </x:c>
-      <x:c r="D22" s="82" t="str">
+      <x:c r="D30" s="98" t="str">
         <x:v>Interface LTFT</x:v>
       </x:c>
-      <x:c r="E22" s="82" t="str">
+      <x:c r="E30" s="98" t="str">
         <x:v>Permitir executar o fluxo produto→caso→resultado de modo compreensível.</x:v>
       </x:c>
-      <x:c r="F22" s="82" t="str">
+      <x:c r="F30" s="98" t="str">
         <x:v>Expor seleção de produto, entradas do caso, distribuição ASF, prontidão, limites e bloqueios.</x:v>
       </x:c>
-      <x:c r="G22" s="85" t="str">
+      <x:c r="G30" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H22" s="82" t="str">
+      <x:c r="H30" s="98" t="str">
         <x:v>app.py testado e publicado no Streamlit com fluxo LTFT e avisos científicos.</x:v>
       </x:c>
-      <x:c r="I22" s="82" t="str">
+      <x:c r="I30" s="98" t="str">
         <x:v>Adicionar persistência, evidências aplicáveis e exportação pelo usuário.</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="54" customHeight="1">
-      <x:c r="A23" s="85" t="str">
+    <x:row r="31" ht="54" customHeight="1">
+      <x:c r="A31" s="97" t="str">
         <x:v>FT-019</x:v>
       </x:c>
-      <x:c r="B23" s="85" t="str">
+      <x:c r="B31" s="97" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="C23" s="85" t="str">
+      <x:c r="C31" s="97" t="str">
         <x:v>LTFT mínimo</x:v>
       </x:c>
-      <x:c r="D23" s="82" t="str">
+      <x:c r="D31" s="97" t="str">
         <x:v>Exportação JSON/CSV</x:v>
       </x:c>
-      <x:c r="E23" s="82" t="str">
+      <x:c r="E31" s="97" t="str">
         <x:v>Permitir reutilização e auditoria dos dados e resultados.</x:v>
       </x:c>
-      <x:c r="F23" s="82" t="str">
+      <x:c r="F31" s="97" t="str">
         <x:v>Exportar entrada, resultado e tabelas em formatos versionados, com metadados e hashes.</x:v>
       </x:c>
-      <x:c r="G23" s="85" t="str">
+      <x:c r="G31" s="111" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="H23" s="82" t="str">
+      <x:c r="H31" s="97" t="str">
         <x:v>Worker exporta JSON reproduzível; não há exportação CSV completa pela interface.</x:v>
       </x:c>
-      <x:c r="I23" s="82" t="str">
+      <x:c r="I31" s="97" t="str">
         <x:v>Implementar exportação CSV e pacote de execução com manifesto.</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="54" customHeight="1">
-      <x:c r="A24" s="85" t="str">
+    <x:row r="32" ht="54" customHeight="1">
+      <x:c r="A32" s="98" t="str">
         <x:v>FT-020</x:v>
       </x:c>
-      <x:c r="B24" s="85" t="str">
+      <x:c r="B32" s="98" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="C24" s="85" t="str">
+      <x:c r="C32" s="98" t="str">
         <x:v>LTFT mínimo</x:v>
       </x:c>
-      <x:c r="D24" s="82" t="str">
+      <x:c r="D32" s="98" t="str">
         <x:v>Relatório científico</x:v>
       </x:c>
-      <x:c r="E24" s="82" t="str">
+      <x:c r="E32" s="98" t="str">
         <x:v>Consolidar premissas, evidências, resultados, incertezas e limitações.</x:v>
       </x:c>
-      <x:c r="F24" s="82" t="str">
+      <x:c r="F32" s="98" t="str">
         <x:v>Gerar relatório legível e auditável com versão, entradas, método, bloqueios e referências.</x:v>
       </x:c>
-      <x:c r="G24" s="85" t="str">
+      <x:c r="G32" s="111" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="H24" s="82" t="str">
+      <x:c r="H32" s="98" t="str">
         <x:v>Resultado JSON e notebook existem; não há relatório científico final formatado.</x:v>
       </x:c>
-      <x:c r="I24" s="82" t="str">
+      <x:c r="I32" s="98" t="str">
         <x:v>Definir template e gerar relatório a partir do contrato de resultado.</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="54" customHeight="1">
-      <x:c r="A25" s="85" t="str">
+    <x:row r="33" ht="54" customHeight="1">
+      <x:c r="A33" s="97" t="str">
         <x:v>FT-021</x:v>
       </x:c>
-      <x:c r="B25" s="85" t="str">
+      <x:c r="B33" s="97" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="C25" s="85" t="str">
+      <x:c r="C33" s="97" t="str">
         <x:v>Validação LTFT</x:v>
       </x:c>
-      <x:c r="D25" s="82" t="str">
+      <x:c r="D33" s="97" t="str">
         <x:v>Corpus LTFT aprovado</x:v>
       </x:c>
-      <x:c r="E25" s="82" t="str">
+      <x:c r="E33" s="97" t="str">
         <x:v>Disponibilizar dados confiáveis e licenciáveis para validação/calibração.</x:v>
       </x:c>
-      <x:c r="F25" s="82" t="str">
+      <x:c r="F33" s="97" t="str">
         <x:v>Curar fontes, conferir valores com tabelas originais, registrar licença, unidades, incerteza e aprovação.</x:v>
       </x:c>
-      <x:c r="G25" s="85" t="str">
+      <x:c r="G33" s="115" t="str">
         <x:v>Bloqueado</x:v>
       </x:c>
-      <x:c r="H25" s="82" t="str">
+      <x:c r="H33" s="97" t="str">
         <x:v>CSVs locais permanecem fora do repositório e não aprovados; o auditor impede calibração automática.</x:v>
       </x:c>
-      <x:c r="I25" s="82" t="str">
+      <x:c r="I33" s="97" t="str">
         <x:v>Verificar licenças e leitura integral e aprovar um primeiro conjunto de uso.</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="54" customHeight="1">
-      <x:c r="A26" s="85" t="str">
+    <x:row r="34" ht="54" customHeight="1">
+      <x:c r="A34" s="98" t="str">
         <x:v>FT-022</x:v>
       </x:c>
-      <x:c r="B26" s="85" t="str">
+      <x:c r="B34" s="98" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="C26" s="85" t="str">
+      <x:c r="C34" s="98" t="str">
         <x:v>Validação LTFT</x:v>
       </x:c>
-      <x:c r="D26" s="82" t="str">
+      <x:c r="D34" s="98" t="str">
         <x:v>Compatibilidade de casos</x:v>
       </x:c>
-      <x:c r="E26" s="82" t="str">
+      <x:c r="E34" s="98" t="str">
         <x:v>Evitar comparação entre experimentos incompatíveis.</x:v>
       </x:c>
-      <x:c r="F26" s="82" t="str">
+      <x:c r="F34" s="98" t="str">
         <x:v>Criar regras para alimentação, reator, catalisador, base analítica e condições; explicar inclusão/exclusão.</x:v>
       </x:c>
-      <x:c r="G26" s="85" t="str">
+      <x:c r="G34" s="111" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="H26" s="82" t="str">
+      <x:c r="H34" s="98" t="str">
         <x:v>A auditoria calcula compatibilidade contextual, mas declara que isso não prova transferibilidade.</x:v>
       </x:c>
-      <x:c r="I26" s="82" t="str">
+      <x:c r="I34" s="98" t="str">
         <x:v>Formalizar regras por caso de uso e validar com especialista.</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="54" customHeight="1">
-      <x:c r="A27" s="85" t="str">
+    <x:row r="35" ht="54" customHeight="1">
+      <x:c r="A35" s="97" t="str">
         <x:v>FT-023</x:v>
       </x:c>
-      <x:c r="B27" s="85" t="str">
+      <x:c r="B35" s="97" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="C27" s="85" t="str">
+      <x:c r="C35" s="97" t="str">
         <x:v>Validação LTFT</x:v>
       </x:c>
-      <x:c r="D27" s="82" t="str">
+      <x:c r="D35" s="97" t="str">
         <x:v>Domínio de aplicabilidade</x:v>
       </x:c>
-      <x:c r="E27" s="82" t="str">
+      <x:c r="E35" s="97" t="str">
         <x:v>Bloquear extrapolações fora da cobertura dos dados/modelos.</x:v>
       </x:c>
-      <x:c r="F27" s="82" t="str">
+      <x:c r="F35" s="97" t="str">
         <x:v>Definir variáveis, limites, distância/cobertura e mensagens de extrapolação testáveis.</x:v>
       </x:c>
-      <x:c r="G27" s="85" t="str">
+      <x:c r="G35" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H27" s="82" t="str">
+      <x:c r="H35" s="97" t="str">
         <x:v>Não há modelo calibrado nem domínio quantitativo implementado.</x:v>
       </x:c>
-      <x:c r="I27" s="82" t="str">
+      <x:c r="I35" s="97" t="str">
         <x:v>Implementar após aprovação do corpus e escolha do primeiro modelo.</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="54" customHeight="1">
-      <x:c r="A28" s="85" t="str">
+    <x:row r="36" ht="54" customHeight="1">
+      <x:c r="A36" s="98" t="str">
         <x:v>FT-024</x:v>
       </x:c>
-      <x:c r="B28" s="85" t="str">
+      <x:c r="B36" s="98" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="C28" s="85" t="str">
+      <x:c r="C36" s="98" t="str">
         <x:v>Validação LTFT</x:v>
       </x:c>
-      <x:c r="D28" s="82" t="str">
+      <x:c r="D36" s="98" t="str">
         <x:v>Modelo quantitativo inicial</x:v>
       </x:c>
-      <x:c r="E28" s="82" t="str">
+      <x:c r="E36" s="98" t="str">
         <x:v>Estimar uma resposta definida dentro de domínio validado.</x:v>
       </x:c>
-      <x:c r="F28" s="82" t="str">
+      <x:c r="F36" s="98" t="str">
         <x:v>Escolher equação/método, separar ajuste e teste, estimar incerteza e validar externamente.</x:v>
       </x:c>
-      <x:c r="G28" s="85" t="str">
+      <x:c r="G36" s="115" t="str">
         <x:v>Bloqueado</x:v>
       </x:c>
-      <x:c r="H28" s="82" t="str">
+      <x:c r="H36" s="98" t="str">
         <x:v>Faltam corpus aprovado, resposta-alvo, parâmetros, unidades e conjunto externo.</x:v>
       </x:c>
-      <x:c r="I28" s="82" t="str">
+      <x:c r="I36" s="98" t="str">
         <x:v>Concluir FT-021 a FT-023 antes de selecionar o modelo.</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="54" customHeight="1">
-      <x:c r="A29" s="85" t="str">
+    <x:row r="37" ht="54" customHeight="1">
+      <x:c r="A37" s="97" t="str">
         <x:v>FT-025</x:v>
       </x:c>
-      <x:c r="B29" s="85" t="str">
+      <x:c r="B37" s="97" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="C29" s="85" t="str">
+      <x:c r="C37" s="97" t="str">
         <x:v>Validação LTFT</x:v>
       </x:c>
-      <x:c r="D29" s="82" t="str">
+      <x:c r="D37" s="97" t="str">
         <x:v>Análise de sensibilidade</x:v>
       </x:c>
-      <x:c r="E29" s="82" t="str">
+      <x:c r="E37" s="97" t="str">
         <x:v>Mostrar efeito e robustez das variáveis no domínio aprovado.</x:v>
       </x:c>
-      <x:c r="F29" s="82" t="str">
+      <x:c r="F37" s="97" t="str">
         <x:v>Variar entradas, propagar incerteza e reportar faixas sem extrapolar.</x:v>
       </x:c>
-      <x:c r="G29" s="85" t="str">
+      <x:c r="G37" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H29" s="82" t="str">
+      <x:c r="H37" s="97" t="str">
         <x:v>Não há modelo quantitativo validado para suportar a análise.</x:v>
       </x:c>
-      <x:c r="I29" s="82" t="str">
+      <x:c r="I37" s="97" t="str">
         <x:v>Implementar depois de FT-024, com testes de fronteira.</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="54" customHeight="1">
-      <x:c r="A30" s="85" t="str">
+    <x:row r="38" ht="54" customHeight="1">
+      <x:c r="A38" s="98" t="str">
         <x:v>FT-026</x:v>
       </x:c>
-      <x:c r="B30" s="85" t="str">
+      <x:c r="B38" s="98" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="C30" s="85" t="str">
+      <x:c r="C38" s="98" t="str">
         <x:v>Validação LTFT</x:v>
       </x:c>
-      <x:c r="D30" s="82" t="str">
+      <x:c r="D38" s="98" t="str">
         <x:v>Gerador de plano experimental</x:v>
       </x:c>
-      <x:c r="E30" s="82" t="str">
+      <x:c r="E38" s="98" t="str">
         <x:v>Transformar objetivos e evidências em plano revisável.</x:v>
       </x:c>
-      <x:c r="F30" s="82" t="str">
+      <x:c r="F38" s="98" t="str">
         <x:v>Gerar faixas, fatores, respostas, controles, replicatas, critérios de parada e campos de aprovação.</x:v>
       </x:c>
-      <x:c r="G30" s="85" t="str">
+      <x:c r="G38" s="111" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="H30" s="82" t="str">
+      <x:c r="H38" s="98" t="str">
         <x:v>product_targets.py fornece orientação qualitativa e mantém recomendação bloqueada; não gera DOE/protocolo completo.</x:v>
       </x:c>
-      <x:c r="I30" s="82" t="str">
+      <x:c r="I38" s="98" t="str">
         <x:v>Definir template experimental e aprovação humana obrigatória.</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="54" customHeight="1">
-      <x:c r="A31" s="85" t="str">
+    <x:row r="39" ht="54" customHeight="1">
+      <x:c r="A39" s="97" t="str">
         <x:v>FT-027</x:v>
       </x:c>
-      <x:c r="B31" s="85" t="str">
+      <x:c r="B39" s="97" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="C31" s="85" t="str">
+      <x:c r="C39" s="97" t="str">
         <x:v>Validação LTFT</x:v>
       </x:c>
-      <x:c r="D31" s="82" t="str">
+      <x:c r="D39" s="97" t="str">
         <x:v>Piloto de laboratório</x:v>
       </x:c>
-      <x:c r="E31" s="82" t="str">
+      <x:c r="E39" s="97" t="str">
         <x:v>Verificar utilidade e limites da plataforma em um ensaio real.</x:v>
       </x:c>
-      <x:c r="F31" s="82" t="str">
+      <x:c r="F39" s="97" t="str">
         <x:v>Selecionar caso aprovado, executar protocolo, comparar previsão/orientação e registrar desvios.</x:v>
       </x:c>
-      <x:c r="G31" s="85" t="str">
+      <x:c r="G39" s="115" t="str">
         <x:v>Bloqueado</x:v>
       </x:c>
-      <x:c r="H31" s="82" t="str">
+      <x:c r="H39" s="97" t="str">
         <x:v>Não há plano experimental validado nem autorização/resultado de laboratório.</x:v>
       </x:c>
-      <x:c r="I31" s="82" t="str">
+      <x:c r="I39" s="97" t="str">
         <x:v>Executar somente após FT-021 a FT-026 e revisão de segurança.</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="54" customHeight="1">
-      <x:c r="A32" s="85" t="str">
+    <x:row r="40" ht="54" customHeight="1">
+      <x:c r="A40" s="98" t="str">
         <x:v>FT-028</x:v>
       </x:c>
-      <x:c r="B32" s="85" t="str">
+      <x:c r="B40" s="98" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="C32" s="85" t="str">
+      <x:c r="C40" s="98" t="str">
         <x:v>Preparação HTFT</x:v>
       </x:c>
-      <x:c r="D32" s="82" t="str">
+      <x:c r="D40" s="98" t="str">
         <x:v>Caso de uso HTFT</x:v>
       </x:c>
-      <x:c r="E32" s="82" t="str">
+      <x:c r="E40" s="98" t="str">
         <x:v>Definir um alvo HTFT específico e mensurável.</x:v>
       </x:c>
-      <x:c r="F32" s="82" t="str">
+      <x:c r="F40" s="98" t="str">
         <x:v>Escolher produto, base de seletividade, alimentação, reator, família e critérios de sucesso.</x:v>
       </x:c>
-      <x:c r="G32" s="85" t="str">
+      <x:c r="G40" s="111" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="H32" s="82" t="str">
+      <x:c r="H40" s="98" t="str">
         <x:v>Planejamento e exemplo HTFT existem, mas o alvo inicial não foi formalmente aprovado.</x:v>
       </x:c>
-      <x:c r="I32" s="82" t="str">
+      <x:c r="I40" s="98" t="str">
         <x:v>Aprovar olefinas leves, gasolina ou outro alvo e registrar responsáveis.</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="54" customHeight="1">
-      <x:c r="A33" s="85" t="str">
+    <x:row r="41" ht="54" customHeight="1">
+      <x:c r="A41" s="97" t="str">
         <x:v>FT-029</x:v>
       </x:c>
-      <x:c r="B33" s="85" t="str">
+      <x:c r="B41" s="97" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="C33" s="85" t="str">
+      <x:c r="C41" s="97" t="str">
         <x:v>Preparação HTFT</x:v>
       </x:c>
-      <x:c r="D33" s="82" t="str">
+      <x:c r="D41" s="97" t="str">
         <x:v>Schema HTFT</x:v>
       </x:c>
-      <x:c r="E33" s="82" t="str">
+      <x:c r="E41" s="97" t="str">
         <x:v>Capturar fenômenos e métricas próprias de HTFT.</x:v>
       </x:c>
-      <x:c r="F33" s="82" t="str">
+      <x:c r="F41" s="97" t="str">
         <x:v>Modelar Fe/promotores, fases, O/P por Cn, coque, gradientes, WGS e reações secundárias.</x:v>
       </x:c>
-      <x:c r="G33" s="85" t="str">
+      <x:c r="G41" s="111" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="H33" s="82" t="str">
+      <x:c r="H41" s="97" t="str">
         <x:v>Contrato v2 identifica HTFT e restringe a Fe, mas ainda não contém toda a taxonomia específica.</x:v>
       </x:c>
-      <x:c r="I33" s="82" t="str">
+      <x:c r="I41" s="97" t="str">
         <x:v>Criar schema HTFT dedicado e exemplos positivos/negativos.</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="54" customHeight="1">
-      <x:c r="A34" s="85" t="str">
+    <x:row r="42" ht="54" customHeight="1">
+      <x:c r="A42" s="98" t="str">
         <x:v>FT-030</x:v>
       </x:c>
-      <x:c r="B34" s="85" t="str">
+      <x:c r="B42" s="98" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="C34" s="85" t="str">
+      <x:c r="C42" s="98" t="str">
         <x:v>Preparação HTFT</x:v>
       </x:c>
-      <x:c r="D34" s="82" t="str">
+      <x:c r="D42" s="98" t="str">
         <x:v>Bloqueio cruzado</x:v>
       </x:c>
-      <x:c r="E34" s="82" t="str">
+      <x:c r="E42" s="98" t="str">
         <x:v>Impedir uso de regras/modelos LTFT em HTFT.</x:v>
       </x:c>
-      <x:c r="F34" s="82" t="str">
+      <x:c r="F42" s="98" t="str">
         <x:v>Validar regime, temperatura e família; rejeitar combinações incompatíveis e manter recomendação bloqueada.</x:v>
       </x:c>
-      <x:c r="G34" s="85" t="str">
+      <x:c r="G42" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H34" s="82" t="str">
+      <x:c r="H42" s="98" t="str">
         <x:v>domain.py, contrato v2 e testes rejeitam família LTFT no escopo HTFT e exigem regime consistente.</x:v>
       </x:c>
-      <x:c r="I34" s="82" t="str">
+      <x:c r="I42" s="98" t="str">
         <x:v>Estender o bloqueio a futuros modelos e datasets por identificador de regime.</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="54" customHeight="1">
-      <x:c r="A35" s="85" t="str">
+    <x:row r="43" ht="54" customHeight="1">
+      <x:c r="A43" s="97" t="str">
         <x:v>FT-031</x:v>
       </x:c>
-      <x:c r="B35" s="85" t="str">
+      <x:c r="B43" s="97" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="C35" s="85" t="str">
+      <x:c r="C43" s="97" t="str">
         <x:v>Preparação HTFT</x:v>
       </x:c>
-      <x:c r="D35" s="82" t="str">
+      <x:c r="D43" s="97" t="str">
         <x:v>Corpus HTFT</x:v>
       </x:c>
-      <x:c r="E35" s="82" t="str">
+      <x:c r="E43" s="97" t="str">
         <x:v>Criar base separada, rastreável e revisada para alta temperatura.</x:v>
       </x:c>
-      <x:c r="F35" s="82" t="str">
+      <x:c r="F43" s="97" t="str">
         <x:v>Curar estudos HTFT compatíveis, licenças, condições, produtos, fases e reações secundárias.</x:v>
       </x:c>
-      <x:c r="G35" s="85" t="str">
+      <x:c r="G43" s="115" t="str">
         <x:v>Bloqueado</x:v>
       </x:c>
-      <x:c r="H35" s="82" t="str">
+      <x:c r="H43" s="97" t="str">
         <x:v>Não existe corpus HTFT aprovado no repositório.</x:v>
       </x:c>
-      <x:c r="I35" s="82" t="str">
+      <x:c r="I43" s="97" t="str">
         <x:v>Definir protocolo de busca/extração após aprovação de FT-028/FT-029.</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="54" customHeight="1">
-      <x:c r="A36" s="85" t="str">
+    <x:row r="44" ht="54" customHeight="1">
+      <x:c r="A44" s="98" t="str">
         <x:v>FT-032</x:v>
       </x:c>
-      <x:c r="B36" s="85" t="str">
+      <x:c r="B44" s="98" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="C36" s="85" t="str">
+      <x:c r="C44" s="98" t="str">
         <x:v>Preparação HTFT</x:v>
       </x:c>
-      <x:c r="D36" s="82" t="str">
+      <x:c r="D44" s="98" t="str">
         <x:v>Balanços HTFT</x:v>
       </x:c>
-      <x:c r="E36" s="82" t="str">
+      <x:c r="E44" s="98" t="str">
         <x:v>Validar CO2, água, C/H/O e produtos não identificados em HTFT.</x:v>
       </x:c>
-      <x:c r="F36" s="82" t="str">
+      <x:c r="F44" s="98" t="str">
         <x:v>Implementar balanços com WGS, carbono/coque e espécies secundárias.</x:v>
       </x:c>
-      <x:c r="G36" s="85" t="str">
+      <x:c r="G44" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H36" s="82" t="str">
+      <x:c r="H44" s="98" t="str">
         <x:v>Não há contrato analítico nem módulo de balanços HTFT.</x:v>
       </x:c>
-      <x:c r="I36" s="82" t="str">
+      <x:c r="I44" s="98" t="str">
         <x:v>Executar após schema e corpus HTFT.</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="54" customHeight="1">
-      <x:c r="A37" s="85" t="str">
+    <x:row r="45" ht="54" customHeight="1">
+      <x:c r="A45" s="97" t="str">
         <x:v>FT-033</x:v>
       </x:c>
-      <x:c r="B37" s="85" t="str">
+      <x:c r="B45" s="97" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="C37" s="85" t="str">
+      <x:c r="C45" s="97" t="str">
         <x:v>Preparação HTFT</x:v>
       </x:c>
-      <x:c r="D37" s="82" t="str">
+      <x:c r="D45" s="97" t="str">
         <x:v>Interface HTFT bloqueada</x:v>
       </x:c>
-      <x:c r="E37" s="82" t="str">
+      <x:c r="E45" s="97" t="str">
         <x:v>Permitir diagnóstico de completude sem emitir recomendação prematura.</x:v>
       </x:c>
-      <x:c r="F37" s="82" t="str">
+      <x:c r="F45" s="97" t="str">
         <x:v>Oferecer seletor HTFT, valores iniciais compatíveis e avisos/bloqueio explícitos.</x:v>
       </x:c>
-      <x:c r="G37" s="85" t="str">
+      <x:c r="G45" s="103" t="str">
         <x:v>Concluído</x:v>
       </x:c>
-      <x:c r="H37" s="82" t="str">
+      <x:c r="H45" s="97" t="str">
         <x:v>Streamlit contém regime HTFT, família Fe, temperatura inicial 320 °C e aviso de preparação; teste de interface cobre o estado.</x:v>
       </x:c>
-      <x:c r="I37" s="82" t="str">
+      <x:c r="I45" s="97" t="str">
         <x:v>Adicionar campos específicos HTFT quando FT-029 estiver concluída.</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="54" customHeight="1">
-      <x:c r="A38" s="85" t="str">
+    <x:row r="46" ht="54" customHeight="1">
+      <x:c r="A46" s="98" t="str">
         <x:v>FT-034</x:v>
       </x:c>
-      <x:c r="B38" s="85" t="str">
+      <x:c r="B46" s="98" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="C38" s="85" t="str">
+      <x:c r="C46" s="98" t="str">
         <x:v>Preparação HTFT</x:v>
       </x:c>
-      <x:c r="D38" s="82" t="str">
+      <x:c r="D46" s="98" t="str">
         <x:v>Validação HTFT</x:v>
       </x:c>
-      <x:c r="E38" s="82" t="str">
+      <x:c r="E46" s="98" t="str">
         <x:v>Demonstrar desempenho fora da amostra e revisar cientificamente.</x:v>
       </x:c>
-      <x:c r="F38" s="82" t="str">
+      <x:c r="F46" s="98" t="str">
         <x:v>Avaliar resíduos, incerteza, domínio, estabilidade, coque e transformação de fase.</x:v>
       </x:c>
-      <x:c r="G38" s="85" t="str">
+      <x:c r="G46" s="115" t="str">
         <x:v>Bloqueado</x:v>
       </x:c>
-      <x:c r="H38" s="82" t="str">
+      <x:c r="H46" s="98" t="str">
         <x:v>Faltam corpus, balanços e modelo HTFT.</x:v>
       </x:c>
-      <x:c r="I38" s="82" t="str">
+      <x:c r="I46" s="98" t="str">
         <x:v>Concluir FT-028 a FT-033 antes de iniciar validação.</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="54" customHeight="1">
-      <x:c r="A39" s="85" t="str">
+    <x:row r="47" ht="54" customHeight="1">
+      <x:c r="A47" s="97" t="str">
         <x:v>FT-035</x:v>
       </x:c>
-      <x:c r="B39" s="85" t="str">
+      <x:c r="B47" s="97" t="str">
         <x:v>P4</x:v>
       </x:c>
-      <x:c r="C39" s="85" t="str">
+      <x:c r="C47" s="97" t="str">
         <x:v>DFT</x:v>
       </x:c>
-      <x:c r="D39" s="82" t="str">
+      <x:c r="D47" s="97" t="str">
         <x:v>Contrato estrutural</x:v>
       </x:c>
-      <x:c r="E39" s="82" t="str">
+      <x:c r="E47" s="97" t="str">
         <x:v>Garantir que apenas estruturas completas e rastreáveis sejam usadas.</x:v>
       </x:c>
-      <x:c r="F39" s="82" t="str">
+      <x:c r="F47" s="97" t="str">
         <x:v>Definir estrutura, proveniência, simetria, ocupação, carga, spin e estado de validação.</x:v>
       </x:c>
-      <x:c r="G39" s="85" t="str">
+      <x:c r="G47" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H39" s="82" t="str">
+      <x:c r="H47" s="97" t="str">
         <x:v>DFT está documentado apenas como requisito; não há schema estrutural.</x:v>
       </x:c>
-      <x:c r="I39" s="82" t="str">
+      <x:c r="I47" s="97" t="str">
         <x:v>Criar schema e exemplos válidos/inválidos antes de qualquer gerador.</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="54" customHeight="1">
-      <x:c r="A40" s="85" t="str">
+    <x:row r="48" ht="54" customHeight="1">
+      <x:c r="A48" s="98" t="str">
         <x:v>FT-036</x:v>
       </x:c>
-      <x:c r="B40" s="85" t="str">
+      <x:c r="B48" s="98" t="str">
         <x:v>P4</x:v>
       </x:c>
-      <x:c r="C40" s="85" t="str">
+      <x:c r="C48" s="98" t="str">
         <x:v>DFT</x:v>
       </x:c>
-      <x:c r="D40" s="82" t="str">
+      <x:c r="D48" s="98" t="str">
         <x:v>Protocolo de superfície</x:v>
       </x:c>
-      <x:c r="E40" s="82" t="str">
+      <x:c r="E48" s="98" t="str">
         <x:v>Padronizar modelos de superfície comparáveis.</x:v>
       </x:c>
-      <x:c r="F40" s="82" t="str">
+      <x:c r="F48" s="98" t="str">
         <x:v>Definir faceta, terminação, slab, vácuo, supercélula, cobertura e sítios.</x:v>
       </x:c>
-      <x:c r="G40" s="85" t="str">
+      <x:c r="G48" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H40" s="82" t="str">
+      <x:c r="H48" s="98" t="str">
         <x:v>Não há protocolo executável de superfície.</x:v>
       </x:c>
-      <x:c r="I40" s="82" t="str">
+      <x:c r="I48" s="98" t="str">
         <x:v>Aprovar protocolos separados para Co, Fe e carbetos relevantes.</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="54" customHeight="1">
-      <x:c r="A41" s="85" t="str">
+    <x:row r="49" ht="54" customHeight="1">
+      <x:c r="A49" s="97" t="str">
         <x:v>FT-037</x:v>
       </x:c>
-      <x:c r="B41" s="85" t="str">
+      <x:c r="B49" s="97" t="str">
         <x:v>P4</x:v>
       </x:c>
-      <x:c r="C41" s="85" t="str">
+      <x:c r="C49" s="97" t="str">
         <x:v>DFT</x:v>
       </x:c>
-      <x:c r="D41" s="82" t="str">
+      <x:c r="D49" s="97" t="str">
         <x:v>Protocolo de adsorção</x:v>
       </x:c>
-      <x:c r="E41" s="82" t="str">
+      <x:c r="E49" s="97" t="str">
         <x:v>Calcular energia de adsorção com referências consistentes.</x:v>
       </x:c>
-      <x:c r="F41" s="82" t="str">
+      <x:c r="F49" s="97" t="str">
         <x:v>Executar superfície limpa, adsorbato isolado e sistema adsorvido com parâmetros comparáveis.</x:v>
       </x:c>
-      <x:c r="G41" s="85" t="str">
+      <x:c r="G49" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H41" s="82" t="str">
+      <x:c r="H49" s="97" t="str">
         <x:v>A fórmula e requisitos estão no planejamento, mas não há implementação.</x:v>
       </x:c>
-      <x:c r="I41" s="82" t="str">
+      <x:c r="I49" s="97" t="str">
         <x:v>Definir adsorbatos, convenções e testes de consistência energética.</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="54" customHeight="1">
-      <x:c r="A42" s="85" t="str">
+    <x:row r="50" ht="54" customHeight="1">
+      <x:c r="A50" s="98" t="str">
         <x:v>FT-038</x:v>
       </x:c>
-      <x:c r="B42" s="85" t="str">
+      <x:c r="B50" s="98" t="str">
         <x:v>P4</x:v>
       </x:c>
-      <x:c r="C42" s="85" t="str">
+      <x:c r="C50" s="98" t="str">
         <x:v>DFT</x:v>
       </x:c>
-      <x:c r="D42" s="82" t="str">
+      <x:c r="D50" s="98" t="str">
         <x:v>Adaptador de engine</x:v>
       </x:c>
-      <x:c r="E42" s="82" t="str">
+      <x:c r="E50" s="98" t="str">
         <x:v>Gerar entradas válidas para o programa computacional aprovado.</x:v>
       </x:c>
-      <x:c r="F42" s="82" t="str">
+      <x:c r="F50" s="98" t="str">
         <x:v>Mapear contrato para engine, validar sintaxe e registrar versão/pseudopotenciais/bases.</x:v>
       </x:c>
-      <x:c r="G42" s="85" t="str">
+      <x:c r="G50" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H42" s="82" t="str">
+      <x:c r="H50" s="98" t="str">
         <x:v>Nenhum engine ou adaptador foi aprovado/implementado.</x:v>
       </x:c>
-      <x:c r="I42" s="82" t="str">
+      <x:c r="I50" s="98" t="str">
         <x:v>Escolher engine e criar adaptador somente após FT-035 a FT-037.</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="54" customHeight="1">
-      <x:c r="A43" s="85" t="str">
+    <x:row r="51" ht="54" customHeight="1">
+      <x:c r="A51" s="97" t="str">
         <x:v>FT-039</x:v>
       </x:c>
-      <x:c r="B43" s="85" t="str">
+      <x:c r="B51" s="97" t="str">
         <x:v>P4</x:v>
       </x:c>
-      <x:c r="C43" s="85" t="str">
+      <x:c r="C51" s="97" t="str">
         <x:v>DFT</x:v>
       </x:c>
-      <x:c r="D43" s="82" t="str">
+      <x:c r="D51" s="97" t="str">
         <x:v>Parser de saída</x:v>
       </x:c>
-      <x:c r="E43" s="82" t="str">
+      <x:c r="E51" s="97" t="str">
         <x:v>Extrair resultados, convergência e falhas sem confundir arquivo com cálculo válido.</x:v>
       </x:c>
-      <x:c r="F43" s="82" t="str">
+      <x:c r="F51" s="97" t="str">
         <x:v>Interpretar logs, energias, geometria, convergência e erros; gerar estado auditável.</x:v>
       </x:c>
-      <x:c r="G43" s="85" t="str">
+      <x:c r="G51" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H43" s="82" t="str">
+      <x:c r="H51" s="97" t="str">
         <x:v>Não há execução ou parser DFT.</x:v>
       </x:c>
-      <x:c r="I43" s="82" t="str">
+      <x:c r="I51" s="97" t="str">
         <x:v>Implementar junto ao primeiro adaptador e validar com saídas conhecidas.</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="54" customHeight="1">
-      <x:c r="A44" s="85" t="str">
+    <x:row r="52" ht="54" customHeight="1">
+      <x:c r="A52" s="98" t="str">
         <x:v>FT-040</x:v>
       </x:c>
-      <x:c r="B44" s="85" t="str">
+      <x:c r="B52" s="98" t="str">
         <x:v>P4</x:v>
       </x:c>
-      <x:c r="C44" s="85" t="str">
+      <x:c r="C52" s="98" t="str">
         <x:v>DFT</x:v>
       </x:c>
-      <x:c r="D44" s="82" t="str">
+      <x:c r="D52" s="98" t="str">
         <x:v>Relatório DFT</x:v>
       </x:c>
-      <x:c r="E44" s="82" t="str">
+      <x:c r="E52" s="98" t="str">
         <x:v>Apresentar hipótese, protocolo, convergência e limitações separadas do experimento.</x:v>
       </x:c>
-      <x:c r="F44" s="82" t="str">
+      <x:c r="F52" s="98" t="str">
         <x:v>Consolidar estruturas, parâmetros, energias, verificações e proveniência.</x:v>
       </x:c>
-      <x:c r="G44" s="85" t="str">
+      <x:c r="G52" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H44" s="82" t="str">
+      <x:c r="H52" s="98" t="str">
         <x:v>Não há resultados DFT executados neste projeto.</x:v>
       </x:c>
-      <x:c r="I44" s="82" t="str">
+      <x:c r="I52" s="98" t="str">
         <x:v>Criar template após parser validado; manter recomendação científica bloqueada.</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="54" customHeight="1">
-      <x:c r="A45" s="85" t="str">
+    <x:row r="53" ht="54" customHeight="1">
+      <x:c r="A53" s="97" t="str">
         <x:v>FT-041</x:v>
       </x:c>
-      <x:c r="B45" s="85" t="str">
+      <x:c r="B53" s="97" t="str">
         <x:v>P5</x:v>
       </x:c>
-      <x:c r="C45" s="85" t="str">
+      <x:c r="C53" s="97" t="str">
         <x:v>Operação</x:v>
       </x:c>
-      <x:c r="D45" s="82" t="str">
+      <x:c r="D53" s="97" t="str">
         <x:v>Banco e migrações</x:v>
       </x:c>
-      <x:c r="E45" s="82" t="str">
+      <x:c r="E53" s="97" t="str">
         <x:v>Persistir entidades e versões com recuperação confiável.</x:v>
       </x:c>
-      <x:c r="F45" s="82" t="str">
+      <x:c r="F53" s="97" t="str">
         <x:v>Implementar banco, migrações, armazenamento de artefatos, backup e teste de restauração.</x:v>
       </x:c>
-      <x:c r="G45" s="85" t="str">
+      <x:c r="G53" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H45" s="82" t="str">
+      <x:c r="H53" s="97" t="str">
         <x:v>Execução atual é local/arquivo; não há banco ou migrações.</x:v>
       </x:c>
-      <x:c r="I45" s="82" t="str">
+      <x:c r="I53" s="97" t="str">
         <x:v>Definir modelo relacional e estratégia de armazenamento.</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="54" customHeight="1">
-      <x:c r="A46" s="85" t="str">
+    <x:row r="54" ht="54" customHeight="1">
+      <x:c r="A54" s="98" t="str">
         <x:v>FT-042</x:v>
       </x:c>
-      <x:c r="B46" s="85" t="str">
+      <x:c r="B54" s="98" t="str">
         <x:v>P5</x:v>
       </x:c>
-      <x:c r="C46" s="85" t="str">
+      <x:c r="C54" s="98" t="str">
         <x:v>Operação</x:v>
       </x:c>
-      <x:c r="D46" s="82" t="str">
+      <x:c r="D54" s="98" t="str">
         <x:v>Autenticação e perfis</x:v>
       </x:c>
-      <x:c r="E46" s="82" t="str">
+      <x:c r="E54" s="98" t="str">
         <x:v>Controlar acesso por menor privilégio e organização/projeto.</x:v>
       </x:c>
-      <x:c r="F46" s="82" t="str">
+      <x:c r="F54" s="98" t="str">
         <x:v>Implementar login, papéis, autorização, segregação e testes de acesso.</x:v>
       </x:c>
-      <x:c r="G46" s="85" t="str">
+      <x:c r="G54" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H46" s="82" t="str">
+      <x:c r="H54" s="98" t="str">
         <x:v>Streamlit público não possui autenticação própria da plataforma.</x:v>
       </x:c>
-      <x:c r="I46" s="82" t="str">
+      <x:c r="I54" s="98" t="str">
         <x:v>Definir perfis e requisitos de privacidade antes da implementação.</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="54" customHeight="1">
-      <x:c r="A47" s="85" t="str">
+    <x:row r="55" ht="54" customHeight="1">
+      <x:c r="A55" s="97" t="str">
         <x:v>FT-043</x:v>
       </x:c>
-      <x:c r="B47" s="85" t="str">
+      <x:c r="B55" s="97" t="str">
         <x:v>P5</x:v>
       </x:c>
-      <x:c r="C47" s="85" t="str">
+      <x:c r="C55" s="97" t="str">
         <x:v>Operação</x:v>
       </x:c>
-      <x:c r="D47" s="82" t="str">
+      <x:c r="D55" s="97" t="str">
         <x:v>Fila e workers</x:v>
       </x:c>
-      <x:c r="E47" s="82" t="str">
+      <x:c r="E55" s="97" t="str">
         <x:v>Executar tarefas demoradas de forma idempotente e observável.</x:v>
       </x:c>
-      <x:c r="F47" s="82" t="str">
+      <x:c r="F55" s="97" t="str">
         <x:v>Adicionar fila, estados, retries, cancelamento, idempotência e armazenamento de artefatos.</x:v>
       </x:c>
-      <x:c r="G47" s="85" t="str">
+      <x:c r="G55" s="111" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="H47" s="82" t="str">
+      <x:c r="H55" s="97" t="str">
         <x:v>Worker local determinístico existe; faltam fila, persistência, retries e cancelamento.</x:v>
       </x:c>
-      <x:c r="I47" s="82" t="str">
+      <x:c r="I55" s="97" t="str">
         <x:v>Definir estados de Run e implementar fila após FT-041.</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="54" customHeight="1">
-      <x:c r="A48" s="85" t="str">
+    <x:row r="56" ht="54" customHeight="1">
+      <x:c r="A56" s="98" t="str">
         <x:v>FT-044</x:v>
       </x:c>
-      <x:c r="B48" s="85" t="str">
+      <x:c r="B56" s="98" t="str">
         <x:v>P5</x:v>
       </x:c>
-      <x:c r="C48" s="85" t="str">
+      <x:c r="C56" s="98" t="str">
         <x:v>Operação</x:v>
       </x:c>
-      <x:c r="D48" s="82" t="str">
+      <x:c r="D56" s="98" t="str">
         <x:v>Auditoria</x:v>
       </x:c>
-      <x:c r="E48" s="82" t="str">
+      <x:c r="E56" s="98" t="str">
         <x:v>Rastrear mudanças científicas e operacionais relevantes.</x:v>
       </x:c>
-      <x:c r="F48" s="82" t="str">
+      <x:c r="F56" s="98" t="str">
         <x:v>Registrar usuário, ação, versões, entrada, dados, modelo, configuração e artefatos.</x:v>
       </x:c>
-      <x:c r="G48" s="85" t="str">
+      <x:c r="G56" s="111" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="H48" s="82" t="str">
+      <x:c r="H56" s="98" t="str">
         <x:v>Git, schemas, JSON e hashes dão rastreabilidade parcial; não há trilha multiusuário persistente.</x:v>
       </x:c>
-      <x:c r="I48" s="82" t="str">
+      <x:c r="I56" s="98" t="str">
         <x:v>Criar modelo de eventos de auditoria junto ao banco e autenticação.</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="54" customHeight="1">
-      <x:c r="A49" s="85" t="str">
+    <x:row r="57" ht="54" customHeight="1">
+      <x:c r="A57" s="97" t="str">
         <x:v>FT-045</x:v>
       </x:c>
-      <x:c r="B49" s="85" t="str">
+      <x:c r="B57" s="97" t="str">
         <x:v>P5</x:v>
       </x:c>
-      <x:c r="C49" s="85" t="str">
+      <x:c r="C57" s="97" t="str">
         <x:v>Operação</x:v>
       </x:c>
-      <x:c r="D49" s="82" t="str">
+      <x:c r="D57" s="97" t="str">
         <x:v>Homologação</x:v>
       </x:c>
-      <x:c r="E49" s="82" t="str">
+      <x:c r="E57" s="97" t="str">
         <x:v>Validar sistema completo com dados aprovados antes de produção.</x:v>
       </x:c>
-      <x:c r="F49" s="82" t="str">
+      <x:c r="F57" s="97" t="str">
         <x:v>Implantar ambiente separado, testar migração, carga, segurança, recuperação e casos de aceite.</x:v>
       </x:c>
-      <x:c r="G49" s="85" t="str">
+      <x:c r="G57" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H49" s="82" t="str">
+      <x:c r="H57" s="97" t="str">
         <x:v>Há protótipo público, mas não ambiente formal de homologação.</x:v>
       </x:c>
-      <x:c r="I49" s="82" t="str">
+      <x:c r="I57" s="97" t="str">
         <x:v>Criar ambiente após persistência, autenticação e corpus aprovado.</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="54" customHeight="1">
-      <x:c r="A50" s="85" t="str">
+    <x:row r="58" ht="54" customHeight="1">
+      <x:c r="A58" s="98" t="str">
         <x:v>FT-046</x:v>
       </x:c>
-      <x:c r="B50" s="85" t="str">
+      <x:c r="B58" s="98" t="str">
         <x:v>P5</x:v>
       </x:c>
-      <x:c r="C50" s="85" t="str">
+      <x:c r="C58" s="98" t="str">
         <x:v>Operação</x:v>
       </x:c>
-      <x:c r="D50" s="82" t="str">
+      <x:c r="D58" s="98" t="str">
         <x:v>Observabilidade</x:v>
       </x:c>
-      <x:c r="E50" s="82" t="str">
+      <x:c r="E58" s="98" t="str">
         <x:v>Detectar falhas, atrasos e degradação da plataforma.</x:v>
       </x:c>
-      <x:c r="F50" s="82" t="str">
+      <x:c r="F58" s="98" t="str">
         <x:v>Implementar logs estruturados, métricas, alertas e painéis por execução/serviço.</x:v>
       </x:c>
-      <x:c r="G50" s="85" t="str">
+      <x:c r="G58" s="107" t="str">
         <x:v>Planejado</x:v>
       </x:c>
-      <x:c r="H50" s="82" t="str">
+      <x:c r="H58" s="98" t="str">
         <x:v>Streamlit fornece logs básicos do provedor; não há observabilidade própria.</x:v>
       </x:c>
-      <x:c r="I50" s="82" t="str">
+      <x:c r="I58" s="98" t="str">
         <x:v>Definir métricas e correlação por project_id, case_id e run_id.</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="54" customHeight="1">
-      <x:c r="A51" s="85" t="str">
+    <x:row r="59" ht="54" customHeight="1">
+      <x:c r="A59" s="97" t="str">
         <x:v>FT-047</x:v>
       </x:c>
-      <x:c r="B51" s="85" t="str">
+      <x:c r="B59" s="97" t="str">
         <x:v>P5</x:v>
       </x:c>
-      <x:c r="C51" s="85" t="str">
+      <x:c r="C59" s="97" t="str">
         <x:v>Operação</x:v>
       </x:c>
-      <x:c r="D51" s="82" t="str">
+      <x:c r="D59" s="97" t="str">
         <x:v>Segurança</x:v>
       </x:c>
-      <x:c r="E51" s="82" t="str">
+      <x:c r="E59" s="97" t="str">
         <x:v>Reduzir riscos de segredo, dependência, acesso e dados.</x:v>
       </x:c>
-      <x:c r="F51" s="82" t="str">
+      <x:c r="F59" s="97" t="str">
         <x:v>Revisar dependências, segredos, permissões, privacidade, retenção e vulnerabilidades.</x:v>
       </x:c>
-      <x:c r="G51" s="85" t="str">
+      <x:c r="G59" s="111" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="H51" s="82" t="str">
+      <x:c r="H59" s="97" t="str">
         <x:v>Segredos/artefatos sensíveis são excluídos e não há secrets necessários no protótipo; falta revisão formal e controles multiusuário.</x:v>
       </x:c>
-      <x:c r="I51" s="82" t="str">
+      <x:c r="I59" s="97" t="str">
         <x:v>Adicionar CI de dependências, política de segredos e revisão de segurança.</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="54" customHeight="1">
-      <x:c r="A52" s="86" t="str">
+    <x:row r="60" ht="54" customHeight="1">
+      <x:c r="A60" s="98" t="str">
         <x:v>FT-048</x:v>
       </x:c>
-      <x:c r="B52" s="86" t="str">
+      <x:c r="B60" s="98" t="str">
         <x:v>P5</x:v>
       </x:c>
-      <x:c r="C52" s="86" t="str">
+      <x:c r="C60" s="98" t="str">
         <x:v>Operação</x:v>
       </x:c>
-      <x:c r="D52" s="83" t="str">
+      <x:c r="D60" s="98" t="str">
         <x:v>Produção</x:v>
       </x:c>
-      <x:c r="E52" s="83" t="str">
+      <x:c r="E60" s="98" t="str">
         <x:v>Operar versão controlada com rollback e teste de fumaça.</x:v>
       </x:c>
-      <x:c r="F52" s="83" t="str">
+      <x:c r="F60" s="98" t="str">
         <x:v>Promover versão imutável após aceite, verificar backup, rollback, monitoramento e suporte.</x:v>
       </x:c>
-      <x:c r="G52" s="86" t="str">
+      <x:c r="G60" s="111" t="str">
         <x:v>Parcial</x:v>
       </x:c>
-      <x:c r="H52" s="83" t="str">
+      <x:c r="H60" s="98" t="str">
         <x:v>Aplicativo está publicado no Streamlit, mas é protótipo sem critérios completos de produção.</x:v>
       </x:c>
-      <x:c r="I52" s="83" t="str">
+      <x:c r="I60" s="98" t="str">
         <x:v>Não classificar como produção até concluir FT-041 a FT-047 e as portas científicas.</x:v>
       </x:c>
     </x:row>
@@ -2839,7 +4081,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ae28640bfa0466a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R568dd0e989b449bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: concluir UX FT-051 e FT-052
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R191b9c0cc0f54ec3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R3bdb7d9b40cd42f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R570443a6c2b94c87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rbb74cb814a1844a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -326,12 +326,6 @@
     <x:t xml:space="preserve">Definir cores semânticas, tipografia, espaçamento, cartões e componentes; validar contraste, teclado, textos alternativos e pontos de quebra responsivos.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Existe tema Streamlit básico em .streamlit/config.toml, sem sistema de componentes ou verificação formal de acessibilidade.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Criar tokens visuais e componentes reutilizáveis; executar auditoria visual em desktop e celular.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">FT-052</x:t>
   </x:si>
   <x:si>
@@ -342,12 +336,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Organizar produto, catalisador, reator, alimentação, condições e proveniência em blocos; incluir ajuda contextual, unidades e validação próxima do campo.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">O formulário atual reúne campos em uma única seção e valida principalmente após o envio.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Implementar depois de FT-049/FT-051 e preservar as validações do domínio.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">FT-053</x:t>
@@ -1274,7 +1262,7 @@
       <x:family val="2"/>
     </x:font>
   </x:fonts>
-  <x:fills count="21">
+  <x:fills count="22">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1374,6 +1362,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF3F8F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEFD8"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -1502,7 +1495,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="46">
+  <x:cellXfs count="48">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1618,6 +1611,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="16" fillId="20" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="21" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="21" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1949,14 +1948,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E5" s="16" t="n">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F5" s="12"/>
       <x:c r="G5" s="15" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="H5" s="17" t="n">
-        <x:v>0.2698412698412698</x:v>
+        <x:v>0.30158730158730157</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -1998,7 +1997,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B9" s="20" t="n">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C9" s="12"/>
       <x:c r="D9" s="12"/>
@@ -2026,7 +2025,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B11" s="20" t="n">
-        <x:v>25</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C11" s="12"/>
       <x:c r="D11" s="12"/>
@@ -2216,7 +2215,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B26" s="21" t="str">
-        <x:v>tests/ — 60 testes e 15 subtestes aprovados na verificação da FT-050 em 2026-10-13</x:v>
+        <x:v>tests/ — 64 testes e 15 subtestes aprovados na verificação de FT-051/FT-052 em 2026-10-13</x:v>
       </x:c>
       <x:c r="C26" s="12"/>
       <x:c r="D26" s="12"/>
@@ -2230,7 +2229,7 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B27" s="21" t="str">
-        <x:v>GitHub no commit 135c958; aplicação local HTTP 200; Streamlit público ainda exibiu a revisão anterior na última verificação</x:v>
+        <x:v>Implementação local verificada em desktop e viewport móvel; publicação depende do redeploy da revisão no Streamlit</x:v>
       </x:c>
       <x:c r="C27" s="12"/>
       <x:c r="D27" s="12"/>
@@ -2696,19 +2695,19 @@
       <x:c r="F16" s="7" t="s">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="G16" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H16" s="7" t="s">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="I16" s="7" t="s">
-        <x:v>106</x:v>
+      <x:c r="G16" s="47" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="H16" s="7" t="str">
+        <x:v>Sistema visual em src/plataforma_ltft/ui_design.py e .streamlit/config.toml: tokens, cartões, foco visível, movimento reduzido e CSS responsivo; revisão visual em desktop e viewport 390 x 844.</x:v>
+      </x:c>
+      <x:c r="I16" s="7" t="str">
+        <x:v>Manter os componentes e critérios de acessibilidade nas próximas telas; executar FT-053.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
       <x:c r="A17" s="7" t="s">
-        <x:v>107</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="B17" s="7" t="s">
         <x:v>37</x:v>
@@ -2717,27 +2716,27 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="D17" s="7" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="E17" s="7" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="F17" s="7" t="s">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="E17" s="7" t="s">
-        <x:v>109</x:v>
-      </x:c>
-      <x:c r="F17" s="7" t="s">
-        <x:v>110</x:v>
-      </x:c>
-      <x:c r="G17" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H17" s="7" t="s">
-        <x:v>111</x:v>
-      </x:c>
-      <x:c r="I17" s="7" t="s">
-        <x:v>112</x:v>
+      <x:c r="G17" s="47" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="H17" s="7" t="str">
+        <x:v>app.py reorganizado em blocos de produto, regime, composição/fase, condições do reator e parâmetro ASF; ajuda e unidades próximas; validação imediata testada. Suíte: 64 testes e 15 subtestes.</x:v>
+      </x:c>
+      <x:c r="I17" s="7" t="str">
+        <x:v>Executar FT-053: painel científico com curva ASF por Cn e faixa-alvo destacada.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
       <x:c r="A18" s="7" t="s">
-        <x:v>113</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B18" s="7" t="s">
         <x:v>37</x:v>
@@ -2746,27 +2745,27 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="D18" s="7" t="s">
-        <x:v>114</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E18" s="7" t="s">
-        <x:v>115</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="F18" s="7" t="s">
-        <x:v>116</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="G18" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H18" s="7" t="s">
-        <x:v>117</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="I18" s="7" t="s">
-        <x:v>118</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
       <x:c r="A19" s="7" t="s">
-        <x:v>119</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="B19" s="7" t="s">
         <x:v>37</x:v>
@@ -2775,27 +2774,27 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="D19" s="7" t="s">
-        <x:v>120</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="E19" s="7" t="s">
-        <x:v>121</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F19" s="7" t="s">
-        <x:v>122</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="G19" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H19" s="7" t="s">
-        <x:v>123</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="I19" s="7" t="s">
-        <x:v>124</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
       <x:c r="A20" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B20" s="7" t="s">
         <x:v>37</x:v>
@@ -2804,27 +2803,27 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="D20" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="E20" s="7" t="s">
-        <x:v>127</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="F20" s="7" t="s">
-        <x:v>128</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="G20" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H20" s="7" t="s">
-        <x:v>129</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="I20" s="7" t="s">
-        <x:v>130</x:v>
+        <x:v>126</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
       <x:c r="A21" s="7" t="s">
-        <x:v>131</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="B21" s="7" t="s">
         <x:v>37</x:v>
@@ -2833,27 +2832,27 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="D21" s="7" t="s">
-        <x:v>132</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E21" s="7" t="s">
-        <x:v>133</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="F21" s="7" t="s">
-        <x:v>134</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="G21" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H21" s="7" t="s">
-        <x:v>135</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="I21" s="7" t="s">
-        <x:v>136</x:v>
+        <x:v>132</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="54" customHeight="1">
       <x:c r="A22" s="6" t="s">
-        <x:v>137</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="B22" s="6" t="s">
         <x:v>37</x:v>
@@ -2862,1124 +2861,1124 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="D22" s="6" t="s">
-        <x:v>138</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="E22" s="6" t="s">
-        <x:v>139</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="F22" s="6" t="s">
-        <x:v>140</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="G22" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H22" s="6" t="s">
-        <x:v>141</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="I22" s="6" t="s">
-        <x:v>142</x:v>
+        <x:v>138</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
       <x:c r="A23" s="5" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="B23" s="5" t="s">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="C23" s="5" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="D23" s="5" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="E23" s="5" t="s">
         <x:v>143</x:v>
       </x:c>
-      <x:c r="B23" s="5" t="s">
+      <x:c r="F23" s="5" t="s">
         <x:v>144</x:v>
-      </x:c>
-      <x:c r="C23" s="5" t="s">
-        <x:v>145</x:v>
-      </x:c>
-      <x:c r="D23" s="5" t="s">
-        <x:v>146</x:v>
-      </x:c>
-      <x:c r="E23" s="5" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="F23" s="5" t="s">
-        <x:v>148</x:v>
       </x:c>
       <x:c r="G23" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H23" s="5" t="s">
-        <x:v>149</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="I23" s="5" t="s">
-        <x:v>150</x:v>
+        <x:v>146</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
       <x:c r="A24" s="6" t="s">
-        <x:v>151</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B24" s="6" t="s">
-        <x:v>144</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C24" s="6" t="s">
-        <x:v>145</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="D24" s="6" t="s">
-        <x:v>152</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="E24" s="6" t="s">
-        <x:v>153</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="F24" s="6" t="s">
-        <x:v>154</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="G24" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H24" s="6" t="s">
-        <x:v>155</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="I24" s="6" t="s">
-        <x:v>156</x:v>
+        <x:v>152</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="54" customHeight="1">
       <x:c r="A25" s="5" t="s">
-        <x:v>157</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="B25" s="5" t="s">
-        <x:v>144</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C25" s="5" t="s">
-        <x:v>145</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="D25" s="5" t="s">
-        <x:v>158</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="E25" s="5" t="s">
-        <x:v>159</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="F25" s="5" t="s">
-        <x:v>160</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="G25" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H25" s="5" t="s">
-        <x:v>161</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I25" s="5" t="s">
-        <x:v>162</x:v>
+        <x:v>158</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="54" customHeight="1">
       <x:c r="A26" s="6" t="s">
-        <x:v>163</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B26" s="6" t="s">
-        <x:v>144</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C26" s="6" t="s">
-        <x:v>145</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="D26" s="6" t="s">
-        <x:v>164</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="E26" s="6" t="s">
-        <x:v>165</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="F26" s="6" t="s">
-        <x:v>166</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="G26" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H26" s="6" t="s">
-        <x:v>167</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="I26" s="6" t="s">
-        <x:v>168</x:v>
+        <x:v>164</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="54" customHeight="1">
       <x:c r="A27" s="5" t="s">
-        <x:v>169</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B27" s="5" t="s">
-        <x:v>144</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C27" s="5" t="s">
-        <x:v>145</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="D27" s="5" t="s">
-        <x:v>170</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="E27" s="5" t="s">
-        <x:v>171</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="F27" s="5" t="s">
-        <x:v>172</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="G27" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H27" s="5" t="s">
-        <x:v>173</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="I27" s="5" t="s">
-        <x:v>174</x:v>
+        <x:v>170</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="54" customHeight="1">
       <x:c r="A28" s="6" t="s">
-        <x:v>175</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="B28" s="6" t="s">
-        <x:v>144</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C28" s="6" t="s">
-        <x:v>145</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="D28" s="6" t="s">
-        <x:v>176</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="E28" s="6" t="s">
-        <x:v>177</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="F28" s="6" t="s">
-        <x:v>178</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="G28" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H28" s="6" t="s">
-        <x:v>179</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="I28" s="6" t="s">
-        <x:v>180</x:v>
+        <x:v>176</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="54" customHeight="1">
       <x:c r="A29" s="5" t="s">
-        <x:v>181</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B29" s="5" t="s">
-        <x:v>144</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C29" s="5" t="s">
-        <x:v>145</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="D29" s="5" t="s">
-        <x:v>182</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="E29" s="5" t="s">
-        <x:v>183</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="F29" s="5" t="s">
-        <x:v>184</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="G29" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H29" s="5" t="s">
-        <x:v>185</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="I29" s="5" t="s">
-        <x:v>186</x:v>
+        <x:v>182</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="54" customHeight="1">
       <x:c r="A30" s="6" t="s">
-        <x:v>187</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B30" s="6" t="s">
-        <x:v>144</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C30" s="6" t="s">
-        <x:v>145</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="D30" s="6" t="s">
-        <x:v>188</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="E30" s="6" t="s">
-        <x:v>189</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="F30" s="6" t="s">
-        <x:v>190</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="G30" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H30" s="6" t="s">
-        <x:v>191</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="I30" s="6" t="s">
-        <x:v>192</x:v>
+        <x:v>188</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="54" customHeight="1">
       <x:c r="A31" s="5" t="s">
-        <x:v>193</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="B31" s="5" t="s">
-        <x:v>144</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C31" s="5" t="s">
-        <x:v>145</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="D31" s="5" t="s">
-        <x:v>194</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="E31" s="5" t="s">
-        <x:v>195</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="F31" s="5" t="s">
-        <x:v>196</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="G31" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H31" s="5" t="s">
-        <x:v>197</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="I31" s="5" t="s">
-        <x:v>198</x:v>
+        <x:v>194</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="54" customHeight="1">
       <x:c r="A32" s="6" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="B32" s="6" t="s">
-        <x:v>144</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C32" s="6" t="s">
-        <x:v>145</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="D32" s="6" t="s">
-        <x:v>200</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="E32" s="6" t="s">
-        <x:v>201</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="F32" s="6" t="s">
-        <x:v>202</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="G32" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H32" s="6" t="s">
-        <x:v>203</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="I32" s="6" t="s">
-        <x:v>204</x:v>
+        <x:v>200</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="54" customHeight="1">
       <x:c r="A33" s="5" t="s">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="B33" s="5" t="s">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="C33" s="5" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="D33" s="5" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="E33" s="5" t="s">
         <x:v>205</x:v>
       </x:c>
-      <x:c r="B33" s="5" t="s">
+      <x:c r="F33" s="5" t="s">
         <x:v>206</x:v>
-      </x:c>
-      <x:c r="C33" s="5" t="s">
-        <x:v>207</x:v>
-      </x:c>
-      <x:c r="D33" s="5" t="s">
-        <x:v>208</x:v>
-      </x:c>
-      <x:c r="E33" s="5" t="s">
-        <x:v>209</x:v>
-      </x:c>
-      <x:c r="F33" s="5" t="s">
-        <x:v>210</x:v>
       </x:c>
       <x:c r="G33" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H33" s="5" t="s">
-        <x:v>211</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="I33" s="5" t="s">
-        <x:v>212</x:v>
+        <x:v>208</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="54" customHeight="1">
       <x:c r="A34" s="6" t="s">
-        <x:v>213</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B34" s="6" t="s">
-        <x:v>206</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C34" s="6" t="s">
-        <x:v>207</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="D34" s="6" t="s">
-        <x:v>214</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="E34" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="F34" s="6" t="s">
-        <x:v>216</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="G34" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H34" s="6" t="s">
-        <x:v>217</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="I34" s="6" t="s">
-        <x:v>218</x:v>
+        <x:v>214</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="54" customHeight="1">
       <x:c r="A35" s="5" t="s">
-        <x:v>219</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="B35" s="5" t="s">
-        <x:v>206</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C35" s="5" t="s">
-        <x:v>207</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="D35" s="5" t="s">
-        <x:v>220</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="E35" s="5" t="s">
-        <x:v>221</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="F35" s="5" t="s">
-        <x:v>222</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G35" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H35" s="5" t="s">
-        <x:v>223</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="I35" s="5" t="s">
-        <x:v>224</x:v>
+        <x:v>220</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="54" customHeight="1">
       <x:c r="A36" s="6" t="s">
-        <x:v>225</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="B36" s="6" t="s">
-        <x:v>206</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C36" s="6" t="s">
-        <x:v>207</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="D36" s="6" t="s">
-        <x:v>226</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="E36" s="6" t="s">
-        <x:v>227</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="F36" s="6" t="s">
-        <x:v>228</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="G36" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H36" s="6" t="s">
-        <x:v>229</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="I36" s="6" t="s">
-        <x:v>230</x:v>
+        <x:v>226</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="54" customHeight="1">
       <x:c r="A37" s="5" t="s">
-        <x:v>231</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="B37" s="5" t="s">
-        <x:v>206</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C37" s="5" t="s">
-        <x:v>207</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="D37" s="5" t="s">
-        <x:v>232</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="E37" s="5" t="s">
-        <x:v>233</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="F37" s="5" t="s">
-        <x:v>234</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="G37" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H37" s="5" t="s">
-        <x:v>235</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="I37" s="5" t="s">
-        <x:v>236</x:v>
+        <x:v>232</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="54" customHeight="1">
       <x:c r="A38" s="6" t="s">
-        <x:v>237</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="B38" s="6" t="s">
-        <x:v>206</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C38" s="6" t="s">
-        <x:v>207</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="D38" s="6" t="s">
-        <x:v>238</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="E38" s="6" t="s">
-        <x:v>239</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="F38" s="6" t="s">
-        <x:v>240</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="G38" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H38" s="6" t="s">
-        <x:v>241</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="I38" s="6" t="s">
-        <x:v>242</x:v>
+        <x:v>238</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="54" customHeight="1">
       <x:c r="A39" s="5" t="s">
-        <x:v>243</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="B39" s="5" t="s">
-        <x:v>206</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C39" s="5" t="s">
-        <x:v>207</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="D39" s="5" t="s">
-        <x:v>244</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="E39" s="5" t="s">
-        <x:v>245</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="F39" s="5" t="s">
-        <x:v>246</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="G39" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H39" s="5" t="s">
-        <x:v>247</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="I39" s="5" t="s">
-        <x:v>248</x:v>
+        <x:v>244</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="54" customHeight="1">
       <x:c r="A40" s="6" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="B40" s="6" t="s">
+        <x:v>246</x:v>
+      </x:c>
+      <x:c r="C40" s="6" t="s">
+        <x:v>247</x:v>
+      </x:c>
+      <x:c r="D40" s="6" t="s">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="E40" s="6" t="s">
         <x:v>249</x:v>
       </x:c>
-      <x:c r="B40" s="6" t="s">
+      <x:c r="F40" s="6" t="s">
         <x:v>250</x:v>
-      </x:c>
-      <x:c r="C40" s="6" t="s">
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="D40" s="6" t="s">
-        <x:v>252</x:v>
-      </x:c>
-      <x:c r="E40" s="6" t="s">
-        <x:v>253</x:v>
-      </x:c>
-      <x:c r="F40" s="6" t="s">
-        <x:v>254</x:v>
       </x:c>
       <x:c r="G40" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H40" s="6" t="s">
-        <x:v>255</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="I40" s="6" t="s">
-        <x:v>256</x:v>
+        <x:v>252</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="54" customHeight="1">
       <x:c r="A41" s="5" t="s">
-        <x:v>257</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="B41" s="5" t="s">
-        <x:v>250</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="C41" s="5" t="s">
-        <x:v>251</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="D41" s="5" t="s">
-        <x:v>258</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="E41" s="5" t="s">
-        <x:v>259</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="F41" s="5" t="s">
-        <x:v>260</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="G41" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H41" s="5" t="s">
-        <x:v>261</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="I41" s="5" t="s">
-        <x:v>262</x:v>
+        <x:v>258</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="54" customHeight="1">
       <x:c r="A42" s="6" t="s">
-        <x:v>263</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="B42" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="C42" s="6" t="s">
-        <x:v>251</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="D42" s="6" t="s">
-        <x:v>264</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="E42" s="6" t="s">
-        <x:v>265</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="F42" s="6" t="s">
-        <x:v>266</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="G42" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H42" s="6" t="s">
-        <x:v>267</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="I42" s="6" t="s">
-        <x:v>268</x:v>
+        <x:v>264</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="54" customHeight="1">
       <x:c r="A43" s="5" t="s">
-        <x:v>269</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="B43" s="5" t="s">
-        <x:v>250</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="C43" s="5" t="s">
-        <x:v>251</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="D43" s="5" t="s">
-        <x:v>270</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="E43" s="5" t="s">
-        <x:v>271</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="F43" s="5" t="s">
-        <x:v>272</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="G43" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H43" s="5" t="s">
-        <x:v>273</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="I43" s="5" t="s">
-        <x:v>274</x:v>
+        <x:v>270</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="54" customHeight="1">
       <x:c r="A44" s="6" t="s">
-        <x:v>275</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="B44" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="C44" s="6" t="s">
-        <x:v>251</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="D44" s="6" t="s">
-        <x:v>276</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="E44" s="6" t="s">
-        <x:v>277</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="F44" s="6" t="s">
-        <x:v>278</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="G44" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H44" s="6" t="s">
-        <x:v>279</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="I44" s="6" t="s">
-        <x:v>280</x:v>
+        <x:v>276</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="54" customHeight="1">
       <x:c r="A45" s="5" t="s">
-        <x:v>281</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="B45" s="5" t="s">
-        <x:v>250</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="C45" s="5" t="s">
-        <x:v>251</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="D45" s="5" t="s">
-        <x:v>282</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="E45" s="5" t="s">
-        <x:v>283</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="F45" s="5" t="s">
-        <x:v>284</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="G45" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H45" s="5" t="s">
-        <x:v>285</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="I45" s="5" t="s">
-        <x:v>286</x:v>
+        <x:v>282</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="54" customHeight="1">
       <x:c r="A46" s="6" t="s">
-        <x:v>287</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="B46" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="C46" s="6" t="s">
-        <x:v>251</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="D46" s="6" t="s">
-        <x:v>288</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="E46" s="6" t="s">
-        <x:v>289</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="F46" s="6" t="s">
-        <x:v>290</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="G46" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H46" s="6" t="s">
-        <x:v>291</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="I46" s="6" t="s">
-        <x:v>292</x:v>
+        <x:v>288</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="54" customHeight="1">
       <x:c r="A47" s="5" t="s">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="B47" s="5" t="s">
+        <x:v>290</x:v>
+      </x:c>
+      <x:c r="C47" s="5" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="D47" s="5" t="s">
+        <x:v>292</x:v>
+      </x:c>
+      <x:c r="E47" s="5" t="s">
         <x:v>293</x:v>
       </x:c>
-      <x:c r="B47" s="5" t="s">
+      <x:c r="F47" s="5" t="s">
         <x:v>294</x:v>
-      </x:c>
-      <x:c r="C47" s="5" t="s">
-        <x:v>295</x:v>
-      </x:c>
-      <x:c r="D47" s="5" t="s">
-        <x:v>296</x:v>
-      </x:c>
-      <x:c r="E47" s="5" t="s">
-        <x:v>297</x:v>
-      </x:c>
-      <x:c r="F47" s="5" t="s">
-        <x:v>298</x:v>
       </x:c>
       <x:c r="G47" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H47" s="5" t="s">
-        <x:v>299</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="I47" s="5" t="s">
-        <x:v>300</x:v>
+        <x:v>296</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="54" customHeight="1">
       <x:c r="A48" s="6" t="s">
-        <x:v>301</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="B48" s="6" t="s">
-        <x:v>294</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="C48" s="6" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="D48" s="6" t="s">
-        <x:v>302</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="E48" s="6" t="s">
-        <x:v>303</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="F48" s="6" t="s">
-        <x:v>304</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="G48" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H48" s="6" t="s">
-        <x:v>305</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="I48" s="6" t="s">
-        <x:v>306</x:v>
+        <x:v>302</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="54" customHeight="1">
       <x:c r="A49" s="5" t="s">
-        <x:v>307</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="B49" s="5" t="s">
-        <x:v>294</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="C49" s="5" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="D49" s="5" t="s">
-        <x:v>308</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="E49" s="5" t="s">
-        <x:v>309</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="F49" s="5" t="s">
-        <x:v>310</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="G49" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H49" s="5" t="s">
-        <x:v>311</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="I49" s="5" t="s">
-        <x:v>312</x:v>
+        <x:v>308</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="54" customHeight="1">
       <x:c r="A50" s="6" t="s">
-        <x:v>313</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="B50" s="6" t="s">
-        <x:v>294</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="C50" s="6" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="D50" s="6" t="s">
-        <x:v>314</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="E50" s="6" t="s">
-        <x:v>315</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="F50" s="6" t="s">
-        <x:v>316</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="G50" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H50" s="6" t="s">
-        <x:v>317</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="I50" s="6" t="s">
-        <x:v>318</x:v>
+        <x:v>314</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="54" customHeight="1">
       <x:c r="A51" s="5" t="s">
-        <x:v>319</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="B51" s="5" t="s">
-        <x:v>294</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="C51" s="5" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="D51" s="5" t="s">
-        <x:v>320</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="E51" s="5" t="s">
-        <x:v>321</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="F51" s="5" t="s">
-        <x:v>322</x:v>
+        <x:v>318</x:v>
       </x:c>
       <x:c r="G51" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H51" s="5" t="s">
-        <x:v>323</x:v>
+        <x:v>319</x:v>
       </x:c>
       <x:c r="I51" s="5" t="s">
-        <x:v>324</x:v>
+        <x:v>320</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="54" customHeight="1">
       <x:c r="A52" s="6" t="s">
-        <x:v>325</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="B52" s="6" t="s">
-        <x:v>294</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="C52" s="6" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="D52" s="6" t="s">
-        <x:v>326</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="E52" s="6" t="s">
-        <x:v>327</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="F52" s="6" t="s">
-        <x:v>328</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="G52" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H52" s="6" t="s">
-        <x:v>329</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="I52" s="6" t="s">
-        <x:v>330</x:v>
+        <x:v>326</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="54" customHeight="1">
       <x:c r="A53" s="5" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="B53" s="5" t="s">
+        <x:v>328</x:v>
+      </x:c>
+      <x:c r="C53" s="5" t="s">
+        <x:v>329</x:v>
+      </x:c>
+      <x:c r="D53" s="5" t="s">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="E53" s="5" t="s">
         <x:v>331</x:v>
       </x:c>
-      <x:c r="B53" s="5" t="s">
+      <x:c r="F53" s="5" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="C53" s="5" t="s">
-        <x:v>333</x:v>
-      </x:c>
-      <x:c r="D53" s="5" t="s">
-        <x:v>334</x:v>
-      </x:c>
-      <x:c r="E53" s="5" t="s">
-        <x:v>335</x:v>
-      </x:c>
-      <x:c r="F53" s="5" t="s">
-        <x:v>336</x:v>
       </x:c>
       <x:c r="G53" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H53" s="5" t="s">
-        <x:v>337</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="I53" s="5" t="s">
-        <x:v>338</x:v>
+        <x:v>334</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="54" customHeight="1">
       <x:c r="A54" s="6" t="s">
-        <x:v>339</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="B54" s="6" t="s">
-        <x:v>332</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="C54" s="6" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="D54" s="6" t="s">
-        <x:v>340</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="E54" s="6" t="s">
-        <x:v>341</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="F54" s="6" t="s">
-        <x:v>342</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="G54" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H54" s="6" t="s">
-        <x:v>343</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="I54" s="6" t="s">
-        <x:v>344</x:v>
+        <x:v>340</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="54" customHeight="1">
       <x:c r="A55" s="5" t="s">
-        <x:v>345</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="B55" s="5" t="s">
-        <x:v>332</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="C55" s="5" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="D55" s="5" t="s">
-        <x:v>346</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="E55" s="5" t="s">
-        <x:v>347</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="F55" s="5" t="s">
-        <x:v>348</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="G55" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H55" s="5" t="s">
-        <x:v>349</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="I55" s="5" t="s">
-        <x:v>350</x:v>
+        <x:v>346</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="54" customHeight="1">
       <x:c r="A56" s="6" t="s">
-        <x:v>351</x:v>
+        <x:v>347</x:v>
       </x:c>
       <x:c r="B56" s="6" t="s">
-        <x:v>332</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="C56" s="6" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="D56" s="6" t="s">
-        <x:v>352</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="E56" s="6" t="s">
-        <x:v>353</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="F56" s="6" t="s">
-        <x:v>354</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="G56" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H56" s="6" t="s">
-        <x:v>355</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="I56" s="6" t="s">
-        <x:v>356</x:v>
+        <x:v>352</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="54" customHeight="1">
       <x:c r="A57" s="5" t="s">
-        <x:v>357</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="B57" s="5" t="s">
-        <x:v>332</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="C57" s="5" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="D57" s="5" t="s">
-        <x:v>358</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="E57" s="5" t="s">
-        <x:v>359</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="F57" s="5" t="s">
-        <x:v>360</x:v>
+        <x:v>356</x:v>
       </x:c>
       <x:c r="G57" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H57" s="5" t="s">
-        <x:v>361</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="I57" s="5" t="s">
-        <x:v>362</x:v>
+        <x:v>358</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="54" customHeight="1">
       <x:c r="A58" s="6" t="s">
-        <x:v>363</x:v>
+        <x:v>359</x:v>
       </x:c>
       <x:c r="B58" s="6" t="s">
-        <x:v>332</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="C58" s="6" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="D58" s="6" t="s">
-        <x:v>364</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="E58" s="6" t="s">
-        <x:v>365</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="F58" s="6" t="s">
-        <x:v>366</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="G58" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H58" s="6" t="s">
-        <x:v>367</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="I58" s="6" t="s">
-        <x:v>368</x:v>
+        <x:v>364</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="54" customHeight="1">
       <x:c r="A59" s="5" t="s">
-        <x:v>369</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="B59" s="5" t="s">
-        <x:v>332</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="C59" s="5" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="D59" s="5" t="s">
-        <x:v>370</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="E59" s="5" t="s">
-        <x:v>371</x:v>
+        <x:v>367</x:v>
       </x:c>
       <x:c r="F59" s="5" t="s">
-        <x:v>372</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="G59" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H59" s="5" t="s">
-        <x:v>373</x:v>
+        <x:v>369</x:v>
       </x:c>
       <x:c r="I59" s="5" t="s">
-        <x:v>374</x:v>
+        <x:v>370</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="54" customHeight="1">
       <x:c r="A60" s="6" t="s">
-        <x:v>375</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="B60" s="6" t="s">
-        <x:v>332</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="C60" s="6" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="D60" s="6" t="s">
-        <x:v>376</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="E60" s="6" t="s">
-        <x:v>377</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="F60" s="6" t="s">
-        <x:v>378</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="G60" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H60" s="6" t="s">
-        <x:v>379</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="I60" s="6" t="s">
-        <x:v>380</x:v>
+        <x:v>376</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="52" customHeight="1">
@@ -4203,7 +4202,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R295c22b887994b7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R720c4e0310b6447c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: concluir painel científico FT-053
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R570443a6c2b94c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rbb74cb814a1844a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R9cc8134812e24f16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rb894e47b376f4e6a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -348,12 +348,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Exibir curva ASF por Cn, faixa-alvo destacada, cortes de produtos, alpha, fração-alvo, condições usadas, prontidão, avisos e limitações em áreas distintas.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">A interface atual usa gráfico de barras por faixa, uma métrica e JSON bruto de prontidão.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Criar visualização interativa sem alterar o cálculo ASF e adicionar testes de consistência dos valores exibidos.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">FT-054</x:t>
@@ -1262,7 +1256,7 @@
       <x:family val="2"/>
     </x:font>
   </x:fonts>
-  <x:fills count="22">
+  <x:fills count="23">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1362,6 +1356,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF3F8F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEFD8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -1495,7 +1494,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="48">
+  <x:cellXfs count="50">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1616,6 +1615,12 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="21" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="22" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="22" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1948,14 +1953,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E5" s="16" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F5" s="12"/>
       <x:c r="G5" s="15" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="H5" s="17" t="n">
-        <x:v>0.30158730158730157</x:v>
+        <x:v>0.31746031746031744</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -1997,7 +2002,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B9" s="20" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C9" s="12"/>
       <x:c r="D9" s="12"/>
@@ -2025,7 +2030,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B11" s="20" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C11" s="12"/>
       <x:c r="D11" s="12"/>
@@ -2215,7 +2220,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B26" s="21" t="str">
-        <x:v>tests/ — 64 testes e 15 subtestes aprovados na verificação de FT-051/FT-052 em 2026-10-13</x:v>
+        <x:v>tests/ — 68 testes e 15 subtestes aprovados na verificação de FT-053 em 2026-10-13</x:v>
       </x:c>
       <x:c r="C26" s="12"/>
       <x:c r="D26" s="12"/>
@@ -2229,7 +2234,7 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B27" s="21" t="str">
-        <x:v>Implementação local verificada em desktop e viewport móvel; publicação depende do redeploy da revisão no Streamlit</x:v>
+        <x:v>FT-053 validada localmente; publicação pública depende do redeploy da revisão no Streamlit</x:v>
       </x:c>
       <x:c r="C27" s="12"/>
       <x:c r="D27" s="12"/>
@@ -2753,19 +2758,19 @@
       <x:c r="F18" s="7" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="G18" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H18" s="7" t="s">
-        <x:v>113</x:v>
-      </x:c>
-      <x:c r="I18" s="7" t="s">
-        <x:v>114</x:v>
+      <x:c r="G18" s="49" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="H18" s="7" t="str">
+        <x:v>Painel científico em app.py e src/plataforma_ltft/result_panel.py: curva ASF C1-C60, alvo destacado, cauda analítica C61+ até C∞, faixas de Cn, condições, prontidão e bloqueio de recomendação. Suíte: 68 testes e 15 subtestes.</x:v>
+      </x:c>
+      <x:c r="I18" s="7" t="str">
+        <x:v>Executar FT-054: categorias visuais rastreáveis para maturidade da evidência.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
       <x:c r="A19" s="7" t="s">
-        <x:v>115</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="B19" s="7" t="s">
         <x:v>37</x:v>
@@ -2774,27 +2779,27 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="D19" s="7" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="E19" s="7" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="F19" s="7" t="s">
         <x:v>116</x:v>
-      </x:c>
-      <x:c r="E19" s="7" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="F19" s="7" t="s">
-        <x:v>118</x:v>
       </x:c>
       <x:c r="G19" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H19" s="7" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="I19" s="7" t="s">
-        <x:v>120</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
       <x:c r="A20" s="7" t="s">
-        <x:v>121</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B20" s="7" t="s">
         <x:v>37</x:v>
@@ -2803,27 +2808,27 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="D20" s="7" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="E20" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F20" s="7" t="s">
         <x:v>122</x:v>
-      </x:c>
-      <x:c r="E20" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="F20" s="7" t="s">
-        <x:v>124</x:v>
       </x:c>
       <x:c r="G20" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H20" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="I20" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
       <x:c r="A21" s="7" t="s">
-        <x:v>127</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B21" s="7" t="s">
         <x:v>37</x:v>
@@ -2832,27 +2837,27 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="D21" s="7" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="E21" s="7" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="F21" s="7" t="s">
         <x:v>128</x:v>
-      </x:c>
-      <x:c r="E21" s="7" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="F21" s="7" t="s">
-        <x:v>130</x:v>
       </x:c>
       <x:c r="G21" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H21" s="7" t="s">
-        <x:v>131</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="I21" s="7" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="54" customHeight="1">
       <x:c r="A22" s="6" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B22" s="6" t="s">
         <x:v>37</x:v>
@@ -2861,1124 +2866,1124 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="D22" s="6" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="E22" s="6" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="F22" s="6" t="s">
         <x:v>134</x:v>
-      </x:c>
-      <x:c r="E22" s="6" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="F22" s="6" t="s">
-        <x:v>136</x:v>
       </x:c>
       <x:c r="G22" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H22" s="6" t="s">
-        <x:v>137</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="I22" s="6" t="s">
-        <x:v>138</x:v>
+        <x:v>136</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
       <x:c r="A23" s="5" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="B23" s="5" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C23" s="5" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="B23" s="5" t="s">
+      <x:c r="D23" s="5" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="C23" s="5" t="s">
+      <x:c r="E23" s="5" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="D23" s="5" t="s">
+      <x:c r="F23" s="5" t="s">
         <x:v>142</x:v>
-      </x:c>
-      <x:c r="E23" s="5" t="s">
-        <x:v>143</x:v>
-      </x:c>
-      <x:c r="F23" s="5" t="s">
-        <x:v>144</x:v>
       </x:c>
       <x:c r="G23" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H23" s="5" t="s">
-        <x:v>145</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="I23" s="5" t="s">
-        <x:v>146</x:v>
+        <x:v>144</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
       <x:c r="A24" s="6" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="B24" s="6" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C24" s="6" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="D24" s="6" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="E24" s="6" t="s">
         <x:v>147</x:v>
       </x:c>
-      <x:c r="B24" s="6" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="C24" s="6" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="D24" s="6" t="s">
+      <x:c r="F24" s="6" t="s">
         <x:v>148</x:v>
-      </x:c>
-      <x:c r="E24" s="6" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="F24" s="6" t="s">
-        <x:v>150</x:v>
       </x:c>
       <x:c r="G24" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H24" s="6" t="s">
-        <x:v>151</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="I24" s="6" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="54" customHeight="1">
       <x:c r="A25" s="5" t="s">
+        <x:v>151</x:v>
+      </x:c>
+      <x:c r="B25" s="5" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C25" s="5" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="D25" s="5" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="E25" s="5" t="s">
         <x:v>153</x:v>
       </x:c>
-      <x:c r="B25" s="5" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="C25" s="5" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="D25" s="5" t="s">
+      <x:c r="F25" s="5" t="s">
         <x:v>154</x:v>
-      </x:c>
-      <x:c r="E25" s="5" t="s">
-        <x:v>155</x:v>
-      </x:c>
-      <x:c r="F25" s="5" t="s">
-        <x:v>156</x:v>
       </x:c>
       <x:c r="G25" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H25" s="5" t="s">
-        <x:v>157</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="I25" s="5" t="s">
-        <x:v>158</x:v>
+        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="54" customHeight="1">
       <x:c r="A26" s="6" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="B26" s="6" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C26" s="6" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="D26" s="6" t="s">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="E26" s="6" t="s">
         <x:v>159</x:v>
       </x:c>
-      <x:c r="B26" s="6" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="C26" s="6" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="D26" s="6" t="s">
+      <x:c r="F26" s="6" t="s">
         <x:v>160</x:v>
-      </x:c>
-      <x:c r="E26" s="6" t="s">
-        <x:v>161</x:v>
-      </x:c>
-      <x:c r="F26" s="6" t="s">
-        <x:v>162</x:v>
       </x:c>
       <x:c r="G26" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H26" s="6" t="s">
-        <x:v>163</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="I26" s="6" t="s">
-        <x:v>164</x:v>
+        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="54" customHeight="1">
       <x:c r="A27" s="5" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="B27" s="5" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C27" s="5" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="D27" s="5" t="s">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="E27" s="5" t="s">
         <x:v>165</x:v>
       </x:c>
-      <x:c r="B27" s="5" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="C27" s="5" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="D27" s="5" t="s">
+      <x:c r="F27" s="5" t="s">
         <x:v>166</x:v>
-      </x:c>
-      <x:c r="E27" s="5" t="s">
-        <x:v>167</x:v>
-      </x:c>
-      <x:c r="F27" s="5" t="s">
-        <x:v>168</x:v>
       </x:c>
       <x:c r="G27" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H27" s="5" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="I27" s="5" t="s">
-        <x:v>170</x:v>
+        <x:v>168</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="54" customHeight="1">
       <x:c r="A28" s="6" t="s">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="B28" s="6" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C28" s="6" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="D28" s="6" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="E28" s="6" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="B28" s="6" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="C28" s="6" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="D28" s="6" t="s">
+      <x:c r="F28" s="6" t="s">
         <x:v>172</x:v>
-      </x:c>
-      <x:c r="E28" s="6" t="s">
-        <x:v>173</x:v>
-      </x:c>
-      <x:c r="F28" s="6" t="s">
-        <x:v>174</x:v>
       </x:c>
       <x:c r="G28" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H28" s="6" t="s">
-        <x:v>175</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="I28" s="6" t="s">
-        <x:v>176</x:v>
+        <x:v>174</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="54" customHeight="1">
       <x:c r="A29" s="5" t="s">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="B29" s="5" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C29" s="5" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="D29" s="5" t="s">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="E29" s="5" t="s">
         <x:v>177</x:v>
       </x:c>
-      <x:c r="B29" s="5" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="C29" s="5" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="D29" s="5" t="s">
+      <x:c r="F29" s="5" t="s">
         <x:v>178</x:v>
-      </x:c>
-      <x:c r="E29" s="5" t="s">
-        <x:v>179</x:v>
-      </x:c>
-      <x:c r="F29" s="5" t="s">
-        <x:v>180</x:v>
       </x:c>
       <x:c r="G29" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H29" s="5" t="s">
-        <x:v>181</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="I29" s="5" t="s">
-        <x:v>182</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="54" customHeight="1">
       <x:c r="A30" s="6" t="s">
+        <x:v>181</x:v>
+      </x:c>
+      <x:c r="B30" s="6" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C30" s="6" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="D30" s="6" t="s">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="E30" s="6" t="s">
         <x:v>183</x:v>
       </x:c>
-      <x:c r="B30" s="6" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="C30" s="6" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="D30" s="6" t="s">
+      <x:c r="F30" s="6" t="s">
         <x:v>184</x:v>
-      </x:c>
-      <x:c r="E30" s="6" t="s">
-        <x:v>185</x:v>
-      </x:c>
-      <x:c r="F30" s="6" t="s">
-        <x:v>186</x:v>
       </x:c>
       <x:c r="G30" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H30" s="6" t="s">
-        <x:v>187</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="I30" s="6" t="s">
-        <x:v>188</x:v>
+        <x:v>186</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="54" customHeight="1">
       <x:c r="A31" s="5" t="s">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="B31" s="5" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C31" s="5" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="D31" s="5" t="s">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="E31" s="5" t="s">
         <x:v>189</x:v>
       </x:c>
-      <x:c r="B31" s="5" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="C31" s="5" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="D31" s="5" t="s">
+      <x:c r="F31" s="5" t="s">
         <x:v>190</x:v>
-      </x:c>
-      <x:c r="E31" s="5" t="s">
-        <x:v>191</x:v>
-      </x:c>
-      <x:c r="F31" s="5" t="s">
-        <x:v>192</x:v>
       </x:c>
       <x:c r="G31" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H31" s="5" t="s">
-        <x:v>193</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="I31" s="5" t="s">
-        <x:v>194</x:v>
+        <x:v>192</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="54" customHeight="1">
       <x:c r="A32" s="6" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="B32" s="6" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C32" s="6" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="D32" s="6" t="s">
+        <x:v>194</x:v>
+      </x:c>
+      <x:c r="E32" s="6" t="s">
         <x:v>195</x:v>
       </x:c>
-      <x:c r="B32" s="6" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="C32" s="6" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="D32" s="6" t="s">
+      <x:c r="F32" s="6" t="s">
         <x:v>196</x:v>
-      </x:c>
-      <x:c r="E32" s="6" t="s">
-        <x:v>197</x:v>
-      </x:c>
-      <x:c r="F32" s="6" t="s">
-        <x:v>198</x:v>
       </x:c>
       <x:c r="G32" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H32" s="6" t="s">
-        <x:v>199</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="I32" s="6" t="s">
-        <x:v>200</x:v>
+        <x:v>198</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="54" customHeight="1">
       <x:c r="A33" s="5" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="B33" s="5" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C33" s="5" t="s">
         <x:v>201</x:v>
       </x:c>
-      <x:c r="B33" s="5" t="s">
+      <x:c r="D33" s="5" t="s">
         <x:v>202</x:v>
       </x:c>
-      <x:c r="C33" s="5" t="s">
+      <x:c r="E33" s="5" t="s">
         <x:v>203</x:v>
       </x:c>
-      <x:c r="D33" s="5" t="s">
+      <x:c r="F33" s="5" t="s">
         <x:v>204</x:v>
-      </x:c>
-      <x:c r="E33" s="5" t="s">
-        <x:v>205</x:v>
-      </x:c>
-      <x:c r="F33" s="5" t="s">
-        <x:v>206</x:v>
       </x:c>
       <x:c r="G33" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H33" s="5" t="s">
-        <x:v>207</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="I33" s="5" t="s">
-        <x:v>208</x:v>
+        <x:v>206</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="54" customHeight="1">
       <x:c r="A34" s="6" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B34" s="6" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C34" s="6" t="s">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="D34" s="6" t="s">
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="E34" s="6" t="s">
         <x:v>209</x:v>
       </x:c>
-      <x:c r="B34" s="6" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="C34" s="6" t="s">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="D34" s="6" t="s">
+      <x:c r="F34" s="6" t="s">
         <x:v>210</x:v>
-      </x:c>
-      <x:c r="E34" s="6" t="s">
-        <x:v>211</x:v>
-      </x:c>
-      <x:c r="F34" s="6" t="s">
-        <x:v>212</x:v>
       </x:c>
       <x:c r="G34" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H34" s="6" t="s">
-        <x:v>213</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="I34" s="6" t="s">
-        <x:v>214</x:v>
+        <x:v>212</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="54" customHeight="1">
       <x:c r="A35" s="5" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="B35" s="5" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C35" s="5" t="s">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="D35" s="5" t="s">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="E35" s="5" t="s">
         <x:v>215</x:v>
       </x:c>
-      <x:c r="B35" s="5" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="C35" s="5" t="s">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="D35" s="5" t="s">
+      <x:c r="F35" s="5" t="s">
         <x:v>216</x:v>
-      </x:c>
-      <x:c r="E35" s="5" t="s">
-        <x:v>217</x:v>
-      </x:c>
-      <x:c r="F35" s="5" t="s">
-        <x:v>218</x:v>
       </x:c>
       <x:c r="G35" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H35" s="5" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="I35" s="5" t="s">
-        <x:v>220</x:v>
+        <x:v>218</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="54" customHeight="1">
       <x:c r="A36" s="6" t="s">
+        <x:v>219</x:v>
+      </x:c>
+      <x:c r="B36" s="6" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C36" s="6" t="s">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="D36" s="6" t="s">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="E36" s="6" t="s">
         <x:v>221</x:v>
       </x:c>
-      <x:c r="B36" s="6" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="C36" s="6" t="s">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="D36" s="6" t="s">
+      <x:c r="F36" s="6" t="s">
         <x:v>222</x:v>
-      </x:c>
-      <x:c r="E36" s="6" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="F36" s="6" t="s">
-        <x:v>224</x:v>
       </x:c>
       <x:c r="G36" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H36" s="6" t="s">
-        <x:v>225</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="I36" s="6" t="s">
-        <x:v>226</x:v>
+        <x:v>224</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="54" customHeight="1">
       <x:c r="A37" s="5" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="B37" s="5" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C37" s="5" t="s">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="D37" s="5" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="E37" s="5" t="s">
         <x:v>227</x:v>
       </x:c>
-      <x:c r="B37" s="5" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="C37" s="5" t="s">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="D37" s="5" t="s">
+      <x:c r="F37" s="5" t="s">
         <x:v>228</x:v>
-      </x:c>
-      <x:c r="E37" s="5" t="s">
-        <x:v>229</x:v>
-      </x:c>
-      <x:c r="F37" s="5" t="s">
-        <x:v>230</x:v>
       </x:c>
       <x:c r="G37" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H37" s="5" t="s">
-        <x:v>231</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="I37" s="5" t="s">
-        <x:v>232</x:v>
+        <x:v>230</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="54" customHeight="1">
       <x:c r="A38" s="6" t="s">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="B38" s="6" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C38" s="6" t="s">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="D38" s="6" t="s">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="E38" s="6" t="s">
         <x:v>233</x:v>
       </x:c>
-      <x:c r="B38" s="6" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="C38" s="6" t="s">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="D38" s="6" t="s">
+      <x:c r="F38" s="6" t="s">
         <x:v>234</x:v>
-      </x:c>
-      <x:c r="E38" s="6" t="s">
-        <x:v>235</x:v>
-      </x:c>
-      <x:c r="F38" s="6" t="s">
-        <x:v>236</x:v>
       </x:c>
       <x:c r="G38" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H38" s="6" t="s">
-        <x:v>237</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="I38" s="6" t="s">
-        <x:v>238</x:v>
+        <x:v>236</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="54" customHeight="1">
       <x:c r="A39" s="5" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="B39" s="5" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C39" s="5" t="s">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="D39" s="5" t="s">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="E39" s="5" t="s">
         <x:v>239</x:v>
       </x:c>
-      <x:c r="B39" s="5" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="C39" s="5" t="s">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="D39" s="5" t="s">
+      <x:c r="F39" s="5" t="s">
         <x:v>240</x:v>
-      </x:c>
-      <x:c r="E39" s="5" t="s">
-        <x:v>241</x:v>
-      </x:c>
-      <x:c r="F39" s="5" t="s">
-        <x:v>242</x:v>
       </x:c>
       <x:c r="G39" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H39" s="5" t="s">
-        <x:v>243</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="I39" s="5" t="s">
-        <x:v>244</x:v>
+        <x:v>242</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="54" customHeight="1">
       <x:c r="A40" s="6" t="s">
+        <x:v>243</x:v>
+      </x:c>
+      <x:c r="B40" s="6" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="C40" s="6" t="s">
         <x:v>245</x:v>
       </x:c>
-      <x:c r="B40" s="6" t="s">
+      <x:c r="D40" s="6" t="s">
         <x:v>246</x:v>
       </x:c>
-      <x:c r="C40" s="6" t="s">
+      <x:c r="E40" s="6" t="s">
         <x:v>247</x:v>
       </x:c>
-      <x:c r="D40" s="6" t="s">
+      <x:c r="F40" s="6" t="s">
         <x:v>248</x:v>
-      </x:c>
-      <x:c r="E40" s="6" t="s">
-        <x:v>249</x:v>
-      </x:c>
-      <x:c r="F40" s="6" t="s">
-        <x:v>250</x:v>
       </x:c>
       <x:c r="G40" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H40" s="6" t="s">
-        <x:v>251</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="I40" s="6" t="s">
-        <x:v>252</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="54" customHeight="1">
       <x:c r="A41" s="5" t="s">
+        <x:v>251</x:v>
+      </x:c>
+      <x:c r="B41" s="5" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="C41" s="5" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="D41" s="5" t="s">
+        <x:v>252</x:v>
+      </x:c>
+      <x:c r="E41" s="5" t="s">
         <x:v>253</x:v>
       </x:c>
-      <x:c r="B41" s="5" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="C41" s="5" t="s">
-        <x:v>247</x:v>
-      </x:c>
-      <x:c r="D41" s="5" t="s">
+      <x:c r="F41" s="5" t="s">
         <x:v>254</x:v>
-      </x:c>
-      <x:c r="E41" s="5" t="s">
-        <x:v>255</x:v>
-      </x:c>
-      <x:c r="F41" s="5" t="s">
-        <x:v>256</x:v>
       </x:c>
       <x:c r="G41" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H41" s="5" t="s">
-        <x:v>257</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="I41" s="5" t="s">
-        <x:v>258</x:v>
+        <x:v>256</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="54" customHeight="1">
       <x:c r="A42" s="6" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="B42" s="6" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="C42" s="6" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="D42" s="6" t="s">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="E42" s="6" t="s">
         <x:v>259</x:v>
       </x:c>
-      <x:c r="B42" s="6" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="C42" s="6" t="s">
-        <x:v>247</x:v>
-      </x:c>
-      <x:c r="D42" s="6" t="s">
+      <x:c r="F42" s="6" t="s">
         <x:v>260</x:v>
-      </x:c>
-      <x:c r="E42" s="6" t="s">
-        <x:v>261</x:v>
-      </x:c>
-      <x:c r="F42" s="6" t="s">
-        <x:v>262</x:v>
       </x:c>
       <x:c r="G42" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H42" s="6" t="s">
-        <x:v>263</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="I42" s="6" t="s">
-        <x:v>264</x:v>
+        <x:v>262</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="54" customHeight="1">
       <x:c r="A43" s="5" t="s">
+        <x:v>263</x:v>
+      </x:c>
+      <x:c r="B43" s="5" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="C43" s="5" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="D43" s="5" t="s">
+        <x:v>264</x:v>
+      </x:c>
+      <x:c r="E43" s="5" t="s">
         <x:v>265</x:v>
       </x:c>
-      <x:c r="B43" s="5" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="C43" s="5" t="s">
-        <x:v>247</x:v>
-      </x:c>
-      <x:c r="D43" s="5" t="s">
+      <x:c r="F43" s="5" t="s">
         <x:v>266</x:v>
-      </x:c>
-      <x:c r="E43" s="5" t="s">
-        <x:v>267</x:v>
-      </x:c>
-      <x:c r="F43" s="5" t="s">
-        <x:v>268</x:v>
       </x:c>
       <x:c r="G43" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H43" s="5" t="s">
-        <x:v>269</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="I43" s="5" t="s">
-        <x:v>270</x:v>
+        <x:v>268</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="54" customHeight="1">
       <x:c r="A44" s="6" t="s">
+        <x:v>269</x:v>
+      </x:c>
+      <x:c r="B44" s="6" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="C44" s="6" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="D44" s="6" t="s">
+        <x:v>270</x:v>
+      </x:c>
+      <x:c r="E44" s="6" t="s">
         <x:v>271</x:v>
       </x:c>
-      <x:c r="B44" s="6" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="C44" s="6" t="s">
-        <x:v>247</x:v>
-      </x:c>
-      <x:c r="D44" s="6" t="s">
+      <x:c r="F44" s="6" t="s">
         <x:v>272</x:v>
-      </x:c>
-      <x:c r="E44" s="6" t="s">
-        <x:v>273</x:v>
-      </x:c>
-      <x:c r="F44" s="6" t="s">
-        <x:v>274</x:v>
       </x:c>
       <x:c r="G44" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H44" s="6" t="s">
-        <x:v>275</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="I44" s="6" t="s">
-        <x:v>276</x:v>
+        <x:v>274</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="54" customHeight="1">
       <x:c r="A45" s="5" t="s">
+        <x:v>275</x:v>
+      </x:c>
+      <x:c r="B45" s="5" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="C45" s="5" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="D45" s="5" t="s">
+        <x:v>276</x:v>
+      </x:c>
+      <x:c r="E45" s="5" t="s">
         <x:v>277</x:v>
       </x:c>
-      <x:c r="B45" s="5" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="C45" s="5" t="s">
-        <x:v>247</x:v>
-      </x:c>
-      <x:c r="D45" s="5" t="s">
+      <x:c r="F45" s="5" t="s">
         <x:v>278</x:v>
-      </x:c>
-      <x:c r="E45" s="5" t="s">
-        <x:v>279</x:v>
-      </x:c>
-      <x:c r="F45" s="5" t="s">
-        <x:v>280</x:v>
       </x:c>
       <x:c r="G45" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H45" s="5" t="s">
-        <x:v>281</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="I45" s="5" t="s">
-        <x:v>282</x:v>
+        <x:v>280</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="54" customHeight="1">
       <x:c r="A46" s="6" t="s">
+        <x:v>281</x:v>
+      </x:c>
+      <x:c r="B46" s="6" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="C46" s="6" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="D46" s="6" t="s">
+        <x:v>282</x:v>
+      </x:c>
+      <x:c r="E46" s="6" t="s">
         <x:v>283</x:v>
       </x:c>
-      <x:c r="B46" s="6" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="C46" s="6" t="s">
-        <x:v>247</x:v>
-      </x:c>
-      <x:c r="D46" s="6" t="s">
+      <x:c r="F46" s="6" t="s">
         <x:v>284</x:v>
-      </x:c>
-      <x:c r="E46" s="6" t="s">
-        <x:v>285</x:v>
-      </x:c>
-      <x:c r="F46" s="6" t="s">
-        <x:v>286</x:v>
       </x:c>
       <x:c r="G46" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H46" s="6" t="s">
-        <x:v>287</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="I46" s="6" t="s">
-        <x:v>288</x:v>
+        <x:v>286</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="54" customHeight="1">
       <x:c r="A47" s="5" t="s">
+        <x:v>287</x:v>
+      </x:c>
+      <x:c r="B47" s="5" t="s">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="C47" s="5" t="s">
         <x:v>289</x:v>
       </x:c>
-      <x:c r="B47" s="5" t="s">
+      <x:c r="D47" s="5" t="s">
         <x:v>290</x:v>
       </x:c>
-      <x:c r="C47" s="5" t="s">
+      <x:c r="E47" s="5" t="s">
         <x:v>291</x:v>
       </x:c>
-      <x:c r="D47" s="5" t="s">
+      <x:c r="F47" s="5" t="s">
         <x:v>292</x:v>
-      </x:c>
-      <x:c r="E47" s="5" t="s">
-        <x:v>293</x:v>
-      </x:c>
-      <x:c r="F47" s="5" t="s">
-        <x:v>294</x:v>
       </x:c>
       <x:c r="G47" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H47" s="5" t="s">
-        <x:v>295</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="I47" s="5" t="s">
-        <x:v>296</x:v>
+        <x:v>294</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="54" customHeight="1">
       <x:c r="A48" s="6" t="s">
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="B48" s="6" t="s">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="C48" s="6" t="s">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="D48" s="6" t="s">
+        <x:v>296</x:v>
+      </x:c>
+      <x:c r="E48" s="6" t="s">
         <x:v>297</x:v>
       </x:c>
-      <x:c r="B48" s="6" t="s">
-        <x:v>290</x:v>
-      </x:c>
-      <x:c r="C48" s="6" t="s">
-        <x:v>291</x:v>
-      </x:c>
-      <x:c r="D48" s="6" t="s">
+      <x:c r="F48" s="6" t="s">
         <x:v>298</x:v>
-      </x:c>
-      <x:c r="E48" s="6" t="s">
-        <x:v>299</x:v>
-      </x:c>
-      <x:c r="F48" s="6" t="s">
-        <x:v>300</x:v>
       </x:c>
       <x:c r="G48" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H48" s="6" t="s">
-        <x:v>301</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="I48" s="6" t="s">
-        <x:v>302</x:v>
+        <x:v>300</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="54" customHeight="1">
       <x:c r="A49" s="5" t="s">
+        <x:v>301</x:v>
+      </x:c>
+      <x:c r="B49" s="5" t="s">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="C49" s="5" t="s">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="D49" s="5" t="s">
+        <x:v>302</x:v>
+      </x:c>
+      <x:c r="E49" s="5" t="s">
         <x:v>303</x:v>
       </x:c>
-      <x:c r="B49" s="5" t="s">
-        <x:v>290</x:v>
-      </x:c>
-      <x:c r="C49" s="5" t="s">
-        <x:v>291</x:v>
-      </x:c>
-      <x:c r="D49" s="5" t="s">
+      <x:c r="F49" s="5" t="s">
         <x:v>304</x:v>
-      </x:c>
-      <x:c r="E49" s="5" t="s">
-        <x:v>305</x:v>
-      </x:c>
-      <x:c r="F49" s="5" t="s">
-        <x:v>306</x:v>
       </x:c>
       <x:c r="G49" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H49" s="5" t="s">
-        <x:v>307</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="I49" s="5" t="s">
-        <x:v>308</x:v>
+        <x:v>306</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="54" customHeight="1">
       <x:c r="A50" s="6" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="B50" s="6" t="s">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="C50" s="6" t="s">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="D50" s="6" t="s">
+        <x:v>308</x:v>
+      </x:c>
+      <x:c r="E50" s="6" t="s">
         <x:v>309</x:v>
       </x:c>
-      <x:c r="B50" s="6" t="s">
-        <x:v>290</x:v>
-      </x:c>
-      <x:c r="C50" s="6" t="s">
-        <x:v>291</x:v>
-      </x:c>
-      <x:c r="D50" s="6" t="s">
+      <x:c r="F50" s="6" t="s">
         <x:v>310</x:v>
-      </x:c>
-      <x:c r="E50" s="6" t="s">
-        <x:v>311</x:v>
-      </x:c>
-      <x:c r="F50" s="6" t="s">
-        <x:v>312</x:v>
       </x:c>
       <x:c r="G50" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H50" s="6" t="s">
-        <x:v>313</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="I50" s="6" t="s">
-        <x:v>314</x:v>
+        <x:v>312</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="54" customHeight="1">
       <x:c r="A51" s="5" t="s">
+        <x:v>313</x:v>
+      </x:c>
+      <x:c r="B51" s="5" t="s">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="C51" s="5" t="s">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="D51" s="5" t="s">
+        <x:v>314</x:v>
+      </x:c>
+      <x:c r="E51" s="5" t="s">
         <x:v>315</x:v>
       </x:c>
-      <x:c r="B51" s="5" t="s">
-        <x:v>290</x:v>
-      </x:c>
-      <x:c r="C51" s="5" t="s">
-        <x:v>291</x:v>
-      </x:c>
-      <x:c r="D51" s="5" t="s">
+      <x:c r="F51" s="5" t="s">
         <x:v>316</x:v>
-      </x:c>
-      <x:c r="E51" s="5" t="s">
-        <x:v>317</x:v>
-      </x:c>
-      <x:c r="F51" s="5" t="s">
-        <x:v>318</x:v>
       </x:c>
       <x:c r="G51" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H51" s="5" t="s">
-        <x:v>319</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="I51" s="5" t="s">
-        <x:v>320</x:v>
+        <x:v>318</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="54" customHeight="1">
       <x:c r="A52" s="6" t="s">
+        <x:v>319</x:v>
+      </x:c>
+      <x:c r="B52" s="6" t="s">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="C52" s="6" t="s">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="D52" s="6" t="s">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="E52" s="6" t="s">
         <x:v>321</x:v>
       </x:c>
-      <x:c r="B52" s="6" t="s">
-        <x:v>290</x:v>
-      </x:c>
-      <x:c r="C52" s="6" t="s">
-        <x:v>291</x:v>
-      </x:c>
-      <x:c r="D52" s="6" t="s">
+      <x:c r="F52" s="6" t="s">
         <x:v>322</x:v>
-      </x:c>
-      <x:c r="E52" s="6" t="s">
-        <x:v>323</x:v>
-      </x:c>
-      <x:c r="F52" s="6" t="s">
-        <x:v>324</x:v>
       </x:c>
       <x:c r="G52" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H52" s="6" t="s">
-        <x:v>325</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="I52" s="6" t="s">
-        <x:v>326</x:v>
+        <x:v>324</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="54" customHeight="1">
       <x:c r="A53" s="5" t="s">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="B53" s="5" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="C53" s="5" t="s">
         <x:v>327</x:v>
       </x:c>
-      <x:c r="B53" s="5" t="s">
+      <x:c r="D53" s="5" t="s">
         <x:v>328</x:v>
       </x:c>
-      <x:c r="C53" s="5" t="s">
+      <x:c r="E53" s="5" t="s">
         <x:v>329</x:v>
       </x:c>
-      <x:c r="D53" s="5" t="s">
+      <x:c r="F53" s="5" t="s">
         <x:v>330</x:v>
-      </x:c>
-      <x:c r="E53" s="5" t="s">
-        <x:v>331</x:v>
-      </x:c>
-      <x:c r="F53" s="5" t="s">
-        <x:v>332</x:v>
       </x:c>
       <x:c r="G53" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H53" s="5" t="s">
-        <x:v>333</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="I53" s="5" t="s">
-        <x:v>334</x:v>
+        <x:v>332</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="54" customHeight="1">
       <x:c r="A54" s="6" t="s">
+        <x:v>333</x:v>
+      </x:c>
+      <x:c r="B54" s="6" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="C54" s="6" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="D54" s="6" t="s">
+        <x:v>334</x:v>
+      </x:c>
+      <x:c r="E54" s="6" t="s">
         <x:v>335</x:v>
       </x:c>
-      <x:c r="B54" s="6" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="C54" s="6" t="s">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="D54" s="6" t="s">
+      <x:c r="F54" s="6" t="s">
         <x:v>336</x:v>
-      </x:c>
-      <x:c r="E54" s="6" t="s">
-        <x:v>337</x:v>
-      </x:c>
-      <x:c r="F54" s="6" t="s">
-        <x:v>338</x:v>
       </x:c>
       <x:c r="G54" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H54" s="6" t="s">
-        <x:v>339</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="I54" s="6" t="s">
-        <x:v>340</x:v>
+        <x:v>338</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="54" customHeight="1">
       <x:c r="A55" s="5" t="s">
+        <x:v>339</x:v>
+      </x:c>
+      <x:c r="B55" s="5" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="C55" s="5" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="D55" s="5" t="s">
+        <x:v>340</x:v>
+      </x:c>
+      <x:c r="E55" s="5" t="s">
         <x:v>341</x:v>
       </x:c>
-      <x:c r="B55" s="5" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="C55" s="5" t="s">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="D55" s="5" t="s">
+      <x:c r="F55" s="5" t="s">
         <x:v>342</x:v>
-      </x:c>
-      <x:c r="E55" s="5" t="s">
-        <x:v>343</x:v>
-      </x:c>
-      <x:c r="F55" s="5" t="s">
-        <x:v>344</x:v>
       </x:c>
       <x:c r="G55" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H55" s="5" t="s">
-        <x:v>345</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="I55" s="5" t="s">
-        <x:v>346</x:v>
+        <x:v>344</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="54" customHeight="1">
       <x:c r="A56" s="6" t="s">
+        <x:v>345</x:v>
+      </x:c>
+      <x:c r="B56" s="6" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="C56" s="6" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="D56" s="6" t="s">
+        <x:v>346</x:v>
+      </x:c>
+      <x:c r="E56" s="6" t="s">
         <x:v>347</x:v>
       </x:c>
-      <x:c r="B56" s="6" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="C56" s="6" t="s">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="D56" s="6" t="s">
+      <x:c r="F56" s="6" t="s">
         <x:v>348</x:v>
-      </x:c>
-      <x:c r="E56" s="6" t="s">
-        <x:v>349</x:v>
-      </x:c>
-      <x:c r="F56" s="6" t="s">
-        <x:v>350</x:v>
       </x:c>
       <x:c r="G56" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H56" s="6" t="s">
-        <x:v>351</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="I56" s="6" t="s">
-        <x:v>352</x:v>
+        <x:v>350</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="54" customHeight="1">
       <x:c r="A57" s="5" t="s">
+        <x:v>351</x:v>
+      </x:c>
+      <x:c r="B57" s="5" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="C57" s="5" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="D57" s="5" t="s">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="E57" s="5" t="s">
         <x:v>353</x:v>
       </x:c>
-      <x:c r="B57" s="5" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="C57" s="5" t="s">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="D57" s="5" t="s">
+      <x:c r="F57" s="5" t="s">
         <x:v>354</x:v>
-      </x:c>
-      <x:c r="E57" s="5" t="s">
-        <x:v>355</x:v>
-      </x:c>
-      <x:c r="F57" s="5" t="s">
-        <x:v>356</x:v>
       </x:c>
       <x:c r="G57" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H57" s="5" t="s">
-        <x:v>357</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="I57" s="5" t="s">
-        <x:v>358</x:v>
+        <x:v>356</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="54" customHeight="1">
       <x:c r="A58" s="6" t="s">
+        <x:v>357</x:v>
+      </x:c>
+      <x:c r="B58" s="6" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="C58" s="6" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="D58" s="6" t="s">
+        <x:v>358</x:v>
+      </x:c>
+      <x:c r="E58" s="6" t="s">
         <x:v>359</x:v>
       </x:c>
-      <x:c r="B58" s="6" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="C58" s="6" t="s">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="D58" s="6" t="s">
+      <x:c r="F58" s="6" t="s">
         <x:v>360</x:v>
-      </x:c>
-      <x:c r="E58" s="6" t="s">
-        <x:v>361</x:v>
-      </x:c>
-      <x:c r="F58" s="6" t="s">
-        <x:v>362</x:v>
       </x:c>
       <x:c r="G58" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H58" s="6" t="s">
-        <x:v>363</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="I58" s="6" t="s">
-        <x:v>364</x:v>
+        <x:v>362</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="54" customHeight="1">
       <x:c r="A59" s="5" t="s">
+        <x:v>363</x:v>
+      </x:c>
+      <x:c r="B59" s="5" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="C59" s="5" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="D59" s="5" t="s">
+        <x:v>364</x:v>
+      </x:c>
+      <x:c r="E59" s="5" t="s">
         <x:v>365</x:v>
       </x:c>
-      <x:c r="B59" s="5" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="C59" s="5" t="s">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="D59" s="5" t="s">
+      <x:c r="F59" s="5" t="s">
         <x:v>366</x:v>
-      </x:c>
-      <x:c r="E59" s="5" t="s">
-        <x:v>367</x:v>
-      </x:c>
-      <x:c r="F59" s="5" t="s">
-        <x:v>368</x:v>
       </x:c>
       <x:c r="G59" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H59" s="5" t="s">
-        <x:v>369</x:v>
+        <x:v>367</x:v>
       </x:c>
       <x:c r="I59" s="5" t="s">
-        <x:v>370</x:v>
+        <x:v>368</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="54" customHeight="1">
       <x:c r="A60" s="6" t="s">
+        <x:v>369</x:v>
+      </x:c>
+      <x:c r="B60" s="6" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="C60" s="6" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="D60" s="6" t="s">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="E60" s="6" t="s">
         <x:v>371</x:v>
       </x:c>
-      <x:c r="B60" s="6" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="C60" s="6" t="s">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="D60" s="6" t="s">
+      <x:c r="F60" s="6" t="s">
         <x:v>372</x:v>
-      </x:c>
-      <x:c r="E60" s="6" t="s">
-        <x:v>373</x:v>
-      </x:c>
-      <x:c r="F60" s="6" t="s">
-        <x:v>374</x:v>
       </x:c>
       <x:c r="G60" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H60" s="6" t="s">
-        <x:v>375</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="I60" s="6" t="s">
-        <x:v>376</x:v>
+        <x:v>374</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="52" customHeight="1">
@@ -4202,7 +4207,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R720c4e0310b6447c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93befcb22a1243bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: concluir FT-054 a FT-057
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R9cc8134812e24f16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rb894e47b376f4e6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rcf70295a3b6b47f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R9211be3e245644f6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,12 +362,6 @@
     <x:t xml:space="preserve">Exibir categorias matemático, heurístico, literatura, experimental, calibrado e bloqueado, vinculadas à proveniência e aos bloqueios já existentes.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Os limites aparecem como texto e recommendation_blocked, mas não há componente visual uniforme de maturidade.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Mapear cada selo para estados contratuais verificáveis; não inferir maturidade pela aparência.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">FT-055</x:t>
   </x:si>
   <x:si>
@@ -380,12 +374,6 @@
     <x:t xml:space="preserve">Comparar dois ou três valores de alpha, catalisadores ou condições; sobrepor curvas e mostrar diferenças, entradas, unidades, evidência e bloqueios.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">A plataforma executa um caso por vez e não mantém comparação visual entre cenários.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Executar após FT-052 a FT-054; limitar comparações às regras e evidências compatíveis.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">FT-056</x:t>
   </x:si>
   <x:si>
@@ -396,12 +384,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Testar fluxos, responsividade, acessibilidade, estados vazios e erros, regressão do worker, Streamlit e contratos; publicar revisão e executar teste de fumaça.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">A suíte atual tem 53 testes, mas ainda não cobre o novo fluxo de UX nem seus pontos de quebra.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Executar após FT-049 a FT-055; só então liberar a retomada do backlog científico anterior.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">FT-010</x:t>
@@ -1143,7 +1125,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="164" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="17">
+  <x:fonts count="18">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -1255,8 +1237,14 @@
       <x:name val="Arial"/>
       <x:family val="2"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF245C2C"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="23">
+  <x:fills count="24">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1356,6 +1344,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF3F8F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEFD8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -1494,7 +1487,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="54">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1621,6 +1614,18 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="22" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="23" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="23" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="23" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="23" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1953,14 +1958,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E5" s="16" t="n">
-        <x:v>20</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F5" s="12"/>
       <x:c r="G5" s="15" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="H5" s="17" t="n">
-        <x:v>0.31746031746031744</x:v>
+        <x:v>0.38095238095238093</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -2002,7 +2007,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B9" s="20" t="n">
-        <x:v>20</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C9" s="12"/>
       <x:c r="D9" s="12"/>
@@ -2030,7 +2035,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B11" s="20" t="n">
-        <x:v>22</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C11" s="12"/>
       <x:c r="D11" s="12"/>
@@ -2220,7 +2225,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B26" s="21" t="str">
-        <x:v>tests/ — 68 testes e 15 subtestes aprovados na verificação de FT-053 em 2026-10-13</x:v>
+        <x:v>tests/ — 78 testes e 15 subtestes aprovados na verificação de FT-054 a FT-057 em 2026-10-13</x:v>
       </x:c>
       <x:c r="C26" s="12"/>
       <x:c r="D26" s="12"/>
@@ -2234,7 +2239,7 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B27" s="21" t="str">
-        <x:v>FT-053 validada localmente; publicação pública depende do redeploy da revisão no Streamlit</x:v>
+        <x:v>Aplicação local e saúde HTTP 200; revisão enviada ao GitHub; conteúdo do deploy público deve ser confirmado após atualização automática</x:v>
       </x:c>
       <x:c r="C27" s="12"/>
       <x:c r="D27" s="12"/>
@@ -2248,7 +2253,7 @@
         <x:v>Expansão planejada</x:v>
       </x:c>
       <x:c r="B28" s="45" t="str">
-        <x:v>FT-057 a FT-063: cinética, reator, termodinâmica, balanços, avaliação econômica e validação integrada</x:v>
+        <x:v>FT-058 a FT-063: reator, termodinâmica, balanços, avaliação econômica e validação integrada</x:v>
       </x:c>
       <x:c r="C28" s="12"/>
       <x:c r="D28" s="12"/>
@@ -2787,19 +2792,19 @@
       <x:c r="F19" s="7" t="s">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="G19" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H19" s="7" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="I19" s="7" t="s">
-        <x:v>118</x:v>
+      <x:c r="G19" s="51" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="H19" s="7" t="str">
+        <x:v>Categorias em evidence_maturity.py e selos textuais/visuais em ui_design.py; proveniência e limitação aparecem junto do resultado; catálogo completo na etapa Evidências.</x:v>
+      </x:c>
+      <x:c r="I19" s="7" t="str">
+        <x:v>Manter as categorias ligadas a estados explícitos; não promover maturidade pela aparência.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
       <x:c r="A20" s="7" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B20" s="7" t="s">
         <x:v>37</x:v>
@@ -2808,27 +2813,27 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="D20" s="7" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="E20" s="7" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="F20" s="7" t="s">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="E20" s="7" t="s">
-        <x:v>121</x:v>
-      </x:c>
-      <x:c r="F20" s="7" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="G20" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H20" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="I20" s="7" t="s">
-        <x:v>124</x:v>
+      <x:c r="G20" s="51" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="H20" s="7" t="str">
+        <x:v>Comparação de 2 ou 3 cenários em scenario_comparison.py e app.py: curvas e faixas ASF na mesma base, entradas visíveis e recommendation_blocked preservado.</x:v>
+      </x:c>
+      <x:c r="I20" s="7" t="str">
+        <x:v>Usar somente como sensibilidade matemática; exigir novo contrato para comparar cinéticas ou desempenho experimental.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
       <x:c r="A21" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B21" s="7" t="s">
         <x:v>37</x:v>
@@ -2837,27 +2842,27 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="D21" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="E21" s="7" t="s">
-        <x:v>127</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="F21" s="7" t="s">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="G21" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H21" s="7" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="I21" s="7" t="s">
-        <x:v>130</x:v>
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="G21" s="51" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="H21" s="7" t="str">
+        <x:v>Aceite em docs/ACEITE_UX_FT_056.md; 78 testes e 15 subtestes; fluxo Streamlit, responsividade 390 x 844, acessibilidade, gráficos e HTTP 200 verificados; CI adicionada.</x:v>
+      </x:c>
+      <x:c r="I21" s="7" t="str">
+        <x:v>Monitorar o deploy público do commit e manter a suíte obrigatória em cada mudança.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="54" customHeight="1">
       <x:c r="A22" s="6" t="s">
-        <x:v>131</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B22" s="6" t="s">
         <x:v>37</x:v>
@@ -2866,1124 +2871,1124 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="D22" s="6" t="s">
-        <x:v>132</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="E22" s="6" t="s">
-        <x:v>133</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="F22" s="6" t="s">
-        <x:v>134</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="G22" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H22" s="6" t="s">
-        <x:v>135</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="I22" s="6" t="s">
-        <x:v>136</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
       <x:c r="A23" s="5" t="s">
-        <x:v>137</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B23" s="5" t="s">
-        <x:v>138</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C23" s="5" t="s">
-        <x:v>139</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D23" s="5" t="s">
-        <x:v>140</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="E23" s="5" t="s">
-        <x:v>141</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="F23" s="5" t="s">
-        <x:v>142</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="G23" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H23" s="5" t="s">
-        <x:v>143</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="I23" s="5" t="s">
-        <x:v>144</x:v>
+        <x:v>138</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
       <x:c r="A24" s="6" t="s">
-        <x:v>145</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B24" s="6" t="s">
-        <x:v>138</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C24" s="6" t="s">
-        <x:v>139</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D24" s="6" t="s">
-        <x:v>146</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="E24" s="6" t="s">
-        <x:v>147</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="F24" s="6" t="s">
-        <x:v>148</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="G24" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H24" s="6" t="s">
-        <x:v>149</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="I24" s="6" t="s">
-        <x:v>150</x:v>
+        <x:v>144</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="54" customHeight="1">
       <x:c r="A25" s="5" t="s">
-        <x:v>151</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="B25" s="5" t="s">
-        <x:v>138</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C25" s="5" t="s">
-        <x:v>139</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D25" s="5" t="s">
-        <x:v>152</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="E25" s="5" t="s">
-        <x:v>153</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="F25" s="5" t="s">
-        <x:v>154</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="G25" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H25" s="5" t="s">
-        <x:v>155</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="I25" s="5" t="s">
-        <x:v>156</x:v>
+        <x:v>150</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="54" customHeight="1">
       <x:c r="A26" s="6" t="s">
-        <x:v>157</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B26" s="6" t="s">
-        <x:v>138</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C26" s="6" t="s">
-        <x:v>139</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D26" s="6" t="s">
-        <x:v>158</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="E26" s="6" t="s">
-        <x:v>159</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="F26" s="6" t="s">
-        <x:v>160</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="G26" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H26" s="6" t="s">
-        <x:v>161</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="I26" s="6" t="s">
-        <x:v>162</x:v>
+        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="54" customHeight="1">
       <x:c r="A27" s="5" t="s">
-        <x:v>163</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="B27" s="5" t="s">
-        <x:v>138</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C27" s="5" t="s">
-        <x:v>139</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D27" s="5" t="s">
-        <x:v>164</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="E27" s="5" t="s">
-        <x:v>165</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="F27" s="5" t="s">
-        <x:v>166</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="G27" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H27" s="5" t="s">
-        <x:v>167</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="I27" s="5" t="s">
-        <x:v>168</x:v>
+        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="54" customHeight="1">
       <x:c r="A28" s="6" t="s">
-        <x:v>169</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="B28" s="6" t="s">
-        <x:v>138</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C28" s="6" t="s">
-        <x:v>139</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D28" s="6" t="s">
-        <x:v>170</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="E28" s="6" t="s">
-        <x:v>171</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="F28" s="6" t="s">
-        <x:v>172</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="G28" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H28" s="6" t="s">
-        <x:v>173</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="I28" s="6" t="s">
-        <x:v>174</x:v>
+        <x:v>168</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="54" customHeight="1">
       <x:c r="A29" s="5" t="s">
-        <x:v>175</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="B29" s="5" t="s">
-        <x:v>138</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C29" s="5" t="s">
-        <x:v>139</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D29" s="5" t="s">
-        <x:v>176</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="E29" s="5" t="s">
-        <x:v>177</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="F29" s="5" t="s">
-        <x:v>178</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="G29" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H29" s="5" t="s">
-        <x:v>179</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="I29" s="5" t="s">
-        <x:v>180</x:v>
+        <x:v>174</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="54" customHeight="1">
       <x:c r="A30" s="6" t="s">
-        <x:v>181</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="B30" s="6" t="s">
-        <x:v>138</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C30" s="6" t="s">
-        <x:v>139</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D30" s="6" t="s">
-        <x:v>182</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="E30" s="6" t="s">
-        <x:v>183</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="F30" s="6" t="s">
-        <x:v>184</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="G30" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H30" s="6" t="s">
-        <x:v>185</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="I30" s="6" t="s">
-        <x:v>186</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="54" customHeight="1">
       <x:c r="A31" s="5" t="s">
-        <x:v>187</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="B31" s="5" t="s">
-        <x:v>138</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C31" s="5" t="s">
-        <x:v>139</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D31" s="5" t="s">
-        <x:v>188</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="E31" s="5" t="s">
-        <x:v>189</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="F31" s="5" t="s">
-        <x:v>190</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="G31" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H31" s="5" t="s">
-        <x:v>191</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="I31" s="5" t="s">
-        <x:v>192</x:v>
+        <x:v>186</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="54" customHeight="1">
       <x:c r="A32" s="6" t="s">
-        <x:v>193</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B32" s="6" t="s">
-        <x:v>138</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C32" s="6" t="s">
-        <x:v>139</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D32" s="6" t="s">
-        <x:v>194</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="E32" s="6" t="s">
-        <x:v>195</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="F32" s="6" t="s">
-        <x:v>196</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="G32" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H32" s="6" t="s">
-        <x:v>197</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="I32" s="6" t="s">
-        <x:v>198</x:v>
+        <x:v>192</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="54" customHeight="1">
       <x:c r="A33" s="5" t="s">
-        <x:v>199</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="B33" s="5" t="s">
-        <x:v>200</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="C33" s="5" t="s">
-        <x:v>201</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="D33" s="5" t="s">
-        <x:v>202</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="E33" s="5" t="s">
-        <x:v>203</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="F33" s="5" t="s">
-        <x:v>204</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="G33" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H33" s="5" t="s">
-        <x:v>205</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="I33" s="5" t="s">
-        <x:v>206</x:v>
+        <x:v>200</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="54" customHeight="1">
       <x:c r="A34" s="6" t="s">
-        <x:v>207</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="B34" s="6" t="s">
-        <x:v>200</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="C34" s="6" t="s">
-        <x:v>201</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="D34" s="6" t="s">
-        <x:v>208</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="E34" s="6" t="s">
-        <x:v>209</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="F34" s="6" t="s">
-        <x:v>210</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="G34" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H34" s="6" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="I34" s="6" t="s">
-        <x:v>212</x:v>
+        <x:v>206</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="54" customHeight="1">
       <x:c r="A35" s="5" t="s">
-        <x:v>213</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="B35" s="5" t="s">
-        <x:v>200</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="C35" s="5" t="s">
-        <x:v>201</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="D35" s="5" t="s">
-        <x:v>214</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="E35" s="5" t="s">
-        <x:v>215</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="F35" s="5" t="s">
-        <x:v>216</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="G35" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H35" s="5" t="s">
-        <x:v>217</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="I35" s="5" t="s">
-        <x:v>218</x:v>
+        <x:v>212</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="54" customHeight="1">
       <x:c r="A36" s="6" t="s">
-        <x:v>219</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="B36" s="6" t="s">
-        <x:v>200</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="C36" s="6" t="s">
-        <x:v>201</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="D36" s="6" t="s">
-        <x:v>220</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="E36" s="6" t="s">
-        <x:v>221</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="F36" s="6" t="s">
-        <x:v>222</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G36" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H36" s="6" t="s">
-        <x:v>223</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="I36" s="6" t="s">
-        <x:v>224</x:v>
+        <x:v>218</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="54" customHeight="1">
       <x:c r="A37" s="5" t="s">
-        <x:v>225</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="B37" s="5" t="s">
-        <x:v>200</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="C37" s="5" t="s">
-        <x:v>201</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="D37" s="5" t="s">
-        <x:v>226</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="E37" s="5" t="s">
-        <x:v>227</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="F37" s="5" t="s">
-        <x:v>228</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="G37" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H37" s="5" t="s">
-        <x:v>229</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="I37" s="5" t="s">
-        <x:v>230</x:v>
+        <x:v>224</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="54" customHeight="1">
       <x:c r="A38" s="6" t="s">
-        <x:v>231</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="B38" s="6" t="s">
-        <x:v>200</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="C38" s="6" t="s">
-        <x:v>201</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="D38" s="6" t="s">
-        <x:v>232</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="E38" s="6" t="s">
-        <x:v>233</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="F38" s="6" t="s">
-        <x:v>234</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="G38" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H38" s="6" t="s">
-        <x:v>235</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="I38" s="6" t="s">
-        <x:v>236</x:v>
+        <x:v>230</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="54" customHeight="1">
       <x:c r="A39" s="5" t="s">
-        <x:v>237</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="B39" s="5" t="s">
-        <x:v>200</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="C39" s="5" t="s">
-        <x:v>201</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="D39" s="5" t="s">
-        <x:v>238</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="E39" s="5" t="s">
-        <x:v>239</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="F39" s="5" t="s">
-        <x:v>240</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="G39" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H39" s="5" t="s">
-        <x:v>241</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="I39" s="5" t="s">
-        <x:v>242</x:v>
+        <x:v>236</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="54" customHeight="1">
       <x:c r="A40" s="6" t="s">
-        <x:v>243</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="B40" s="6" t="s">
-        <x:v>244</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="C40" s="6" t="s">
-        <x:v>245</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D40" s="6" t="s">
-        <x:v>246</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="E40" s="6" t="s">
-        <x:v>247</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="F40" s="6" t="s">
-        <x:v>248</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="G40" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H40" s="6" t="s">
-        <x:v>249</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="I40" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>244</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="54" customHeight="1">
       <x:c r="A41" s="5" t="s">
-        <x:v>251</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="B41" s="5" t="s">
-        <x:v>244</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="C41" s="5" t="s">
-        <x:v>245</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D41" s="5" t="s">
-        <x:v>252</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="E41" s="5" t="s">
-        <x:v>253</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="F41" s="5" t="s">
-        <x:v>254</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="G41" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H41" s="5" t="s">
-        <x:v>255</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="I41" s="5" t="s">
-        <x:v>256</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="54" customHeight="1">
       <x:c r="A42" s="6" t="s">
-        <x:v>257</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="B42" s="6" t="s">
-        <x:v>244</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="C42" s="6" t="s">
-        <x:v>245</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D42" s="6" t="s">
-        <x:v>258</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="E42" s="6" t="s">
-        <x:v>259</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="F42" s="6" t="s">
-        <x:v>260</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="G42" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H42" s="6" t="s">
-        <x:v>261</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="I42" s="6" t="s">
-        <x:v>262</x:v>
+        <x:v>256</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="54" customHeight="1">
       <x:c r="A43" s="5" t="s">
-        <x:v>263</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="B43" s="5" t="s">
-        <x:v>244</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="C43" s="5" t="s">
-        <x:v>245</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D43" s="5" t="s">
-        <x:v>264</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="E43" s="5" t="s">
-        <x:v>265</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="F43" s="5" t="s">
-        <x:v>266</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="G43" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H43" s="5" t="s">
-        <x:v>267</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="I43" s="5" t="s">
-        <x:v>268</x:v>
+        <x:v>262</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="54" customHeight="1">
       <x:c r="A44" s="6" t="s">
-        <x:v>269</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="B44" s="6" t="s">
-        <x:v>244</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="C44" s="6" t="s">
-        <x:v>245</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D44" s="6" t="s">
-        <x:v>270</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="E44" s="6" t="s">
-        <x:v>271</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="F44" s="6" t="s">
-        <x:v>272</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="G44" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H44" s="6" t="s">
-        <x:v>273</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="I44" s="6" t="s">
-        <x:v>274</x:v>
+        <x:v>268</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="54" customHeight="1">
       <x:c r="A45" s="5" t="s">
-        <x:v>275</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="B45" s="5" t="s">
-        <x:v>244</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="C45" s="5" t="s">
-        <x:v>245</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D45" s="5" t="s">
-        <x:v>276</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="E45" s="5" t="s">
-        <x:v>277</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="F45" s="5" t="s">
-        <x:v>278</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="G45" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H45" s="5" t="s">
-        <x:v>279</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="I45" s="5" t="s">
-        <x:v>280</x:v>
+        <x:v>274</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="54" customHeight="1">
       <x:c r="A46" s="6" t="s">
-        <x:v>281</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="B46" s="6" t="s">
-        <x:v>244</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="C46" s="6" t="s">
-        <x:v>245</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D46" s="6" t="s">
-        <x:v>282</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="E46" s="6" t="s">
-        <x:v>283</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="F46" s="6" t="s">
-        <x:v>284</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="G46" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H46" s="6" t="s">
-        <x:v>285</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="I46" s="6" t="s">
-        <x:v>286</x:v>
+        <x:v>280</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="54" customHeight="1">
       <x:c r="A47" s="5" t="s">
-        <x:v>287</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="B47" s="5" t="s">
-        <x:v>288</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="C47" s="5" t="s">
-        <x:v>289</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="D47" s="5" t="s">
-        <x:v>290</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="E47" s="5" t="s">
-        <x:v>291</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="F47" s="5" t="s">
-        <x:v>292</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="G47" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H47" s="5" t="s">
-        <x:v>293</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="I47" s="5" t="s">
-        <x:v>294</x:v>
+        <x:v>288</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="54" customHeight="1">
       <x:c r="A48" s="6" t="s">
-        <x:v>295</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="B48" s="6" t="s">
-        <x:v>288</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="C48" s="6" t="s">
-        <x:v>289</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="D48" s="6" t="s">
-        <x:v>296</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="E48" s="6" t="s">
-        <x:v>297</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="F48" s="6" t="s">
-        <x:v>298</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="G48" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H48" s="6" t="s">
-        <x:v>299</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="I48" s="6" t="s">
-        <x:v>300</x:v>
+        <x:v>294</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="54" customHeight="1">
       <x:c r="A49" s="5" t="s">
-        <x:v>301</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="B49" s="5" t="s">
-        <x:v>288</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="C49" s="5" t="s">
-        <x:v>289</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="D49" s="5" t="s">
-        <x:v>302</x:v>
+        <x:v>296</x:v>
       </x:c>
       <x:c r="E49" s="5" t="s">
-        <x:v>303</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="F49" s="5" t="s">
-        <x:v>304</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="G49" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H49" s="5" t="s">
-        <x:v>305</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="I49" s="5" t="s">
-        <x:v>306</x:v>
+        <x:v>300</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="54" customHeight="1">
       <x:c r="A50" s="6" t="s">
-        <x:v>307</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="B50" s="6" t="s">
-        <x:v>288</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="C50" s="6" t="s">
-        <x:v>289</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="D50" s="6" t="s">
-        <x:v>308</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="E50" s="6" t="s">
-        <x:v>309</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="F50" s="6" t="s">
-        <x:v>310</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="G50" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H50" s="6" t="s">
-        <x:v>311</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="I50" s="6" t="s">
-        <x:v>312</x:v>
+        <x:v>306</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="54" customHeight="1">
       <x:c r="A51" s="5" t="s">
-        <x:v>313</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="B51" s="5" t="s">
-        <x:v>288</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="C51" s="5" t="s">
-        <x:v>289</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="D51" s="5" t="s">
-        <x:v>314</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="E51" s="5" t="s">
-        <x:v>315</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="F51" s="5" t="s">
-        <x:v>316</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="G51" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H51" s="5" t="s">
-        <x:v>317</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="I51" s="5" t="s">
-        <x:v>318</x:v>
+        <x:v>312</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="54" customHeight="1">
       <x:c r="A52" s="6" t="s">
-        <x:v>319</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="B52" s="6" t="s">
-        <x:v>288</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="C52" s="6" t="s">
-        <x:v>289</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="D52" s="6" t="s">
-        <x:v>320</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="E52" s="6" t="s">
-        <x:v>321</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="F52" s="6" t="s">
-        <x:v>322</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="G52" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H52" s="6" t="s">
-        <x:v>323</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="I52" s="6" t="s">
-        <x:v>324</x:v>
+        <x:v>318</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="54" customHeight="1">
       <x:c r="A53" s="5" t="s">
-        <x:v>325</x:v>
+        <x:v>319</x:v>
       </x:c>
       <x:c r="B53" s="5" t="s">
-        <x:v>326</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="C53" s="5" t="s">
-        <x:v>327</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="D53" s="5" t="s">
-        <x:v>328</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="E53" s="5" t="s">
-        <x:v>329</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="F53" s="5" t="s">
-        <x:v>330</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="G53" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H53" s="5" t="s">
-        <x:v>331</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="I53" s="5" t="s">
-        <x:v>332</x:v>
+        <x:v>326</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="54" customHeight="1">
       <x:c r="A54" s="6" t="s">
-        <x:v>333</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="B54" s="6" t="s">
-        <x:v>326</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="C54" s="6" t="s">
-        <x:v>327</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="D54" s="6" t="s">
-        <x:v>334</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="E54" s="6" t="s">
-        <x:v>335</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="F54" s="6" t="s">
-        <x:v>336</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="G54" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H54" s="6" t="s">
-        <x:v>337</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="I54" s="6" t="s">
-        <x:v>338</x:v>
+        <x:v>332</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="54" customHeight="1">
       <x:c r="A55" s="5" t="s">
-        <x:v>339</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="B55" s="5" t="s">
-        <x:v>326</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="C55" s="5" t="s">
-        <x:v>327</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="D55" s="5" t="s">
-        <x:v>340</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="E55" s="5" t="s">
-        <x:v>341</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="F55" s="5" t="s">
-        <x:v>342</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="G55" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H55" s="5" t="s">
-        <x:v>343</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="I55" s="5" t="s">
-        <x:v>344</x:v>
+        <x:v>338</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="54" customHeight="1">
       <x:c r="A56" s="6" t="s">
-        <x:v>345</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="B56" s="6" t="s">
-        <x:v>326</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="C56" s="6" t="s">
-        <x:v>327</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="D56" s="6" t="s">
-        <x:v>346</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="E56" s="6" t="s">
-        <x:v>347</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="F56" s="6" t="s">
-        <x:v>348</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="G56" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H56" s="6" t="s">
-        <x:v>349</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="I56" s="6" t="s">
-        <x:v>350</x:v>
+        <x:v>344</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="54" customHeight="1">
       <x:c r="A57" s="5" t="s">
-        <x:v>351</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="B57" s="5" t="s">
-        <x:v>326</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="C57" s="5" t="s">
-        <x:v>327</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="D57" s="5" t="s">
-        <x:v>352</x:v>
+        <x:v>346</x:v>
       </x:c>
       <x:c r="E57" s="5" t="s">
-        <x:v>353</x:v>
+        <x:v>347</x:v>
       </x:c>
       <x:c r="F57" s="5" t="s">
-        <x:v>354</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="G57" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H57" s="5" t="s">
-        <x:v>355</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="I57" s="5" t="s">
-        <x:v>356</x:v>
+        <x:v>350</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="54" customHeight="1">
       <x:c r="A58" s="6" t="s">
-        <x:v>357</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="B58" s="6" t="s">
-        <x:v>326</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="C58" s="6" t="s">
-        <x:v>327</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="D58" s="6" t="s">
-        <x:v>358</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="E58" s="6" t="s">
-        <x:v>359</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="F58" s="6" t="s">
-        <x:v>360</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="G58" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H58" s="6" t="s">
-        <x:v>361</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="I58" s="6" t="s">
-        <x:v>362</x:v>
+        <x:v>356</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="54" customHeight="1">
       <x:c r="A59" s="5" t="s">
-        <x:v>363</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="B59" s="5" t="s">
-        <x:v>326</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="C59" s="5" t="s">
-        <x:v>327</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="D59" s="5" t="s">
-        <x:v>364</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="E59" s="5" t="s">
-        <x:v>365</x:v>
+        <x:v>359</x:v>
       </x:c>
       <x:c r="F59" s="5" t="s">
-        <x:v>366</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="G59" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H59" s="5" t="s">
-        <x:v>367</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="I59" s="5" t="s">
-        <x:v>368</x:v>
+        <x:v>362</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="54" customHeight="1">
       <x:c r="A60" s="6" t="s">
-        <x:v>369</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="B60" s="6" t="s">
-        <x:v>326</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="C60" s="6" t="s">
-        <x:v>327</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="D60" s="6" t="s">
-        <x:v>370</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="E60" s="6" t="s">
-        <x:v>371</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="F60" s="6" t="s">
-        <x:v>372</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="G60" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H60" s="6" t="s">
-        <x:v>373</x:v>
+        <x:v>367</x:v>
       </x:c>
       <x:c r="I60" s="6" t="s">
-        <x:v>374</x:v>
+        <x:v>368</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="52" customHeight="1">
@@ -4005,14 +4010,14 @@
       <x:c r="F61" s="33" t="str">
         <x:v>Documentar equações, respostas, variáveis, unidades, parâmetros, fonte, ajuste, domínio e incerteza; impedir conversão inferida apenas de temperatura e pressão.</x:v>
       </x:c>
-      <x:c r="G61" s="37" t="str">
-        <x:v>Planejado</x:v>
+      <x:c r="G61" s="53" t="str">
+        <x:v>Concluído</x:v>
       </x:c>
       <x:c r="H61" s="33" t="str">
-        <x:v>Atividade incorporada ao planejamento mestre e ao backlog em 2026-10-13.</x:v>
+        <x:v>Contrato cinético v1 em kinetics.py, schema JSON e docs/CONTRATO_CINETICO_V1.md: variáveis, parâmetros, unidades, domínio, fontes, incerteza, validação e bloqueio de cálculo.</x:v>
       </x:c>
       <x:c r="I61" s="33" t="str">
-        <x:v>Selecionar o primeiro conjunto cinético e os dados de calibração e validação.</x:v>
+        <x:v>Executar FT-058 somente após selecionar e aprovar uma cinética e dados de calibração/validação.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="52" customHeight="1">
@@ -4207,7 +4212,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93befcb22a1243bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcab9aa2ab15d47e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: preparar FT-058 e FT-059
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rcf70295a3b6b47f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R9211be3e245644f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R269845c9c8cf44aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Ra8a3c645e958459c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1125,7 +1125,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="164" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="18">
+  <x:fonts count="19">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -1243,8 +1243,14 @@
       <x:color rgb="FF245C2C"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="24">
+  <x:fills count="26">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1359,6 +1365,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFDCEFD8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -1487,7 +1503,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="54">
+  <x:cellXfs count="58">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1626,6 +1642,18 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="17" fillId="23" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="24" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="24" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="24" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="25" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2021,7 +2049,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B10" s="20" t="n">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C10" s="12"/>
       <x:c r="D10" s="12"/>
@@ -2035,7 +2063,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B11" s="20" t="n">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C11" s="12"/>
       <x:c r="D11" s="12"/>
@@ -2049,7 +2077,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B12" s="20" t="n">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C12" s="12"/>
       <x:c r="D12" s="12"/>
@@ -2225,7 +2253,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B26" s="21" t="str">
-        <x:v>tests/ — 78 testes e 15 subtestes aprovados na verificação de FT-054 a FT-057 em 2026-10-13</x:v>
+        <x:v>tests/ — 87 testes e 15 subtestes aprovados na verificação de FT-058 e FT-059 em 2026-10-13</x:v>
       </x:c>
       <x:c r="C26" s="12"/>
       <x:c r="D26" s="12"/>
@@ -2253,7 +2281,7 @@
         <x:v>Expansão planejada</x:v>
       </x:c>
       <x:c r="B28" s="45" t="str">
-        <x:v>FT-058 a FT-063: reator, termodinâmica, balanços, avaliação econômica e validação integrada</x:v>
+        <x:v>FT-058 e FT-059: infraestrutura parcial; faltam cinética aprovada e dados termodinâmicos de comparação antes de FT-060</x:v>
       </x:c>
       <x:c r="C28" s="12"/>
       <x:c r="D28" s="12"/>
@@ -4039,14 +4067,14 @@
       <x:c r="F62" s="33" t="str">
         <x:v>Formular balanços molares e de energia, alimentação, vazão/GHSV ou WHSV, geometria, pressão, transporte, WGS e desativação conforme a hipótese.</x:v>
       </x:c>
-      <x:c r="G62" s="40" t="str">
-        <x:v>Bloqueado</x:v>
+      <x:c r="G62" s="57" t="str">
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="H62" s="33" t="str">
-        <x:v>Depende de FT-013 a FT-015, FT-017, FT-024 e FT-057.</x:v>
+        <x:v>Contrato do reator, validação de alimentação, geometria, GHSV/WHSV, inventário molar e porta de prontidão implementados em reactor.py, schema e documentação. Não calcula conversão ou produtividade.</x:v>
       </x:c>
       <x:c r="I62" s="33" t="str">
-        <x:v>Concluir caso, balanços e cinética calibrada antes da implementação.</x:v>
+        <x:v>Selecionar e aprovar cinética LTFT e modelos de energia, queda de pressão, transporte, WGS e desativação; então validar balanços e saídas.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="52" customHeight="1">
@@ -4068,14 +4096,14 @@
       <x:c r="F63" s="33" t="str">
         <x:v>Avaliar EOS, regras de mistura, pseudocomponentes e VLE para syngas, água, hidrocarbonetos e ceras, com faixa de validade e comparação experimental.</x:v>
       </x:c>
-      <x:c r="G63" s="37" t="str">
-        <x:v>Planejado</x:v>
+      <x:c r="G63" s="57" t="str">
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="H63" s="33" t="str">
-        <x:v>Biblioteca e pacote de propriedades ainda não foram selecionados.</x:v>
+        <x:v>Contrato termodinâmico, schema e porta de validação implementados em thermodynamics.py; cobre EOS, mistura, pseudocomponentes, VLE, domínio, métricas e cinco grupos de fases.</x:v>
       </x:c>
       <x:c r="I63" s="33" t="str">
-        <x:v>Definir matriz de propriedades, fases e dados experimentais de referência.</x:v>
+        <x:v>Selecionar pacotes candidatos e compará-los com dados rastreáveis de syngas, água, hidrocarbonetos líquidos e ceras antes da integração.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="52" customHeight="1">
@@ -4212,7 +4240,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcab9aa2ab15d47e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ffeb8295a574977"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: concluir FT-014 e FT-015
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R6a5c878ea1324feb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rc6a0af3b9a994960"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rd3954467731c44c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rb543f19a0e8e4a14"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -515,12 +515,6 @@
     <x:t xml:space="preserve">Calcular entrada/saída de carbono, incluir CO2 e espécies não identificadas, aplicar tolerância versionada e emitir relatório.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Auditoria verifica fechamento de seletividades; ainda não calcula balanço material completo de carbono.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Definir tolerância e implementar módulo de balanço com casos sintéticos.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">FT-015</x:t>
   </x:si>
   <x:si>
@@ -533,12 +527,6 @@
     <x:t xml:space="preserve">Definir espécies/bases, calcular fechamentos H e O e propagar incerteza.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Não há módulo nem campos suficientes para balanços completos de H/O.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Aprovar contrato analítico e implementar após o balanço de carbono.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">FT-016</x:t>
   </x:si>
   <x:si>
@@ -1224,12 +1212,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Conectar produção e condicionamento de syngas, síntese FT e upgrading; fechar C/H/O e energia; distinguir O2 coproduzido na eletrólise de O2 consumido na gaseificação.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Depende de FT-014, FT-015, FT-058 e FT-059.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Definir a fronteira e o diagrama de correntes após concluir as dependências.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">FT-061</x:t>
@@ -2125,7 +2107,7 @@
       <x:c r="A5" s="15" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B5" s="16">
+      <x:c r="B5" s="16" t="n">
         <x:v>63</x:v>
       </x:c>
       <x:c r="C5" s="12"/>
@@ -2133,14 +2115,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E5" s="16" t="n">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="F5" s="12"/>
       <x:c r="G5" s="15" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="H5" s="17" t="n">
-        <x:v>0.4126984126984127</x:v>
+        <x:v>0.4444444444444444</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -2182,7 +2164,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B9" s="20" t="n">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C9" s="12"/>
       <x:c r="D9" s="12"/>
@@ -2196,7 +2178,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B10" s="20" t="n">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C10" s="12"/>
       <x:c r="D10" s="12"/>
@@ -2210,7 +2192,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B11" s="20" t="n">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C11" s="12"/>
       <x:c r="D11" s="12"/>
@@ -2400,7 +2382,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B26" s="21" t="str">
-        <x:v>tests/ — 94 testes e 15 subtestes; 9 schemas, 7 exemplos e 6 notebooks aprovados na verificação de FT-013 em 2026-10-13</x:v>
+        <x:v>tests/ — 99 testes e 15 subtestes; 10 schemas, 8 exemplos e 6 notebooks aprovados na verificação de FT-014/FT-015 em 2026-10-13</x:v>
       </x:c>
       <x:c r="C26" s="12"/>
       <x:c r="D26" s="12"/>
@@ -2428,7 +2410,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B28" s="27" t="str">
-        <x:v>Próximo: FT-014 e FT-015 — balanços de C/H/O, com tolerâncias, espécies e bases documentadas</x:v>
+        <x:v>Próximo: FT-017 — comparar ASF com medições aprovadas, alinhar bases e relatar resíduos e incerteza</x:v>
       </x:c>
       <x:c r="C28" s="12"/>
       <x:c r="D28" s="12"/>
@@ -3170,19 +3152,19 @@
       <x:c r="F26" s="6" t="s">
         <x:v>167</x:v>
       </x:c>
-      <x:c r="G26" s="10" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H26" s="6" t="s">
-        <x:v>168</x:v>
-      </x:c>
-      <x:c r="I26" s="6" t="s">
-        <x:v>169</x:v>
+      <x:c r="G26" s="10" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="H26" s="6" t="str">
+        <x:v>elemental_balance.py e contrato JSON v1 calculam C de entrada/saída, residual, fechamento, desvio e tolerância configurável; CLI e exemplo sintético auditável incluídos; suíte completa aprovada.</x:v>
+      </x:c>
+      <x:c r="I26" s="6" t="str">
+        <x:v>Substituir o exemplo sintético por correntes medidas, fontes aprovadas e tolerância definida pelo método analítico antes de interpretar dados experimentais.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="54" customHeight="1">
       <x:c r="A27" s="5" t="s">
-        <x:v>170</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B27" s="5" t="s">
         <x:v>147</x:v>
@@ -3191,27 +3173,27 @@
         <x:v>148</x:v>
       </x:c>
       <x:c r="D27" s="5" t="s">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="E27" s="5" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="F27" s="5" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="E27" s="5" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="F27" s="5" t="s">
-        <x:v>173</x:v>
-      </x:c>
-      <x:c r="G27" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H27" s="5" t="s">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="I27" s="5" t="s">
-        <x:v>175</x:v>
+      <x:c r="G27" s="9" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="H27" s="5" t="str">
+        <x:v>Balanços H/O usam espécies e bases explícitas, propagam incertezas independentes e bloqueiam avaliação total em base seca; documentação e testes positivos/negativos incluídos.</x:v>
+      </x:c>
+      <x:c r="I27" s="5" t="str">
+        <x:v>Registrar incertezas e correlações do método real; manter avaliação H/O em wet_total e obter revisão humana antes do uso experimental.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="54" customHeight="1">
       <x:c r="A28" s="6" t="s">
-        <x:v>176</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="B28" s="6" t="s">
         <x:v>147</x:v>
@@ -3220,27 +3202,27 @@
         <x:v>148</x:v>
       </x:c>
       <x:c r="D28" s="6" t="s">
-        <x:v>177</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="E28" s="6" t="s">
-        <x:v>178</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="F28" s="6" t="s">
-        <x:v>179</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="G28" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H28" s="6" t="s">
-        <x:v>180</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="I28" s="6" t="s">
-        <x:v>181</x:v>
+        <x:v>177</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="54" customHeight="1">
       <x:c r="A29" s="5" t="s">
-        <x:v>182</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B29" s="5" t="s">
         <x:v>147</x:v>
@@ -3249,27 +3231,27 @@
         <x:v>148</x:v>
       </x:c>
       <x:c r="D29" s="5" t="s">
-        <x:v>183</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="E29" s="5" t="s">
-        <x:v>184</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="F29" s="5" t="s">
-        <x:v>185</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="G29" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H29" s="5" t="s">
-        <x:v>186</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="I29" s="5" t="s">
-        <x:v>187</x:v>
+        <x:v>183</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="54" customHeight="1">
       <x:c r="A30" s="6" t="s">
-        <x:v>188</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="B30" s="6" t="s">
         <x:v>147</x:v>
@@ -3278,27 +3260,27 @@
         <x:v>148</x:v>
       </x:c>
       <x:c r="D30" s="6" t="s">
-        <x:v>189</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="E30" s="6" t="s">
-        <x:v>190</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="F30" s="6" t="s">
-        <x:v>191</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="G30" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H30" s="6" t="s">
-        <x:v>192</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="I30" s="6" t="s">
-        <x:v>193</x:v>
+        <x:v>189</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="54" customHeight="1">
       <x:c r="A31" s="5" t="s">
-        <x:v>194</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="B31" s="5" t="s">
         <x:v>147</x:v>
@@ -3307,27 +3289,27 @@
         <x:v>148</x:v>
       </x:c>
       <x:c r="D31" s="5" t="s">
-        <x:v>195</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="E31" s="5" t="s">
-        <x:v>196</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="F31" s="5" t="s">
-        <x:v>197</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="G31" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H31" s="5" t="s">
-        <x:v>198</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="I31" s="5" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="54" customHeight="1">
       <x:c r="A32" s="6" t="s">
-        <x:v>200</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="B32" s="6" t="s">
         <x:v>147</x:v>
@@ -3336,1037 +3318,1037 @@
         <x:v>148</x:v>
       </x:c>
       <x:c r="D32" s="6" t="s">
-        <x:v>201</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="E32" s="6" t="s">
-        <x:v>202</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="F32" s="6" t="s">
-        <x:v>203</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="G32" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H32" s="6" t="s">
-        <x:v>204</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="I32" s="6" t="s">
-        <x:v>205</x:v>
+        <x:v>201</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="54" customHeight="1">
       <x:c r="A33" s="5" t="s">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="B33" s="5" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="C33" s="5" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="D33" s="5" t="s">
+        <x:v>205</x:v>
+      </x:c>
+      <x:c r="E33" s="5" t="s">
         <x:v>206</x:v>
       </x:c>
-      <x:c r="B33" s="5" t="s">
+      <x:c r="F33" s="5" t="s">
         <x:v>207</x:v>
-      </x:c>
-      <x:c r="C33" s="5" t="s">
-        <x:v>208</x:v>
-      </x:c>
-      <x:c r="D33" s="5" t="s">
-        <x:v>209</x:v>
-      </x:c>
-      <x:c r="E33" s="5" t="s">
-        <x:v>210</x:v>
-      </x:c>
-      <x:c r="F33" s="5" t="s">
-        <x:v>211</x:v>
       </x:c>
       <x:c r="G33" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H33" s="5" t="s">
-        <x:v>212</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="I33" s="5" t="s">
-        <x:v>213</x:v>
+        <x:v>209</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="54" customHeight="1">
       <x:c r="A34" s="6" t="s">
-        <x:v>214</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="B34" s="6" t="s">
-        <x:v>207</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C34" s="6" t="s">
-        <x:v>208</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D34" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="E34" s="6" t="s">
-        <x:v>216</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="F34" s="6" t="s">
-        <x:v>217</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="G34" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H34" s="6" t="s">
-        <x:v>218</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="I34" s="6" t="s">
-        <x:v>219</x:v>
+        <x:v>215</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="54" customHeight="1">
       <x:c r="A35" s="5" t="s">
-        <x:v>220</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="B35" s="5" t="s">
-        <x:v>207</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C35" s="5" t="s">
-        <x:v>208</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D35" s="5" t="s">
-        <x:v>221</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="E35" s="5" t="s">
-        <x:v>222</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="F35" s="5" t="s">
-        <x:v>223</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="G35" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H35" s="5" t="s">
-        <x:v>224</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="I35" s="5" t="s">
-        <x:v>225</x:v>
+        <x:v>221</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="54" customHeight="1">
       <x:c r="A36" s="6" t="s">
-        <x:v>226</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="B36" s="6" t="s">
-        <x:v>207</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C36" s="6" t="s">
-        <x:v>208</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D36" s="6" t="s">
-        <x:v>227</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="E36" s="6" t="s">
-        <x:v>228</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="F36" s="6" t="s">
-        <x:v>229</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="G36" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H36" s="6" t="s">
-        <x:v>230</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="I36" s="6" t="s">
-        <x:v>231</x:v>
+        <x:v>227</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="54" customHeight="1">
       <x:c r="A37" s="5" t="s">
-        <x:v>232</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="B37" s="5" t="s">
-        <x:v>207</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C37" s="5" t="s">
-        <x:v>208</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D37" s="5" t="s">
-        <x:v>233</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="E37" s="5" t="s">
-        <x:v>234</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="F37" s="5" t="s">
-        <x:v>235</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="G37" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H37" s="5" t="s">
-        <x:v>236</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="I37" s="5" t="s">
-        <x:v>237</x:v>
+        <x:v>233</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="54" customHeight="1">
       <x:c r="A38" s="6" t="s">
-        <x:v>238</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="B38" s="6" t="s">
-        <x:v>207</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C38" s="6" t="s">
-        <x:v>208</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D38" s="6" t="s">
-        <x:v>239</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="E38" s="6" t="s">
-        <x:v>240</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="F38" s="6" t="s">
-        <x:v>241</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="G38" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H38" s="6" t="s">
-        <x:v>242</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="I38" s="6" t="s">
-        <x:v>243</x:v>
+        <x:v>239</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="54" customHeight="1">
       <x:c r="A39" s="5" t="s">
-        <x:v>244</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="B39" s="5" t="s">
-        <x:v>207</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C39" s="5" t="s">
-        <x:v>208</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D39" s="5" t="s">
-        <x:v>245</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="E39" s="5" t="s">
-        <x:v>246</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="F39" s="5" t="s">
-        <x:v>247</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="G39" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H39" s="5" t="s">
-        <x:v>248</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="I39" s="5" t="s">
-        <x:v>249</x:v>
+        <x:v>245</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="54" customHeight="1">
       <x:c r="A40" s="6" t="s">
+        <x:v>246</x:v>
+      </x:c>
+      <x:c r="B40" s="6" t="s">
+        <x:v>247</x:v>
+      </x:c>
+      <x:c r="C40" s="6" t="s">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="D40" s="6" t="s">
+        <x:v>249</x:v>
+      </x:c>
+      <x:c r="E40" s="6" t="s">
         <x:v>250</x:v>
       </x:c>
-      <x:c r="B40" s="6" t="s">
+      <x:c r="F40" s="6" t="s">
         <x:v>251</x:v>
-      </x:c>
-      <x:c r="C40" s="6" t="s">
-        <x:v>252</x:v>
-      </x:c>
-      <x:c r="D40" s="6" t="s">
-        <x:v>253</x:v>
-      </x:c>
-      <x:c r="E40" s="6" t="s">
-        <x:v>254</x:v>
-      </x:c>
-      <x:c r="F40" s="6" t="s">
-        <x:v>255</x:v>
       </x:c>
       <x:c r="G40" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H40" s="6" t="s">
-        <x:v>256</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="I40" s="6" t="s">
-        <x:v>257</x:v>
+        <x:v>253</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="54" customHeight="1">
       <x:c r="A41" s="5" t="s">
-        <x:v>258</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="B41" s="5" t="s">
-        <x:v>251</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="C41" s="5" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="D41" s="5" t="s">
-        <x:v>259</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="E41" s="5" t="s">
-        <x:v>260</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="F41" s="5" t="s">
-        <x:v>261</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="G41" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H41" s="5" t="s">
-        <x:v>262</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="I41" s="5" t="s">
-        <x:v>263</x:v>
+        <x:v>259</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="54" customHeight="1">
       <x:c r="A42" s="6" t="s">
-        <x:v>264</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="B42" s="6" t="s">
-        <x:v>251</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="C42" s="6" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="D42" s="6" t="s">
-        <x:v>265</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="E42" s="6" t="s">
-        <x:v>266</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="F42" s="6" t="s">
-        <x:v>267</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="G42" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H42" s="6" t="s">
-        <x:v>268</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="I42" s="6" t="s">
-        <x:v>269</x:v>
+        <x:v>265</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="54" customHeight="1">
       <x:c r="A43" s="5" t="s">
-        <x:v>270</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="B43" s="5" t="s">
-        <x:v>251</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="C43" s="5" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="D43" s="5" t="s">
-        <x:v>271</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="E43" s="5" t="s">
-        <x:v>272</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="F43" s="5" t="s">
-        <x:v>273</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="G43" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H43" s="5" t="s">
-        <x:v>274</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="I43" s="5" t="s">
-        <x:v>275</x:v>
+        <x:v>271</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="54" customHeight="1">
       <x:c r="A44" s="6" t="s">
-        <x:v>276</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="B44" s="6" t="s">
-        <x:v>251</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="C44" s="6" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="D44" s="6" t="s">
-        <x:v>277</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="E44" s="6" t="s">
-        <x:v>278</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="F44" s="6" t="s">
-        <x:v>279</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="G44" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H44" s="6" t="s">
-        <x:v>280</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="I44" s="6" t="s">
-        <x:v>281</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="54" customHeight="1">
       <x:c r="A45" s="5" t="s">
-        <x:v>282</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="B45" s="5" t="s">
-        <x:v>251</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="C45" s="5" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="D45" s="5" t="s">
-        <x:v>283</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="E45" s="5" t="s">
-        <x:v>284</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="F45" s="5" t="s">
-        <x:v>285</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="G45" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H45" s="5" t="s">
-        <x:v>286</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="I45" s="5" t="s">
-        <x:v>287</x:v>
+        <x:v>283</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="54" customHeight="1">
       <x:c r="A46" s="6" t="s">
-        <x:v>288</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="B46" s="6" t="s">
-        <x:v>251</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="C46" s="6" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="D46" s="6" t="s">
-        <x:v>289</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="E46" s="6" t="s">
-        <x:v>290</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="F46" s="6" t="s">
-        <x:v>291</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="G46" s="11" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H46" s="6" t="s">
-        <x:v>292</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="I46" s="6" t="s">
-        <x:v>293</x:v>
+        <x:v>289</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="54" customHeight="1">
       <x:c r="A47" s="5" t="s">
+        <x:v>290</x:v>
+      </x:c>
+      <x:c r="B47" s="5" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="C47" s="5" t="s">
+        <x:v>292</x:v>
+      </x:c>
+      <x:c r="D47" s="5" t="s">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="E47" s="5" t="s">
         <x:v>294</x:v>
       </x:c>
-      <x:c r="B47" s="5" t="s">
+      <x:c r="F47" s="5" t="s">
         <x:v>295</x:v>
-      </x:c>
-      <x:c r="C47" s="5" t="s">
-        <x:v>296</x:v>
-      </x:c>
-      <x:c r="D47" s="5" t="s">
-        <x:v>297</x:v>
-      </x:c>
-      <x:c r="E47" s="5" t="s">
-        <x:v>298</x:v>
-      </x:c>
-      <x:c r="F47" s="5" t="s">
-        <x:v>299</x:v>
       </x:c>
       <x:c r="G47" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H47" s="5" t="s">
-        <x:v>300</x:v>
+        <x:v>296</x:v>
       </x:c>
       <x:c r="I47" s="5" t="s">
-        <x:v>301</x:v>
+        <x:v>297</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="54" customHeight="1">
       <x:c r="A48" s="6" t="s">
-        <x:v>302</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="B48" s="6" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C48" s="6" t="s">
-        <x:v>296</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="D48" s="6" t="s">
-        <x:v>303</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="E48" s="6" t="s">
-        <x:v>304</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="F48" s="6" t="s">
-        <x:v>305</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="G48" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H48" s="6" t="s">
-        <x:v>306</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="I48" s="6" t="s">
-        <x:v>307</x:v>
+        <x:v>303</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="54" customHeight="1">
       <x:c r="A49" s="5" t="s">
-        <x:v>308</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="B49" s="5" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C49" s="5" t="s">
-        <x:v>296</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="D49" s="5" t="s">
-        <x:v>309</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="E49" s="5" t="s">
-        <x:v>310</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="F49" s="5" t="s">
-        <x:v>311</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="G49" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H49" s="5" t="s">
-        <x:v>312</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="I49" s="5" t="s">
-        <x:v>313</x:v>
+        <x:v>309</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="54" customHeight="1">
       <x:c r="A50" s="6" t="s">
-        <x:v>314</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="B50" s="6" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C50" s="6" t="s">
-        <x:v>296</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="D50" s="6" t="s">
-        <x:v>315</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="E50" s="6" t="s">
-        <x:v>316</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="F50" s="6" t="s">
-        <x:v>317</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="G50" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H50" s="6" t="s">
-        <x:v>318</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="I50" s="6" t="s">
-        <x:v>319</x:v>
+        <x:v>315</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="54" customHeight="1">
       <x:c r="A51" s="5" t="s">
-        <x:v>320</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="B51" s="5" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C51" s="5" t="s">
-        <x:v>296</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="D51" s="5" t="s">
-        <x:v>321</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="E51" s="5" t="s">
-        <x:v>322</x:v>
+        <x:v>318</x:v>
       </x:c>
       <x:c r="F51" s="5" t="s">
-        <x:v>323</x:v>
+        <x:v>319</x:v>
       </x:c>
       <x:c r="G51" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H51" s="5" t="s">
-        <x:v>324</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="I51" s="5" t="s">
-        <x:v>325</x:v>
+        <x:v>321</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="54" customHeight="1">
       <x:c r="A52" s="6" t="s">
-        <x:v>326</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="B52" s="6" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C52" s="6" t="s">
-        <x:v>296</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="D52" s="6" t="s">
-        <x:v>327</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="E52" s="6" t="s">
-        <x:v>328</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="F52" s="6" t="s">
-        <x:v>329</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="G52" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H52" s="6" t="s">
-        <x:v>330</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="I52" s="6" t="s">
-        <x:v>331</x:v>
+        <x:v>327</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="54" customHeight="1">
       <x:c r="A53" s="5" t="s">
+        <x:v>328</x:v>
+      </x:c>
+      <x:c r="B53" s="5" t="s">
+        <x:v>329</x:v>
+      </x:c>
+      <x:c r="C53" s="5" t="s">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="D53" s="5" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="E53" s="5" t="s">
         <x:v>332</x:v>
       </x:c>
-      <x:c r="B53" s="5" t="s">
+      <x:c r="F53" s="5" t="s">
         <x:v>333</x:v>
-      </x:c>
-      <x:c r="C53" s="5" t="s">
-        <x:v>334</x:v>
-      </x:c>
-      <x:c r="D53" s="5" t="s">
-        <x:v>335</x:v>
-      </x:c>
-      <x:c r="E53" s="5" t="s">
-        <x:v>336</x:v>
-      </x:c>
-      <x:c r="F53" s="5" t="s">
-        <x:v>337</x:v>
       </x:c>
       <x:c r="G53" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H53" s="5" t="s">
-        <x:v>338</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="I53" s="5" t="s">
-        <x:v>339</x:v>
+        <x:v>335</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="54" customHeight="1">
       <x:c r="A54" s="6" t="s">
-        <x:v>340</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="B54" s="6" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="C54" s="6" t="s">
-        <x:v>334</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="D54" s="6" t="s">
-        <x:v>341</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="E54" s="6" t="s">
-        <x:v>342</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="F54" s="6" t="s">
-        <x:v>343</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="G54" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H54" s="6" t="s">
-        <x:v>344</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="I54" s="6" t="s">
-        <x:v>345</x:v>
+        <x:v>341</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="54" customHeight="1">
       <x:c r="A55" s="5" t="s">
-        <x:v>346</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B55" s="5" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="C55" s="5" t="s">
-        <x:v>334</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="D55" s="5" t="s">
-        <x:v>347</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="E55" s="5" t="s">
-        <x:v>348</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="F55" s="5" t="s">
-        <x:v>349</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="G55" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H55" s="5" t="s">
-        <x:v>350</x:v>
+        <x:v>346</x:v>
       </x:c>
       <x:c r="I55" s="5" t="s">
-        <x:v>351</x:v>
+        <x:v>347</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="54" customHeight="1">
       <x:c r="A56" s="6" t="s">
-        <x:v>352</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="B56" s="6" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="C56" s="6" t="s">
-        <x:v>334</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="D56" s="6" t="s">
-        <x:v>353</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="E56" s="6" t="s">
-        <x:v>354</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="F56" s="6" t="s">
-        <x:v>355</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="G56" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H56" s="6" t="s">
-        <x:v>356</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="I56" s="6" t="s">
-        <x:v>357</x:v>
+        <x:v>353</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="54" customHeight="1">
       <x:c r="A57" s="5" t="s">
-        <x:v>358</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="B57" s="5" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="C57" s="5" t="s">
-        <x:v>334</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="D57" s="5" t="s">
-        <x:v>359</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="E57" s="5" t="s">
-        <x:v>360</x:v>
+        <x:v>356</x:v>
       </x:c>
       <x:c r="F57" s="5" t="s">
-        <x:v>361</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="G57" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H57" s="5" t="s">
-        <x:v>362</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="I57" s="5" t="s">
-        <x:v>363</x:v>
+        <x:v>359</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="54" customHeight="1">
       <x:c r="A58" s="6" t="s">
-        <x:v>364</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="B58" s="6" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="C58" s="6" t="s">
-        <x:v>334</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="D58" s="6" t="s">
-        <x:v>365</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="E58" s="6" t="s">
-        <x:v>366</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="F58" s="6" t="s">
-        <x:v>367</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="G58" s="9" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H58" s="6" t="s">
-        <x:v>368</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="I58" s="6" t="s">
-        <x:v>369</x:v>
+        <x:v>365</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="54" customHeight="1">
       <x:c r="A59" s="5" t="s">
-        <x:v>370</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="B59" s="5" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="C59" s="5" t="s">
-        <x:v>334</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="D59" s="5" t="s">
-        <x:v>371</x:v>
+        <x:v>367</x:v>
       </x:c>
       <x:c r="E59" s="5" t="s">
-        <x:v>372</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="F59" s="5" t="s">
-        <x:v>373</x:v>
+        <x:v>369</x:v>
       </x:c>
       <x:c r="G59" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H59" s="5" t="s">
-        <x:v>374</x:v>
+        <x:v>370</x:v>
       </x:c>
       <x:c r="I59" s="5" t="s">
-        <x:v>375</x:v>
+        <x:v>371</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="54" customHeight="1">
       <x:c r="A60" s="6" t="s">
-        <x:v>376</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="B60" s="6" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="C60" s="6" t="s">
-        <x:v>334</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="D60" s="6" t="s">
-        <x:v>377</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="E60" s="6" t="s">
-        <x:v>378</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="F60" s="6" t="s">
-        <x:v>379</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="G60" s="10" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H60" s="6" t="s">
-        <x:v>380</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="I60" s="6" t="s">
-        <x:v>381</x:v>
+        <x:v>377</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="52" customHeight="1">
       <x:c r="A61" s="24" t="s">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="B61" s="24" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="C61" s="24" t="s">
+        <x:v>379</x:v>
+      </x:c>
+      <x:c r="D61" s="24" t="s">
+        <x:v>380</x:v>
+      </x:c>
+      <x:c r="E61" s="24" t="s">
+        <x:v>381</x:v>
+      </x:c>
+      <x:c r="F61" s="24" t="s">
         <x:v>382</x:v>
-      </x:c>
-      <x:c r="B61" s="24" t="s">
-        <x:v>295</x:v>
-      </x:c>
-      <x:c r="C61" s="24" t="s">
-        <x:v>383</x:v>
-      </x:c>
-      <x:c r="D61" s="24" t="s">
-        <x:v>384</x:v>
-      </x:c>
-      <x:c r="E61" s="24" t="s">
-        <x:v>385</x:v>
-      </x:c>
-      <x:c r="F61" s="24" t="s">
-        <x:v>386</x:v>
       </x:c>
       <x:c r="G61" s="31" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="H61" s="24" t="s">
-        <x:v>387</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="I61" s="24" t="s">
-        <x:v>388</x:v>
+        <x:v>384</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="52" customHeight="1">
       <x:c r="A62" s="24" t="s">
-        <x:v>389</x:v>
+        <x:v>385</x:v>
       </x:c>
       <x:c r="B62" s="24" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C62" s="24" t="s">
-        <x:v>383</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D62" s="24" t="s">
-        <x:v>390</x:v>
+        <x:v>386</x:v>
       </x:c>
       <x:c r="E62" s="24" t="s">
-        <x:v>391</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="F62" s="24" t="s">
-        <x:v>392</x:v>
+        <x:v>388</x:v>
       </x:c>
       <x:c r="G62" s="32" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H62" s="24" t="s">
-        <x:v>393</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="I62" s="24" t="s">
-        <x:v>394</x:v>
+        <x:v>390</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="52" customHeight="1">
       <x:c r="A63" s="24" t="s">
-        <x:v>395</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="B63" s="24" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C63" s="24" t="s">
-        <x:v>383</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D63" s="24" t="s">
-        <x:v>396</x:v>
+        <x:v>392</x:v>
       </x:c>
       <x:c r="E63" s="24" t="s">
-        <x:v>397</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="F63" s="24" t="s">
-        <x:v>398</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="G63" s="32" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="H63" s="24" t="s">
-        <x:v>399</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="I63" s="24" t="s">
-        <x:v>400</x:v>
+        <x:v>396</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="52" customHeight="1">
       <x:c r="A64" s="24" t="s">
-        <x:v>401</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="B64" s="24" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C64" s="24" t="s">
-        <x:v>383</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D64" s="24" t="s">
-        <x:v>402</x:v>
+        <x:v>398</x:v>
       </x:c>
       <x:c r="E64" s="24" t="s">
-        <x:v>403</x:v>
+        <x:v>399</x:v>
       </x:c>
       <x:c r="F64" s="24" t="s">
-        <x:v>404</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="G64" s="26" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="H64" s="24" t="s">
-        <x:v>405</x:v>
-      </x:c>
-      <x:c r="I64" s="24" t="s">
-        <x:v>406</x:v>
+      <x:c r="H64" s="24" t="str">
+        <x:v>FT-014 e FT-015 concluídas. O balanço integrado permanece bloqueado enquanto FT-058 e FT-059 não tiverem modelos selecionados e validados.</x:v>
+      </x:c>
+      <x:c r="I64" s="24" t="str">
+        <x:v>Concluir e validar FT-058 e FT-059; depois definir a fronteira, o diagrama de correntes e o balanço energético integrado.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="52" customHeight="1">
       <x:c r="A65" s="24" t="s">
-        <x:v>407</x:v>
+        <x:v>401</x:v>
       </x:c>
       <x:c r="B65" s="24" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C65" s="24" t="s">
-        <x:v>408</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="D65" s="24" t="s">
-        <x:v>409</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="E65" s="24" t="s">
-        <x:v>410</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="F65" s="24" t="s">
-        <x:v>411</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="G65" s="25" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="H65" s="24" t="s">
-        <x:v>412</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="I65" s="24" t="s">
-        <x:v>413</x:v>
+        <x:v>407</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="52" customHeight="1">
       <x:c r="A66" s="24" t="s">
-        <x:v>414</x:v>
+        <x:v>408</x:v>
       </x:c>
       <x:c r="B66" s="24" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C66" s="24" t="s">
-        <x:v>408</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="D66" s="24" t="s">
-        <x:v>415</x:v>
+        <x:v>409</x:v>
       </x:c>
       <x:c r="E66" s="24" t="s">
-        <x:v>416</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="F66" s="24" t="s">
-        <x:v>417</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="G66" s="26" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H66" s="24" t="s">
-        <x:v>418</x:v>
+        <x:v>412</x:v>
       </x:c>
       <x:c r="I66" s="24" t="s">
-        <x:v>419</x:v>
+        <x:v>413</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="52" customHeight="1">
       <x:c r="A67" s="24" t="s">
-        <x:v>420</x:v>
+        <x:v>414</x:v>
       </x:c>
       <x:c r="B67" s="24" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C67" s="24" t="s">
-        <x:v>421</x:v>
+        <x:v>415</x:v>
       </x:c>
       <x:c r="D67" s="24" t="s">
-        <x:v>422</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="E67" s="24" t="s">
-        <x:v>423</x:v>
+        <x:v>417</x:v>
       </x:c>
       <x:c r="F67" s="24" t="s">
-        <x:v>424</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="G67" s="26" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H67" s="24" t="s">
-        <x:v>425</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="I67" s="24" t="s">
-        <x:v>426</x:v>
+        <x:v>420</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4387,7 +4369,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7948e93c883d4374"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bdde117320f47d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: planejar ASF avancada e transporte
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R5bb41b5940c54561"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rae533713b3ac474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rfded73320ccf4087"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R255673a71fd84c3e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1662,7 +1662,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="44">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1777,6 +1777,15 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="26" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="19" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="18" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2102,7 +2111,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
-        <x:v>63</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C5" s="12"/>
       <x:c r="D5" s="15" t="s">
@@ -2116,7 +2125,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H5" s="17" t="n">
-        <x:v>0.4444444444444444</x:v>
+        <x:v>0.417910447761194</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -2186,7 +2195,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B11" s="20" t="n">
-        <x:v>13</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C11" s="12"/>
       <x:c r="D11" s="12"/>
@@ -2200,7 +2209,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B12" s="20" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C12" s="12"/>
       <x:c r="D12" s="12"/>
@@ -2404,7 +2413,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B28" s="27" t="str">
-        <x:v>FT-017 em execução — infraestrutura concluída; próxima porta: aprovar e conectar uma distribuição experimental compatível</x:v>
+        <x:v>Ordem aprovada: FT-012A → FT-013A → FT-013B; FT-017A aguarda FT-012A e dados experimentais aprovados por FT-021</x:v>
       </x:c>
       <x:c r="C28" s="12"/>
       <x:c r="D28" s="12"/>
@@ -4345,6 +4354,122 @@
         <x:v>418</x:v>
       </x:c>
     </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="44" t="str">
+        <x:v>FT-012A</x:v>
+      </x:c>
+      <x:c r="B68" s="44" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C68" s="44" t="str">
+        <x:v>LTFT mínimo</x:v>
+      </x:c>
+      <x:c r="D68" s="44" t="str">
+        <x:v>ASF avançada</x:v>
+      </x:c>
+      <x:c r="E68" s="44" t="str">
+        <x:v>Representar desvios da ASF ideal sem impor interpretação mecanicista não demonstrada.</x:v>
+      </x:c>
+      <x:c r="F68" s="44" t="str">
+        <x:v>Contratar ASF simples, mistura de duas ASF e segmentação; separar correções C1/C2; preservar cauda analítica, normalização e proveniência.</x:v>
+      </x:c>
+      <x:c r="G68" s="45" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="H68" s="44" t="str">
+        <x:v>Planejamento aprovado em docs/PLANO_ASF_AVANCADA_TRANSPORTE.md; nenhuma implementação ou superioridade do modelo avançado foi validada.</x:v>
+      </x:c>
+      <x:c r="I68" s="44" t="str">
+        <x:v>Implementar contrato e testes de fechamento, independência de max_n, continuidade aplicável e identificabilidade.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="44" t="str">
+        <x:v>FT-013A</x:v>
+      </x:c>
+      <x:c r="B69" s="44" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C69" s="44" t="str">
+        <x:v>LTFT mínimo</x:v>
+      </x:c>
+      <x:c r="D69" s="44" t="str">
+        <x:v>Contrato experimental v2</x:v>
+      </x:c>
+      <x:c r="E69" s="44" t="str">
+        <x:v>Ampliar a reprodutibilidade e fornecer entradas para diagnósticos de transporte.</x:v>
+      </x:c>
+      <x:c r="F69" s="44" t="str">
+        <x:v>Adicionar diluente, razão e partículas; geometria/porosidade; ativação completa; detectores, faixas, calibração, limites e recuperação da fração pesada.</x:v>
+      </x:c>
+      <x:c r="G69" s="46" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="H69" s="44" t="str">
+        <x:v>Campos aprovados no planejamento; o contrato atual já cobre parte do caso, mas a migração v2 ainda não foi implementada.</x:v>
+      </x:c>
+      <x:c r="I69" s="44" t="str">
+        <x:v>Definir schema e migração sem defaults arbitrários; criar exemplos positivos/negativos e testes de compatibilidade.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="44" t="str">
+        <x:v>FT-013B</x:v>
+      </x:c>
+      <x:c r="B70" s="44" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C70" s="44" t="str">
+        <x:v>LTFT mínimo</x:v>
+      </x:c>
+      <x:c r="D70" s="44" t="str">
+        <x:v>Diagnóstico de transporte</x:v>
+      </x:c>
+      <x:c r="E70" s="44" t="str">
+        <x:v>Verificar se dados podem sustentar interpretação cinética sem limitações de transporte não avaliadas.</x:v>
+      </x:c>
+      <x:c r="F70" s="44" t="str">
+        <x:v>Calcular Weisz–Prater, Mears de massa e Mears térmico com entradas/unidades/fontes explícitas e estados passed, failed ou not_assessable_missing_inputs.</x:v>
+      </x:c>
+      <x:c r="G70" s="45" t="str">
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="H70" s="44" t="str">
+        <x:v>Escopo e estados aprovados; ainda não há módulo, contrato ou dados suficientes para cálculo no repositório.</x:v>
+      </x:c>
+      <x:c r="I70" s="44" t="str">
+        <x:v>Implementar após FT-013A; validar equações, unidades, limites e casos independentes sem converter ausência de dados em aprovação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="44" t="str">
+        <x:v>FT-017A</x:v>
+      </x:c>
+      <x:c r="B71" s="44" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C71" s="44" t="str">
+        <x:v>Validação LTFT</x:v>
+      </x:c>
+      <x:c r="D71" s="44" t="str">
+        <x:v>Ajuste e seleção do modelo ASF</x:v>
+      </x:c>
+      <x:c r="E71" s="44" t="str">
+        <x:v>Selecionar entre ASF simples e variantes avançadas usando dados aprovados e critérios reproduzíveis.</x:v>
+      </x:c>
+      <x:c r="F71" s="44" t="str">
+        <x:v>Ajustar modelos, estimar incerteza/covariância, comparar resíduos, MAE, RMSE, qui-quadrado e AIC/BIC e avaliar fora do ajuste quando possível.</x:v>
+      </x:c>
+      <x:c r="G71" s="45" t="str">
+        <x:v>Bloqueado</x:v>
+      </x:c>
+      <x:c r="H71" s="44" t="str">
+        <x:v>Planejamento aprovado; depende de FT-012A, da infraestrutura FT-017 e de ao menos uma distribuição experimental aprovada por FT-021.</x:v>
+      </x:c>
+      <x:c r="I71" s="44" t="str">
+        <x:v>Concluir FT-012A e aprovar dados em FT-021; depois definir protocolo de ajuste, conjunto de avaliação e revisão humana.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:I2"/>
@@ -4363,7 +4488,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b59ef89cfca4dd3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14e54cbe2a4447e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: concluir FT-012A e FT-013A
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rfded73320ccf4087"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R255673a71fd84c3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R460663465a574ca6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Raab74e6108914ffc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2118,14 +2118,14 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E5" s="16" t="n">
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F5" s="12"/>
       <x:c r="G5" s="15" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="H5" s="17" t="n">
-        <x:v>0.417910447761194</x:v>
+        <x:v>0.44776119402985076</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -2167,7 +2167,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B9" s="20" t="n">
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C9" s="12"/>
       <x:c r="D9" s="12"/>
@@ -2195,7 +2195,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B11" s="20" t="n">
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C11" s="12"/>
       <x:c r="D11" s="12"/>
@@ -2385,7 +2385,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B26" s="21" t="str">
-        <x:v>tests/ — 104 testes e 15 subtestes; 11 schemas, 9 exemplos e 6 notebooks aprovados no início da FT-017 em 2026-10-13</x:v>
+        <x:v>tests/ — 113 testes e 15 subtestes; 13 schemas, 12 exemplos e 6 notebooks aprovados na conclusão de FT-012A/FT-013A em 2026-10-13</x:v>
       </x:c>
       <x:c r="C26" s="12"/>
       <x:c r="D26" s="12"/>
@@ -2413,7 +2413,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B28" s="27" t="str">
-        <x:v>Ordem aprovada: FT-012A → FT-013A → FT-013B; FT-017A aguarda FT-012A e dados experimentais aprovados por FT-021</x:v>
+        <x:v>Próximo: FT-013B — diagnósticos Weisz–Prater e Mears; FT-017A permanece bloqueada até aprovação de dados em FT-021</x:v>
       </x:c>
       <x:c r="C28" s="12"/>
       <x:c r="D28" s="12"/>
@@ -4374,13 +4374,13 @@
         <x:v>Contratar ASF simples, mistura de duas ASF e segmentação; separar correções C1/C2; preservar cauda analítica, normalização e proveniência.</x:v>
       </x:c>
       <x:c r="G68" s="45" t="str">
-        <x:v>Planejado</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
       <x:c r="H68" s="44" t="str">
-        <x:v>Planejamento aprovado em docs/PLANO_ASF_AVANCADA_TRANSPORTE.md; nenhuma implementação ou superioridade do modelo avançado foi validada.</x:v>
+        <x:v>advanced_asf.py, schema e CLI implementam ASF simples, mistura de duas ASF e segmentação, correções C1/C2 separadas, normalização e cauda C∞. Testes cobrem equivalência, fechamento e independência de max_n.</x:v>
       </x:c>
       <x:c r="I68" s="44" t="str">
-        <x:v>Implementar contrato e testes de fechamento, independência de max_n, continuidade aplicável e identificabilidade.</x:v>
+        <x:v>Usar FT-017A somente após dados aprovados; comparar modelos sem presumir superioridade da ASF avançada.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -4403,13 +4403,13 @@
         <x:v>Adicionar diluente, razão e partículas; geometria/porosidade; ativação completa; detectores, faixas, calibração, limites e recuperação da fração pesada.</x:v>
       </x:c>
       <x:c r="G69" s="46" t="str">
-        <x:v>Planejado</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
       <x:c r="H69" s="44" t="str">
-        <x:v>Campos aprovados no planejamento; o contrato atual já cobre parte do caso, mas a migração v2 ainda não foi implementada.</x:v>
+        <x:v>experimental_protocol.py, schema v2, migração, template e exemplo sintético completo cobrem diluição, partículas, geometria, ativação, analytics e fontes por campo sem inventar valores ausentes.</x:v>
       </x:c>
       <x:c r="I69" s="44" t="str">
-        <x:v>Definir schema e migração sem defaults arbitrários; criar exemplos positivos/negativos e testes de compatibilidade.</x:v>
+        <x:v>Usar o contrato como entrada da FT-013B; substituir exemplos sintéticos pelo protocolo real e manter revisão humana antes da execução.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -4435,10 +4435,10 @@
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="H70" s="44" t="str">
-        <x:v>Escopo e estados aprovados; ainda não há módulo, contrato ou dados suficientes para cálculo no repositório.</x:v>
+        <x:v>FT-013A concluída e fornece os campos estruturais necessários; ainda não existem equações, limites e cálculo versionado de Weisz–Prater/Mears.</x:v>
       </x:c>
       <x:c r="I70" s="44" t="str">
-        <x:v>Implementar após FT-013A; validar equações, unidades, limites e casos independentes sem converter ausência de dados em aprovação.</x:v>
+        <x:v>Implementar módulo e contrato de transporte com unidades, fontes, limites, casos independentes e estado not_assessable_missing_inputs.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -4464,10 +4464,10 @@
         <x:v>Bloqueado</x:v>
       </x:c>
       <x:c r="H71" s="44" t="str">
-        <x:v>Planejamento aprovado; depende de FT-012A, da infraestrutura FT-017 e de ao menos uma distribuição experimental aprovada por FT-021.</x:v>
+        <x:v>FT-012A concluída e infraestrutura FT-017 disponível; ajuste e seleção continuam bloqueados até haver distribuição experimental aprovada por FT-021.</x:v>
       </x:c>
       <x:c r="I71" s="44" t="str">
-        <x:v>Concluir FT-012A e aprovar dados em FT-021; depois definir protocolo de ajuste, conjunto de avaliação e revisão humana.</x:v>
+        <x:v>Aprovar dados em FT-021; então definir protocolo de ajuste, conjunto de avaliação, critérios AIC/BIC e revisão humana.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4488,7 +4488,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14e54cbe2a4447e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab84628b92ce4c32"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: concluir FT-019 e FT-020
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rb7246968a6f941f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R558907cfaba649ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rb5ef86c88fec4c12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R4e027cf4335f46d0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,9 +14,6 @@
     <x:t xml:space="preserve">Atividades da Plataforma Reação Fischer–Tropsch</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Situação verificada no repositório principal em 2026-10-13</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Total de atividades</x:t>
   </x:si>
   <x:si>
@@ -587,12 +584,6 @@
     <x:t xml:space="preserve">Exportar entrada, resultado e tabelas em formatos versionados, com metadados e hashes.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Worker exporta JSON reproduzível; não há exportação CSV completa pela interface.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Implementar exportação CSV e pacote de execução com manifesto.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">FT-020</x:t>
   </x:si>
   <x:si>
@@ -603,12 +594,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Gerar relatório legível e auditável com versão, entradas, método, bloqueios e referências.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Resultado JSON e notebook existem; não há relatório científico final formatado.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Definir template e gerar relatório a partir do contrato de resultado.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">FT-021</x:t>
@@ -2085,8 +2070,8 @@
       <x:c r="H2" s="13"/>
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
-      <x:c r="A3" s="14" t="s">
-        <x:v>1</x:v>
+      <x:c r="A3" s="14" t="str">
+        <x:v>Situação verificada no repositório principal em 2026-10-14</x:v>
       </x:c>
       <x:c r="B3" s="14"/>
       <x:c r="C3" s="14"/>
@@ -2108,24 +2093,24 @@
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="15" t="s">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>67</x:v>
       </x:c>
       <x:c r="C5" s="12"/>
       <x:c r="D5" s="15" t="s">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E5" s="16" t="n">
-        <x:v>31</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="F5" s="12"/>
       <x:c r="G5" s="15" t="s">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H5" s="17" t="n">
-        <x:v>0.4626865671641791</x:v>
+        <x:v>0.4925373134328358</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -2150,10 +2135,10 @@
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="18" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="18" t="s">
         <x:v>5</x:v>
-      </x:c>
-      <x:c r="B8" s="18" t="s">
-        <x:v>6</x:v>
       </x:c>
       <x:c r="C8" s="12"/>
       <x:c r="D8" s="12"/>
@@ -2164,10 +2149,10 @@
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
       <x:c r="A9" s="19" t="s">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B9" s="20" t="n">
-        <x:v>31</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C9" s="12"/>
       <x:c r="D9" s="12"/>
@@ -2178,10 +2163,10 @@
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
       <x:c r="A10" s="19" t="s">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B10" s="20" t="n">
-        <x:v>14</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C10" s="12"/>
       <x:c r="D10" s="12"/>
@@ -2192,7 +2177,7 @@
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
       <x:c r="A11" s="19" t="s">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B11" s="20" t="n">
         <x:v>13</x:v>
@@ -2206,7 +2191,7 @@
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
       <x:c r="A12" s="19" t="s">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B12" s="20" t="n">
         <x:v>9</x:v>
@@ -2240,7 +2225,7 @@
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
       <x:c r="A15" s="33" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B15" s="33"/>
       <x:c r="C15" s="12"/>
@@ -2252,10 +2237,10 @@
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
       <x:c r="A16" s="21" t="s">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B16" s="21" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C16" s="12"/>
       <x:c r="D16" s="12"/>
@@ -2266,10 +2251,10 @@
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
       <x:c r="A17" s="21" t="s">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B17" s="21" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C17" s="12"/>
       <x:c r="D17" s="12"/>
@@ -2280,10 +2265,10 @@
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
       <x:c r="A18" s="21" t="s">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B18" s="21" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C18" s="12"/>
       <x:c r="D18" s="12"/>
@@ -2294,10 +2279,10 @@
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
       <x:c r="A19" s="21" t="s">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B19" s="21" t="s">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C19" s="12"/>
       <x:c r="D19" s="12"/>
@@ -2328,7 +2313,7 @@
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
       <x:c r="A22" s="34" t="s">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B22" s="34"/>
       <x:c r="C22" s="12"/>
@@ -2340,10 +2325,10 @@
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
       <x:c r="A23" s="21" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B23" s="21" t="s">
         <x:v>17</x:v>
-      </x:c>
-      <x:c r="B23" s="21" t="s">
-        <x:v>18</x:v>
       </x:c>
       <x:c r="C23" s="12"/>
       <x:c r="D23" s="12"/>
@@ -2354,10 +2339,10 @@
     </x:row>
     <x:row r="24" ht="28" customHeight="1">
       <x:c r="A24" s="21" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B24" s="21" t="s">
         <x:v>19</x:v>
-      </x:c>
-      <x:c r="B24" s="21" t="s">
-        <x:v>20</x:v>
       </x:c>
       <x:c r="C24" s="12"/>
       <x:c r="D24" s="12"/>
@@ -2368,10 +2353,10 @@
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
       <x:c r="A25" s="21" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B25" s="21" t="s">
         <x:v>21</x:v>
-      </x:c>
-      <x:c r="B25" s="21" t="s">
-        <x:v>22</x:v>
       </x:c>
       <x:c r="C25" s="12"/>
       <x:c r="D25" s="12"/>
@@ -2382,10 +2367,10 @@
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
       <x:c r="A26" s="21" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B26" s="21" t="str">
-        <x:v>tests/ — 118 testes e 15 subtestes; 14 schemas, 13 exemplos e 6 notebooks aprovados na conclusão de FT-013B em 2026-10-13</x:v>
+        <x:v>tests/ — 123 testes e 15 subtestes; 15 schemas, 14 exemplos e 6 notebooks aprovados na conclusão de FT-019/FT-020 em 2026-10-14</x:v>
       </x:c>
       <x:c r="C26" s="12"/>
       <x:c r="D26" s="12"/>
@@ -2396,7 +2381,7 @@
     </x:row>
     <x:row r="27" ht="28" customHeight="1">
       <x:c r="A27" s="21" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B27" s="21" t="str">
         <x:v>GitHub Actions obrigatório em push para main e pull request; deploy público Streamlit verificado separadamente</x:v>
@@ -2410,10 +2395,10 @@
     </x:row>
     <x:row r="28" ht="20" customHeight="1">
       <x:c r="A28" s="27" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B28" s="27" t="str">
-        <x:v>Próximo: obter dados aprovados em FT-021 para liberar FT-017A; diagnóstico FT-013B permanece sujeito a entradas reais e revisão humana</x:v>
+        <x:v>Próximo: qualificar e aprovar dados em FT-021; FT-017/FT-017A permanecem limitadas enquanto não houver distribuição experimental aprovada</x:v>
       </x:c>
       <x:c r="C28" s="12"/>
       <x:c r="D28" s="12"/>
@@ -2424,7 +2409,7 @@
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="35" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B29" s="36"/>
       <x:c r="C29" s="36"/>
@@ -2474,7 +2459,7 @@
   <x:sheetData>
     <x:row r="2" ht="18">
       <x:c r="A2" s="38" t="s">
-        <x:v>27</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B2" s="38"/>
       <x:c r="C2" s="38"/>
@@ -2487,7 +2472,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="39" t="s">
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B3" s="39"/>
       <x:c r="C3" s="39"/>
@@ -2500,544 +2485,544 @@
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="4" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B4" s="4" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B4" s="4" t="s">
+      <x:c r="C4" s="4" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="C4" s="4" t="s">
+      <x:c r="D4" s="4" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="D4" s="4" t="s">
+      <x:c r="E4" s="4" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="E4" s="4" t="s">
+      <x:c r="F4" s="4" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="F4" s="4" t="s">
+      <x:c r="G4" s="4" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H4" s="4" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="G4" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="H4" s="4" t="s">
+      <x:c r="I4" s="4" t="s">
         <x:v>35</x:v>
-      </x:c>
-      <x:c r="I4" s="4" t="s">
-        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="54" customHeight="1">
       <x:c r="A5" s="5" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B5" s="5" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="s">
+      <x:c r="C5" s="5" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="C5" s="5" t="s">
+      <x:c r="D5" s="5" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="D5" s="5" t="s">
+      <x:c r="E5" s="5" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="E5" s="5" t="s">
+      <x:c r="F5" s="5" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="F5" s="5" t="s">
+      <x:c r="G5" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H5" s="5" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="G5" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H5" s="5" t="s">
+      <x:c r="I5" s="5" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="I5" s="5" t="s">
-        <x:v>44</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
       <x:c r="A6" s="6" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="B6" s="6" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C6" s="6" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D6" s="6" t="s">
+      <x:c r="E6" s="6" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="E6" s="6" t="s">
+      <x:c r="F6" s="6" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="F6" s="6" t="s">
+      <x:c r="G6" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="G6" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H6" s="6" t="s">
+      <x:c r="I6" s="6" t="s">
         <x:v>49</x:v>
-      </x:c>
-      <x:c r="I6" s="6" t="s">
-        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
       <x:c r="A7" s="5" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C7" s="5" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D7" s="5" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C7" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D7" s="5" t="s">
+      <x:c r="E7" s="5" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="E7" s="5" t="s">
+      <x:c r="F7" s="5" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="F7" s="5" t="s">
+      <x:c r="G7" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H7" s="5" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="G7" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H7" s="5" t="s">
+      <x:c r="I7" s="5" t="s">
         <x:v>55</x:v>
-      </x:c>
-      <x:c r="I7" s="5" t="s">
-        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
       <x:c r="A8" s="6" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="B8" s="6" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C8" s="6" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D8" s="6" t="s">
+      <x:c r="E8" s="6" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="E8" s="6" t="s">
+      <x:c r="F8" s="6" t="s">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="F8" s="6" t="s">
+      <x:c r="G8" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="s">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="G8" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H8" s="6" t="s">
+      <x:c r="I8" s="6" t="s">
         <x:v>61</x:v>
-      </x:c>
-      <x:c r="I8" s="6" t="s">
-        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
       <x:c r="A9" s="5" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B9" s="5" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C9" s="5" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D9" s="5" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C9" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="s">
+      <x:c r="E9" s="5" t="s">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="E9" s="5" t="s">
+      <x:c r="F9" s="5" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="F9" s="5" t="s">
+      <x:c r="G9" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H9" s="5" t="s">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="G9" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H9" s="5" t="s">
+      <x:c r="I9" s="5" t="s">
         <x:v>67</x:v>
-      </x:c>
-      <x:c r="I9" s="5" t="s">
-        <x:v>68</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
       <x:c r="A10" s="6" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="B10" s="6" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C10" s="6" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D10" s="6" t="s">
+      <x:c r="E10" s="6" t="s">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="E10" s="6" t="s">
+      <x:c r="F10" s="6" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="F10" s="6" t="s">
+      <x:c r="G10" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H10" s="6" t="s">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="G10" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H10" s="6" t="s">
+      <x:c r="I10" s="6" t="s">
         <x:v>73</x:v>
-      </x:c>
-      <x:c r="I10" s="6" t="s">
-        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
       <x:c r="A11" s="5" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="B11" s="5" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C11" s="5" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D11" s="5" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="B11" s="5" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C11" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D11" s="5" t="s">
+      <x:c r="E11" s="5" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="E11" s="5" t="s">
+      <x:c r="F11" s="5" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="F11" s="5" t="s">
+      <x:c r="G11" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H11" s="5" t="s">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="G11" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H11" s="5" t="s">
+      <x:c r="I11" s="5" t="s">
         <x:v>79</x:v>
-      </x:c>
-      <x:c r="I11" s="5" t="s">
-        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
       <x:c r="A12" s="6" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="s">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="B12" s="6" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C12" s="6" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D12" s="6" t="s">
+      <x:c r="E12" s="6" t="s">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="E12" s="6" t="s">
+      <x:c r="F12" s="6" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="F12" s="6" t="s">
+      <x:c r="G12" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H12" s="6" t="s">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="G12" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H12" s="6" t="s">
+      <x:c r="I12" s="6" t="s">
         <x:v>85</x:v>
-      </x:c>
-      <x:c r="I12" s="6" t="s">
-        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
       <x:c r="A13" s="5" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="B13" s="5" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C13" s="5" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D13" s="5" t="s">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="B13" s="5" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C13" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D13" s="5" t="s">
+      <x:c r="E13" s="5" t="s">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="E13" s="5" t="s">
+      <x:c r="F13" s="5" t="s">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="F13" s="5" t="s">
+      <x:c r="G13" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H13" s="5" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="G13" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H13" s="5" t="s">
+      <x:c r="I13" s="5" t="s">
         <x:v>91</x:v>
-      </x:c>
-      <x:c r="I13" s="5" t="s">
-        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="54" customHeight="1">
       <x:c r="A14" s="7" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="B14" s="7" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C14" s="7" t="s">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="B14" s="7" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C14" s="7" t="s">
+      <x:c r="D14" s="7" t="s">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="D14" s="7" t="s">
+      <x:c r="E14" s="7" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="E14" s="7" t="s">
+      <x:c r="F14" s="7" t="s">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="F14" s="7" t="s">
+      <x:c r="G14" s="23" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H14" s="7" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="G14" s="23" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H14" s="7" t="s">
+      <x:c r="I14" s="7" t="s">
         <x:v>98</x:v>
-      </x:c>
-      <x:c r="I14" s="7" t="s">
-        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
       <x:c r="A15" s="7" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C15" s="7" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="D15" s="7" t="s">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="B15" s="7" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="D15" s="7" t="s">
+      <x:c r="E15" s="7" t="s">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="E15" s="7" t="s">
+      <x:c r="F15" s="7" t="s">
         <x:v>102</x:v>
       </x:c>
-      <x:c r="F15" s="7" t="s">
+      <x:c r="G15" s="23" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H15" s="7" t="s">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="G15" s="23" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H15" s="7" t="s">
+      <x:c r="I15" s="7" t="s">
         <x:v>104</x:v>
-      </x:c>
-      <x:c r="I15" s="7" t="s">
-        <x:v>105</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
       <x:c r="A16" s="7" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="B16" s="7" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C16" s="7" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="D16" s="7" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="B16" s="7" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C16" s="7" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="D16" s="7" t="s">
+      <x:c r="E16" s="7" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="E16" s="7" t="s">
+      <x:c r="F16" s="7" t="s">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="F16" s="7" t="s">
+      <x:c r="G16" s="28" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H16" s="7" t="s">
         <x:v>109</x:v>
       </x:c>
-      <x:c r="G16" s="28" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H16" s="7" t="s">
+      <x:c r="I16" s="7" t="s">
         <x:v>110</x:v>
-      </x:c>
-      <x:c r="I16" s="7" t="s">
-        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
       <x:c r="A17" s="7" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="B17" s="7" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C17" s="7" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="D17" s="7" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="B17" s="7" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C17" s="7" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="D17" s="7" t="s">
+      <x:c r="E17" s="7" t="s">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="E17" s="7" t="s">
+      <x:c r="F17" s="7" t="s">
         <x:v>114</x:v>
       </x:c>
-      <x:c r="F17" s="7" t="s">
+      <x:c r="G17" s="28" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H17" s="7" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="G17" s="28" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H17" s="7" t="s">
+      <x:c r="I17" s="7" t="s">
         <x:v>116</x:v>
-      </x:c>
-      <x:c r="I17" s="7" t="s">
-        <x:v>117</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
       <x:c r="A18" s="7" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="B18" s="7" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C18" s="7" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="D18" s="7" t="s">
         <x:v>118</x:v>
       </x:c>
-      <x:c r="B18" s="7" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C18" s="7" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="D18" s="7" t="s">
+      <x:c r="E18" s="7" t="s">
         <x:v>119</x:v>
       </x:c>
-      <x:c r="E18" s="7" t="s">
+      <x:c r="F18" s="7" t="s">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="F18" s="7" t="s">
+      <x:c r="G18" s="29" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H18" s="7" t="s">
         <x:v>121</x:v>
       </x:c>
-      <x:c r="G18" s="29" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H18" s="7" t="s">
+      <x:c r="I18" s="7" t="s">
         <x:v>122</x:v>
-      </x:c>
-      <x:c r="I18" s="7" t="s">
-        <x:v>123</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
       <x:c r="A19" s="7" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C19" s="7" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="D19" s="7" t="s">
         <x:v>124</x:v>
       </x:c>
-      <x:c r="B19" s="7" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="D19" s="7" t="s">
+      <x:c r="E19" s="7" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="E19" s="7" t="s">
+      <x:c r="F19" s="7" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="F19" s="7" t="s">
+      <x:c r="G19" s="30" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H19" s="7" t="s">
         <x:v>127</x:v>
       </x:c>
-      <x:c r="G19" s="30" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H19" s="7" t="s">
+      <x:c r="I19" s="7" t="s">
         <x:v>128</x:v>
-      </x:c>
-      <x:c r="I19" s="7" t="s">
-        <x:v>129</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
       <x:c r="A20" s="7" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C20" s="7" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="D20" s="7" t="s">
         <x:v>130</x:v>
       </x:c>
-      <x:c r="B20" s="7" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="D20" s="7" t="s">
+      <x:c r="E20" s="7" t="s">
         <x:v>131</x:v>
       </x:c>
-      <x:c r="E20" s="7" t="s">
+      <x:c r="F20" s="7" t="s">
         <x:v>132</x:v>
       </x:c>
-      <x:c r="F20" s="7" t="s">
+      <x:c r="G20" s="30" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H20" s="7" t="s">
         <x:v>133</x:v>
       </x:c>
-      <x:c r="G20" s="30" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H20" s="7" t="s">
+      <x:c r="I20" s="7" t="s">
         <x:v>134</x:v>
-      </x:c>
-      <x:c r="I20" s="7" t="s">
-        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
       <x:c r="A21" s="7" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C21" s="7" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="D21" s="7" t="s">
         <x:v>136</x:v>
       </x:c>
-      <x:c r="B21" s="7" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C21" s="7" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="D21" s="7" t="s">
+      <x:c r="E21" s="7" t="s">
         <x:v>137</x:v>
       </x:c>
-      <x:c r="E21" s="7" t="s">
+      <x:c r="F21" s="7" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="F21" s="7" t="s">
+      <x:c r="G21" s="30" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H21" s="7" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="G21" s="30" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H21" s="7" t="s">
+      <x:c r="I21" s="7" t="s">
         <x:v>140</x:v>
-      </x:c>
-      <x:c r="I21" s="7" t="s">
-        <x:v>141</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="54" customHeight="1">
       <x:c r="A22" s="6" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="B22" s="6" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C22" s="6" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D22" s="6" t="s">
         <x:v>142</x:v>
       </x:c>
-      <x:c r="B22" s="6" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C22" s="6" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D22" s="6" t="s">
+      <x:c r="E22" s="6" t="s">
         <x:v>143</x:v>
       </x:c>
-      <x:c r="E22" s="6" t="s">
+      <x:c r="F22" s="6" t="s">
         <x:v>144</x:v>
-      </x:c>
-      <x:c r="F22" s="6" t="s">
-        <x:v>145</x:v>
       </x:c>
       <x:c r="G22" s="41" t="str">
         <x:v>Concluído</x:v>
@@ -3051,80 +3036,80 @@
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
       <x:c r="A23" s="5" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="B23" s="5" t="s">
         <x:v>146</x:v>
       </x:c>
-      <x:c r="B23" s="5" t="s">
+      <x:c r="C23" s="5" t="s">
         <x:v>147</x:v>
       </x:c>
-      <x:c r="C23" s="5" t="s">
+      <x:c r="D23" s="5" t="s">
         <x:v>148</x:v>
       </x:c>
-      <x:c r="D23" s="5" t="s">
+      <x:c r="E23" s="5" t="s">
         <x:v>149</x:v>
       </x:c>
-      <x:c r="E23" s="5" t="s">
+      <x:c r="F23" s="5" t="s">
         <x:v>150</x:v>
       </x:c>
-      <x:c r="F23" s="5" t="s">
+      <x:c r="G23" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H23" s="5" t="s">
         <x:v>151</x:v>
       </x:c>
-      <x:c r="G23" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H23" s="5" t="s">
+      <x:c r="I23" s="5" t="s">
         <x:v>152</x:v>
-      </x:c>
-      <x:c r="I23" s="5" t="s">
-        <x:v>153</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
       <x:c r="A24" s="6" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="B24" s="6" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="C24" s="6" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="D24" s="6" t="s">
         <x:v>154</x:v>
       </x:c>
-      <x:c r="B24" s="6" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C24" s="6" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="D24" s="6" t="s">
+      <x:c r="E24" s="6" t="s">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="E24" s="6" t="s">
+      <x:c r="F24" s="6" t="s">
         <x:v>156</x:v>
       </x:c>
-      <x:c r="F24" s="6" t="s">
+      <x:c r="G24" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H24" s="6" t="s">
         <x:v>157</x:v>
       </x:c>
-      <x:c r="G24" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H24" s="6" t="s">
+      <x:c r="I24" s="6" t="s">
         <x:v>158</x:v>
-      </x:c>
-      <x:c r="I24" s="6" t="s">
-        <x:v>159</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="54" customHeight="1">
       <x:c r="A25" s="5" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="B25" s="5" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="C25" s="5" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="D25" s="5" t="s">
         <x:v>160</x:v>
       </x:c>
-      <x:c r="B25" s="5" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C25" s="5" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="D25" s="5" t="s">
+      <x:c r="E25" s="5" t="s">
         <x:v>161</x:v>
       </x:c>
-      <x:c r="E25" s="5" t="s">
+      <x:c r="F25" s="5" t="s">
         <x:v>162</x:v>
-      </x:c>
-      <x:c r="F25" s="5" t="s">
-        <x:v>163</x:v>
       </x:c>
       <x:c r="G25" s="43" t="str">
         <x:v>Concluído</x:v>
@@ -3138,22 +3123,22 @@
     </x:row>
     <x:row r="26" ht="54" customHeight="1">
       <x:c r="A26" s="6" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="B26" s="6" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="C26" s="6" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="D26" s="6" t="s">
         <x:v>164</x:v>
       </x:c>
-      <x:c r="B26" s="6" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C26" s="6" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="D26" s="6" t="s">
+      <x:c r="E26" s="6" t="s">
         <x:v>165</x:v>
       </x:c>
-      <x:c r="E26" s="6" t="s">
+      <x:c r="F26" s="6" t="s">
         <x:v>166</x:v>
-      </x:c>
-      <x:c r="F26" s="6" t="s">
-        <x:v>167</x:v>
       </x:c>
       <x:c r="G26" s="10" t="str">
         <x:v>Concluído</x:v>
@@ -3167,22 +3152,22 @@
     </x:row>
     <x:row r="27" ht="54" customHeight="1">
       <x:c r="A27" s="5" t="s">
+        <x:v>167</x:v>
+      </x:c>
+      <x:c r="B27" s="5" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="C27" s="5" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="D27" s="5" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="B27" s="5" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C27" s="5" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="D27" s="5" t="s">
+      <x:c r="E27" s="5" t="s">
         <x:v>169</x:v>
       </x:c>
-      <x:c r="E27" s="5" t="s">
+      <x:c r="F27" s="5" t="s">
         <x:v>170</x:v>
-      </x:c>
-      <x:c r="F27" s="5" t="s">
-        <x:v>171</x:v>
       </x:c>
       <x:c r="G27" s="9" t="str">
         <x:v>Concluído</x:v>
@@ -3196,51 +3181,51 @@
     </x:row>
     <x:row r="28" ht="54" customHeight="1">
       <x:c r="A28" s="6" t="s">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="B28" s="6" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="C28" s="6" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="D28" s="6" t="s">
         <x:v>172</x:v>
       </x:c>
-      <x:c r="B28" s="6" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C28" s="6" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="D28" s="6" t="s">
+      <x:c r="E28" s="6" t="s">
         <x:v>173</x:v>
       </x:c>
-      <x:c r="E28" s="6" t="s">
+      <x:c r="F28" s="6" t="s">
         <x:v>174</x:v>
       </x:c>
-      <x:c r="F28" s="6" t="s">
+      <x:c r="G28" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H28" s="6" t="s">
         <x:v>175</x:v>
       </x:c>
-      <x:c r="G28" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H28" s="6" t="s">
+      <x:c r="I28" s="6" t="s">
         <x:v>176</x:v>
-      </x:c>
-      <x:c r="I28" s="6" t="s">
-        <x:v>177</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="54" customHeight="1">
       <x:c r="A29" s="5" t="s">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="B29" s="5" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="C29" s="5" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="D29" s="5" t="s">
         <x:v>178</x:v>
       </x:c>
-      <x:c r="B29" s="5" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C29" s="5" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="D29" s="5" t="s">
+      <x:c r="E29" s="5" t="s">
         <x:v>179</x:v>
       </x:c>
-      <x:c r="E29" s="5" t="s">
+      <x:c r="F29" s="5" t="s">
         <x:v>180</x:v>
-      </x:c>
-      <x:c r="F29" s="5" t="s">
-        <x:v>181</x:v>
       </x:c>
       <x:c r="G29" s="9" t="str">
         <x:v>Parcial</x:v>
@@ -3254,1011 +3239,1011 @@
     </x:row>
     <x:row r="30" ht="54" customHeight="1">
       <x:c r="A30" s="6" t="s">
+        <x:v>181</x:v>
+      </x:c>
+      <x:c r="B30" s="6" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="C30" s="6" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="D30" s="6" t="s">
         <x:v>182</x:v>
       </x:c>
-      <x:c r="B30" s="6" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C30" s="6" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="D30" s="6" t="s">
+      <x:c r="E30" s="6" t="s">
         <x:v>183</x:v>
       </x:c>
-      <x:c r="E30" s="6" t="s">
+      <x:c r="F30" s="6" t="s">
         <x:v>184</x:v>
       </x:c>
-      <x:c r="F30" s="6" t="s">
+      <x:c r="G30" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H30" s="6" t="s">
         <x:v>185</x:v>
       </x:c>
-      <x:c r="G30" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H30" s="6" t="s">
+      <x:c r="I30" s="6" t="s">
         <x:v>186</x:v>
-      </x:c>
-      <x:c r="I30" s="6" t="s">
-        <x:v>187</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="54" customHeight="1">
       <x:c r="A31" s="5" t="s">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="B31" s="5" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="C31" s="5" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="D31" s="5" t="s">
         <x:v>188</x:v>
       </x:c>
-      <x:c r="B31" s="5" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C31" s="5" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="D31" s="5" t="s">
+      <x:c r="E31" s="5" t="s">
         <x:v>189</x:v>
       </x:c>
-      <x:c r="E31" s="5" t="s">
+      <x:c r="F31" s="5" t="s">
         <x:v>190</x:v>
       </x:c>
-      <x:c r="F31" s="5" t="s">
-        <x:v>191</x:v>
-      </x:c>
-      <x:c r="G31" s="10" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H31" s="5" t="s">
-        <x:v>192</x:v>
-      </x:c>
-      <x:c r="I31" s="5" t="s">
-        <x:v>193</x:v>
+      <x:c r="G31" s="10" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="H31" s="5" t="str">
+        <x:v>reporting.py gera JSON canônico, resumo CSV, faixas ASF CSV e manifesto com SHA-256, tipo e tamanho. A interface oferece os downloads e os testes confirmam determinismo, integridade, round-trip e leitura dos CSVs.</x:v>
+      </x:c>
+      <x:c r="I31" s="5" t="str">
+        <x:v>Aplicar os artefatos a novos módulos mantendo o contrato versionado; qualquer alteração incompatível exige nova versão.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="54" customHeight="1">
       <x:c r="A32" s="6" t="s">
+        <x:v>191</x:v>
+      </x:c>
+      <x:c r="B32" s="6" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="C32" s="6" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="D32" s="6" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="E32" s="6" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="F32" s="6" t="s">
         <x:v>194</x:v>
       </x:c>
-      <x:c r="B32" s="6" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C32" s="6" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="D32" s="6" t="s">
-        <x:v>195</x:v>
-      </x:c>
-      <x:c r="E32" s="6" t="s">
-        <x:v>196</x:v>
-      </x:c>
-      <x:c r="F32" s="6" t="s">
-        <x:v>197</x:v>
-      </x:c>
-      <x:c r="G32" s="10" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H32" s="6" t="s">
-        <x:v>198</x:v>
-      </x:c>
-      <x:c r="I32" s="6" t="s">
-        <x:v>199</x:v>
+      <x:c r="G32" s="10" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="H32" s="6" t="str">
+        <x:v>reporting.py e a interface geram relatório científico Markdown v1 com fingerprint, premissas, resultados, fontes anexadas ou ausência explícita, prontidão, campos ausentes, limitações e bloqueio de recomendação.</x:v>
+      </x:c>
+      <x:c r="I32" s="6" t="str">
+        <x:v>Evoluir o template somente com fontes aprovadas e resultados adicionais; preservar a distinção entre cálculo, evidência e validação.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="54" customHeight="1">
       <x:c r="A33" s="5" t="s">
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="B33" s="5" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="C33" s="5" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="D33" s="5" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="E33" s="5" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="F33" s="5" t="s">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="B33" s="5" t="s">
+      <x:c r="G33" s="11" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H33" s="5" t="s">
         <x:v>201</x:v>
       </x:c>
-      <x:c r="C33" s="5" t="s">
+      <x:c r="I33" s="5" t="s">
         <x:v>202</x:v>
-      </x:c>
-      <x:c r="D33" s="5" t="s">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="E33" s="5" t="s">
-        <x:v>204</x:v>
-      </x:c>
-      <x:c r="F33" s="5" t="s">
-        <x:v>205</x:v>
-      </x:c>
-      <x:c r="G33" s="11" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="H33" s="5" t="s">
-        <x:v>206</x:v>
-      </x:c>
-      <x:c r="I33" s="5" t="s">
-        <x:v>207</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="54" customHeight="1">
       <x:c r="A34" s="6" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="B34" s="6" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="C34" s="6" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="D34" s="6" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="E34" s="6" t="s">
+        <x:v>205</x:v>
+      </x:c>
+      <x:c r="F34" s="6" t="s">
+        <x:v>206</x:v>
+      </x:c>
+      <x:c r="G34" s="10" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H34" s="6" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="I34" s="6" t="s">
         <x:v>208</x:v>
-      </x:c>
-      <x:c r="B34" s="6" t="s">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="C34" s="6" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="D34" s="6" t="s">
-        <x:v>209</x:v>
-      </x:c>
-      <x:c r="E34" s="6" t="s">
-        <x:v>210</x:v>
-      </x:c>
-      <x:c r="F34" s="6" t="s">
-        <x:v>211</x:v>
-      </x:c>
-      <x:c r="G34" s="10" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H34" s="6" t="s">
-        <x:v>212</x:v>
-      </x:c>
-      <x:c r="I34" s="6" t="s">
-        <x:v>213</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="54" customHeight="1">
       <x:c r="A35" s="5" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="B35" s="5" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="C35" s="5" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="D35" s="5" t="s">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="E35" s="5" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="F35" s="5" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="G35" s="9" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H35" s="5" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="I35" s="5" t="s">
         <x:v>214</x:v>
-      </x:c>
-      <x:c r="B35" s="5" t="s">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="C35" s="5" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="D35" s="5" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="E35" s="5" t="s">
-        <x:v>216</x:v>
-      </x:c>
-      <x:c r="F35" s="5" t="s">
-        <x:v>217</x:v>
-      </x:c>
-      <x:c r="G35" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H35" s="5" t="s">
-        <x:v>218</x:v>
-      </x:c>
-      <x:c r="I35" s="5" t="s">
-        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="54" customHeight="1">
       <x:c r="A36" s="6" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="B36" s="6" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="C36" s="6" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="D36" s="6" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="E36" s="6" t="s">
+        <x:v>217</x:v>
+      </x:c>
+      <x:c r="F36" s="6" t="s">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="G36" s="11" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H36" s="6" t="s">
+        <x:v>219</x:v>
+      </x:c>
+      <x:c r="I36" s="6" t="s">
         <x:v>220</x:v>
-      </x:c>
-      <x:c r="B36" s="6" t="s">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="C36" s="6" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="D36" s="6" t="s">
-        <x:v>221</x:v>
-      </x:c>
-      <x:c r="E36" s="6" t="s">
-        <x:v>222</x:v>
-      </x:c>
-      <x:c r="F36" s="6" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="G36" s="11" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="H36" s="6" t="s">
-        <x:v>224</x:v>
-      </x:c>
-      <x:c r="I36" s="6" t="s">
-        <x:v>225</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="54" customHeight="1">
       <x:c r="A37" s="5" t="s">
+        <x:v>221</x:v>
+      </x:c>
+      <x:c r="B37" s="5" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="C37" s="5" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="D37" s="5" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="E37" s="5" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="F37" s="5" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="G37" s="9" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H37" s="5" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="I37" s="5" t="s">
         <x:v>226</x:v>
-      </x:c>
-      <x:c r="B37" s="5" t="s">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="C37" s="5" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="D37" s="5" t="s">
-        <x:v>227</x:v>
-      </x:c>
-      <x:c r="E37" s="5" t="s">
-        <x:v>228</x:v>
-      </x:c>
-      <x:c r="F37" s="5" t="s">
-        <x:v>229</x:v>
-      </x:c>
-      <x:c r="G37" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H37" s="5" t="s">
-        <x:v>230</x:v>
-      </x:c>
-      <x:c r="I37" s="5" t="s">
-        <x:v>231</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="54" customHeight="1">
       <x:c r="A38" s="6" t="s">
+        <x:v>227</x:v>
+      </x:c>
+      <x:c r="B38" s="6" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="C38" s="6" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="D38" s="6" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="E38" s="6" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="F38" s="6" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="G38" s="10" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H38" s="6" t="s">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="I38" s="6" t="s">
         <x:v>232</x:v>
-      </x:c>
-      <x:c r="B38" s="6" t="s">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="C38" s="6" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="D38" s="6" t="s">
-        <x:v>233</x:v>
-      </x:c>
-      <x:c r="E38" s="6" t="s">
-        <x:v>234</x:v>
-      </x:c>
-      <x:c r="F38" s="6" t="s">
-        <x:v>235</x:v>
-      </x:c>
-      <x:c r="G38" s="10" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H38" s="6" t="s">
-        <x:v>236</x:v>
-      </x:c>
-      <x:c r="I38" s="6" t="s">
-        <x:v>237</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="54" customHeight="1">
       <x:c r="A39" s="5" t="s">
+        <x:v>233</x:v>
+      </x:c>
+      <x:c r="B39" s="5" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="C39" s="5" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="D39" s="5" t="s">
+        <x:v>234</x:v>
+      </x:c>
+      <x:c r="E39" s="5" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="F39" s="5" t="s">
+        <x:v>236</x:v>
+      </x:c>
+      <x:c r="G39" s="11" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H39" s="5" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="I39" s="5" t="s">
         <x:v>238</x:v>
-      </x:c>
-      <x:c r="B39" s="5" t="s">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="C39" s="5" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="D39" s="5" t="s">
-        <x:v>239</x:v>
-      </x:c>
-      <x:c r="E39" s="5" t="s">
-        <x:v>240</x:v>
-      </x:c>
-      <x:c r="F39" s="5" t="s">
-        <x:v>241</x:v>
-      </x:c>
-      <x:c r="G39" s="11" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="H39" s="5" t="s">
-        <x:v>242</x:v>
-      </x:c>
-      <x:c r="I39" s="5" t="s">
-        <x:v>243</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="54" customHeight="1">
       <x:c r="A40" s="6" t="s">
+        <x:v>239</x:v>
+      </x:c>
+      <x:c r="B40" s="6" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="C40" s="6" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="D40" s="6" t="s">
+        <x:v>242</x:v>
+      </x:c>
+      <x:c r="E40" s="6" t="s">
+        <x:v>243</x:v>
+      </x:c>
+      <x:c r="F40" s="6" t="s">
         <x:v>244</x:v>
       </x:c>
-      <x:c r="B40" s="6" t="s">
+      <x:c r="G40" s="10" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H40" s="6" t="s">
         <x:v>245</x:v>
       </x:c>
-      <x:c r="C40" s="6" t="s">
+      <x:c r="I40" s="6" t="s">
         <x:v>246</x:v>
-      </x:c>
-      <x:c r="D40" s="6" t="s">
-        <x:v>247</x:v>
-      </x:c>
-      <x:c r="E40" s="6" t="s">
-        <x:v>248</x:v>
-      </x:c>
-      <x:c r="F40" s="6" t="s">
-        <x:v>249</x:v>
-      </x:c>
-      <x:c r="G40" s="10" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H40" s="6" t="s">
-        <x:v>250</x:v>
-      </x:c>
-      <x:c r="I40" s="6" t="s">
-        <x:v>251</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="54" customHeight="1">
       <x:c r="A41" s="5" t="s">
+        <x:v>247</x:v>
+      </x:c>
+      <x:c r="B41" s="5" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="C41" s="5" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="D41" s="5" t="s">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="E41" s="5" t="s">
+        <x:v>249</x:v>
+      </x:c>
+      <x:c r="F41" s="5" t="s">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="G41" s="10" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H41" s="5" t="s">
+        <x:v>251</x:v>
+      </x:c>
+      <x:c r="I41" s="5" t="s">
         <x:v>252</x:v>
-      </x:c>
-      <x:c r="B41" s="5" t="s">
-        <x:v>245</x:v>
-      </x:c>
-      <x:c r="C41" s="5" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="D41" s="5" t="s">
-        <x:v>253</x:v>
-      </x:c>
-      <x:c r="E41" s="5" t="s">
-        <x:v>254</x:v>
-      </x:c>
-      <x:c r="F41" s="5" t="s">
-        <x:v>255</x:v>
-      </x:c>
-      <x:c r="G41" s="10" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H41" s="5" t="s">
-        <x:v>256</x:v>
-      </x:c>
-      <x:c r="I41" s="5" t="s">
-        <x:v>257</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="54" customHeight="1">
       <x:c r="A42" s="6" t="s">
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="B42" s="6" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="C42" s="6" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="D42" s="6" t="s">
+        <x:v>254</x:v>
+      </x:c>
+      <x:c r="E42" s="6" t="s">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="F42" s="6" t="s">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="G42" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H42" s="6" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="I42" s="6" t="s">
         <x:v>258</x:v>
-      </x:c>
-      <x:c r="B42" s="6" t="s">
-        <x:v>245</x:v>
-      </x:c>
-      <x:c r="C42" s="6" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="D42" s="6" t="s">
-        <x:v>259</x:v>
-      </x:c>
-      <x:c r="E42" s="6" t="s">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="F42" s="6" t="s">
-        <x:v>261</x:v>
-      </x:c>
-      <x:c r="G42" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H42" s="6" t="s">
-        <x:v>262</x:v>
-      </x:c>
-      <x:c r="I42" s="6" t="s">
-        <x:v>263</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="54" customHeight="1">
       <x:c r="A43" s="5" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="B43" s="5" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="C43" s="5" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="D43" s="5" t="s">
+        <x:v>260</x:v>
+      </x:c>
+      <x:c r="E43" s="5" t="s">
+        <x:v>261</x:v>
+      </x:c>
+      <x:c r="F43" s="5" t="s">
+        <x:v>262</x:v>
+      </x:c>
+      <x:c r="G43" s="11" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H43" s="5" t="s">
+        <x:v>263</x:v>
+      </x:c>
+      <x:c r="I43" s="5" t="s">
         <x:v>264</x:v>
-      </x:c>
-      <x:c r="B43" s="5" t="s">
-        <x:v>245</x:v>
-      </x:c>
-      <x:c r="C43" s="5" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="D43" s="5" t="s">
-        <x:v>265</x:v>
-      </x:c>
-      <x:c r="E43" s="5" t="s">
-        <x:v>266</x:v>
-      </x:c>
-      <x:c r="F43" s="5" t="s">
-        <x:v>267</x:v>
-      </x:c>
-      <x:c r="G43" s="11" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="H43" s="5" t="s">
-        <x:v>268</x:v>
-      </x:c>
-      <x:c r="I43" s="5" t="s">
-        <x:v>269</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="54" customHeight="1">
       <x:c r="A44" s="6" t="s">
+        <x:v>265</x:v>
+      </x:c>
+      <x:c r="B44" s="6" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="C44" s="6" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="D44" s="6" t="s">
+        <x:v>266</x:v>
+      </x:c>
+      <x:c r="E44" s="6" t="s">
+        <x:v>267</x:v>
+      </x:c>
+      <x:c r="F44" s="6" t="s">
+        <x:v>268</x:v>
+      </x:c>
+      <x:c r="G44" s="9" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H44" s="6" t="s">
+        <x:v>269</x:v>
+      </x:c>
+      <x:c r="I44" s="6" t="s">
         <x:v>270</x:v>
-      </x:c>
-      <x:c r="B44" s="6" t="s">
-        <x:v>245</x:v>
-      </x:c>
-      <x:c r="C44" s="6" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="D44" s="6" t="s">
-        <x:v>271</x:v>
-      </x:c>
-      <x:c r="E44" s="6" t="s">
-        <x:v>272</x:v>
-      </x:c>
-      <x:c r="F44" s="6" t="s">
-        <x:v>273</x:v>
-      </x:c>
-      <x:c r="G44" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H44" s="6" t="s">
-        <x:v>274</x:v>
-      </x:c>
-      <x:c r="I44" s="6" t="s">
-        <x:v>275</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="54" customHeight="1">
       <x:c r="A45" s="5" t="s">
+        <x:v>271</x:v>
+      </x:c>
+      <x:c r="B45" s="5" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="C45" s="5" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="D45" s="5" t="s">
+        <x:v>272</x:v>
+      </x:c>
+      <x:c r="E45" s="5" t="s">
+        <x:v>273</x:v>
+      </x:c>
+      <x:c r="F45" s="5" t="s">
+        <x:v>274</x:v>
+      </x:c>
+      <x:c r="G45" s="8" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H45" s="5" t="s">
+        <x:v>275</x:v>
+      </x:c>
+      <x:c r="I45" s="5" t="s">
         <x:v>276</x:v>
-      </x:c>
-      <x:c r="B45" s="5" t="s">
-        <x:v>245</x:v>
-      </x:c>
-      <x:c r="C45" s="5" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="D45" s="5" t="s">
-        <x:v>277</x:v>
-      </x:c>
-      <x:c r="E45" s="5" t="s">
-        <x:v>278</x:v>
-      </x:c>
-      <x:c r="F45" s="5" t="s">
-        <x:v>279</x:v>
-      </x:c>
-      <x:c r="G45" s="8" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H45" s="5" t="s">
-        <x:v>280</x:v>
-      </x:c>
-      <x:c r="I45" s="5" t="s">
-        <x:v>281</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="54" customHeight="1">
       <x:c r="A46" s="6" t="s">
+        <x:v>277</x:v>
+      </x:c>
+      <x:c r="B46" s="6" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="C46" s="6" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="D46" s="6" t="s">
+        <x:v>278</x:v>
+      </x:c>
+      <x:c r="E46" s="6" t="s">
+        <x:v>279</x:v>
+      </x:c>
+      <x:c r="F46" s="6" t="s">
+        <x:v>280</x:v>
+      </x:c>
+      <x:c r="G46" s="11" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H46" s="6" t="s">
+        <x:v>281</x:v>
+      </x:c>
+      <x:c r="I46" s="6" t="s">
         <x:v>282</x:v>
-      </x:c>
-      <x:c r="B46" s="6" t="s">
-        <x:v>245</x:v>
-      </x:c>
-      <x:c r="C46" s="6" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="D46" s="6" t="s">
-        <x:v>283</x:v>
-      </x:c>
-      <x:c r="E46" s="6" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="F46" s="6" t="s">
-        <x:v>285</x:v>
-      </x:c>
-      <x:c r="G46" s="11" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="H46" s="6" t="s">
-        <x:v>286</x:v>
-      </x:c>
-      <x:c r="I46" s="6" t="s">
-        <x:v>287</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="54" customHeight="1">
       <x:c r="A47" s="5" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="B47" s="5" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="C47" s="5" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="D47" s="5" t="s">
+        <x:v>286</x:v>
+      </x:c>
+      <x:c r="E47" s="5" t="s">
+        <x:v>287</x:v>
+      </x:c>
+      <x:c r="F47" s="5" t="s">
         <x:v>288</x:v>
       </x:c>
-      <x:c r="B47" s="5" t="s">
+      <x:c r="G47" s="9" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H47" s="5" t="s">
         <x:v>289</x:v>
       </x:c>
-      <x:c r="C47" s="5" t="s">
+      <x:c r="I47" s="5" t="s">
         <x:v>290</x:v>
-      </x:c>
-      <x:c r="D47" s="5" t="s">
-        <x:v>291</x:v>
-      </x:c>
-      <x:c r="E47" s="5" t="s">
-        <x:v>292</x:v>
-      </x:c>
-      <x:c r="F47" s="5" t="s">
-        <x:v>293</x:v>
-      </x:c>
-      <x:c r="G47" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H47" s="5" t="s">
-        <x:v>294</x:v>
-      </x:c>
-      <x:c r="I47" s="5" t="s">
-        <x:v>295</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="54" customHeight="1">
       <x:c r="A48" s="6" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="B48" s="6" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="C48" s="6" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="D48" s="6" t="s">
+        <x:v>292</x:v>
+      </x:c>
+      <x:c r="E48" s="6" t="s">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="F48" s="6" t="s">
+        <x:v>294</x:v>
+      </x:c>
+      <x:c r="G48" s="9" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H48" s="6" t="s">
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="I48" s="6" t="s">
         <x:v>296</x:v>
-      </x:c>
-      <x:c r="B48" s="6" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="C48" s="6" t="s">
-        <x:v>290</x:v>
-      </x:c>
-      <x:c r="D48" s="6" t="s">
-        <x:v>297</x:v>
-      </x:c>
-      <x:c r="E48" s="6" t="s">
-        <x:v>298</x:v>
-      </x:c>
-      <x:c r="F48" s="6" t="s">
-        <x:v>299</x:v>
-      </x:c>
-      <x:c r="G48" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H48" s="6" t="s">
-        <x:v>300</x:v>
-      </x:c>
-      <x:c r="I48" s="6" t="s">
-        <x:v>301</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="54" customHeight="1">
       <x:c r="A49" s="5" t="s">
+        <x:v>297</x:v>
+      </x:c>
+      <x:c r="B49" s="5" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="C49" s="5" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="D49" s="5" t="s">
+        <x:v>298</x:v>
+      </x:c>
+      <x:c r="E49" s="5" t="s">
+        <x:v>299</x:v>
+      </x:c>
+      <x:c r="F49" s="5" t="s">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="G49" s="9" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H49" s="5" t="s">
+        <x:v>301</x:v>
+      </x:c>
+      <x:c r="I49" s="5" t="s">
         <x:v>302</x:v>
-      </x:c>
-      <x:c r="B49" s="5" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="C49" s="5" t="s">
-        <x:v>290</x:v>
-      </x:c>
-      <x:c r="D49" s="5" t="s">
-        <x:v>303</x:v>
-      </x:c>
-      <x:c r="E49" s="5" t="s">
-        <x:v>304</x:v>
-      </x:c>
-      <x:c r="F49" s="5" t="s">
-        <x:v>305</x:v>
-      </x:c>
-      <x:c r="G49" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H49" s="5" t="s">
-        <x:v>306</x:v>
-      </x:c>
-      <x:c r="I49" s="5" t="s">
-        <x:v>307</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="54" customHeight="1">
       <x:c r="A50" s="6" t="s">
+        <x:v>303</x:v>
+      </x:c>
+      <x:c r="B50" s="6" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="C50" s="6" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="D50" s="6" t="s">
+        <x:v>304</x:v>
+      </x:c>
+      <x:c r="E50" s="6" t="s">
+        <x:v>305</x:v>
+      </x:c>
+      <x:c r="F50" s="6" t="s">
+        <x:v>306</x:v>
+      </x:c>
+      <x:c r="G50" s="9" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H50" s="6" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="I50" s="6" t="s">
         <x:v>308</x:v>
-      </x:c>
-      <x:c r="B50" s="6" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="C50" s="6" t="s">
-        <x:v>290</x:v>
-      </x:c>
-      <x:c r="D50" s="6" t="s">
-        <x:v>309</x:v>
-      </x:c>
-      <x:c r="E50" s="6" t="s">
-        <x:v>310</x:v>
-      </x:c>
-      <x:c r="F50" s="6" t="s">
-        <x:v>311</x:v>
-      </x:c>
-      <x:c r="G50" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H50" s="6" t="s">
-        <x:v>312</x:v>
-      </x:c>
-      <x:c r="I50" s="6" t="s">
-        <x:v>313</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="54" customHeight="1">
       <x:c r="A51" s="5" t="s">
+        <x:v>309</x:v>
+      </x:c>
+      <x:c r="B51" s="5" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="C51" s="5" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="D51" s="5" t="s">
+        <x:v>310</x:v>
+      </x:c>
+      <x:c r="E51" s="5" t="s">
+        <x:v>311</x:v>
+      </x:c>
+      <x:c r="F51" s="5" t="s">
+        <x:v>312</x:v>
+      </x:c>
+      <x:c r="G51" s="9" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H51" s="5" t="s">
+        <x:v>313</x:v>
+      </x:c>
+      <x:c r="I51" s="5" t="s">
         <x:v>314</x:v>
-      </x:c>
-      <x:c r="B51" s="5" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="C51" s="5" t="s">
-        <x:v>290</x:v>
-      </x:c>
-      <x:c r="D51" s="5" t="s">
-        <x:v>315</x:v>
-      </x:c>
-      <x:c r="E51" s="5" t="s">
-        <x:v>316</x:v>
-      </x:c>
-      <x:c r="F51" s="5" t="s">
-        <x:v>317</x:v>
-      </x:c>
-      <x:c r="G51" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H51" s="5" t="s">
-        <x:v>318</x:v>
-      </x:c>
-      <x:c r="I51" s="5" t="s">
-        <x:v>319</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="54" customHeight="1">
       <x:c r="A52" s="6" t="s">
+        <x:v>315</x:v>
+      </x:c>
+      <x:c r="B52" s="6" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="C52" s="6" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="D52" s="6" t="s">
+        <x:v>316</x:v>
+      </x:c>
+      <x:c r="E52" s="6" t="s">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c r="F52" s="6" t="s">
+        <x:v>318</x:v>
+      </x:c>
+      <x:c r="G52" s="9" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H52" s="6" t="s">
+        <x:v>319</x:v>
+      </x:c>
+      <x:c r="I52" s="6" t="s">
         <x:v>320</x:v>
-      </x:c>
-      <x:c r="B52" s="6" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="C52" s="6" t="s">
-        <x:v>290</x:v>
-      </x:c>
-      <x:c r="D52" s="6" t="s">
-        <x:v>321</x:v>
-      </x:c>
-      <x:c r="E52" s="6" t="s">
-        <x:v>322</x:v>
-      </x:c>
-      <x:c r="F52" s="6" t="s">
-        <x:v>323</x:v>
-      </x:c>
-      <x:c r="G52" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H52" s="6" t="s">
-        <x:v>324</x:v>
-      </x:c>
-      <x:c r="I52" s="6" t="s">
-        <x:v>325</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="54" customHeight="1">
       <x:c r="A53" s="5" t="s">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="B53" s="5" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="C53" s="5" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="D53" s="5" t="s">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="E53" s="5" t="s">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="F53" s="5" t="s">
         <x:v>326</x:v>
       </x:c>
-      <x:c r="B53" s="5" t="s">
+      <x:c r="G53" s="9" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H53" s="5" t="s">
         <x:v>327</x:v>
       </x:c>
-      <x:c r="C53" s="5" t="s">
+      <x:c r="I53" s="5" t="s">
         <x:v>328</x:v>
-      </x:c>
-      <x:c r="D53" s="5" t="s">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="E53" s="5" t="s">
-        <x:v>330</x:v>
-      </x:c>
-      <x:c r="F53" s="5" t="s">
-        <x:v>331</x:v>
-      </x:c>
-      <x:c r="G53" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H53" s="5" t="s">
-        <x:v>332</x:v>
-      </x:c>
-      <x:c r="I53" s="5" t="s">
-        <x:v>333</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="54" customHeight="1">
       <x:c r="A54" s="6" t="s">
+        <x:v>329</x:v>
+      </x:c>
+      <x:c r="B54" s="6" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="C54" s="6" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="D54" s="6" t="s">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="E54" s="6" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="F54" s="6" t="s">
+        <x:v>332</x:v>
+      </x:c>
+      <x:c r="G54" s="9" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H54" s="6" t="s">
+        <x:v>333</x:v>
+      </x:c>
+      <x:c r="I54" s="6" t="s">
         <x:v>334</x:v>
-      </x:c>
-      <x:c r="B54" s="6" t="s">
-        <x:v>327</x:v>
-      </x:c>
-      <x:c r="C54" s="6" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="D54" s="6" t="s">
-        <x:v>335</x:v>
-      </x:c>
-      <x:c r="E54" s="6" t="s">
-        <x:v>336</x:v>
-      </x:c>
-      <x:c r="F54" s="6" t="s">
-        <x:v>337</x:v>
-      </x:c>
-      <x:c r="G54" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H54" s="6" t="s">
-        <x:v>338</x:v>
-      </x:c>
-      <x:c r="I54" s="6" t="s">
-        <x:v>339</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="54" customHeight="1">
       <x:c r="A55" s="5" t="s">
+        <x:v>335</x:v>
+      </x:c>
+      <x:c r="B55" s="5" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="C55" s="5" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="D55" s="5" t="s">
+        <x:v>336</x:v>
+      </x:c>
+      <x:c r="E55" s="5" t="s">
+        <x:v>337</x:v>
+      </x:c>
+      <x:c r="F55" s="5" t="s">
+        <x:v>338</x:v>
+      </x:c>
+      <x:c r="G55" s="10" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H55" s="5" t="s">
+        <x:v>339</x:v>
+      </x:c>
+      <x:c r="I55" s="5" t="s">
         <x:v>340</x:v>
-      </x:c>
-      <x:c r="B55" s="5" t="s">
-        <x:v>327</x:v>
-      </x:c>
-      <x:c r="C55" s="5" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="D55" s="5" t="s">
-        <x:v>341</x:v>
-      </x:c>
-      <x:c r="E55" s="5" t="s">
-        <x:v>342</x:v>
-      </x:c>
-      <x:c r="F55" s="5" t="s">
-        <x:v>343</x:v>
-      </x:c>
-      <x:c r="G55" s="10" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H55" s="5" t="s">
-        <x:v>344</x:v>
-      </x:c>
-      <x:c r="I55" s="5" t="s">
-        <x:v>345</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="54" customHeight="1">
       <x:c r="A56" s="6" t="s">
+        <x:v>341</x:v>
+      </x:c>
+      <x:c r="B56" s="6" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="C56" s="6" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="D56" s="6" t="s">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="E56" s="6" t="s">
+        <x:v>343</x:v>
+      </x:c>
+      <x:c r="F56" s="6" t="s">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="G56" s="10" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H56" s="6" t="s">
+        <x:v>345</x:v>
+      </x:c>
+      <x:c r="I56" s="6" t="s">
         <x:v>346</x:v>
-      </x:c>
-      <x:c r="B56" s="6" t="s">
-        <x:v>327</x:v>
-      </x:c>
-      <x:c r="C56" s="6" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="D56" s="6" t="s">
-        <x:v>347</x:v>
-      </x:c>
-      <x:c r="E56" s="6" t="s">
-        <x:v>348</x:v>
-      </x:c>
-      <x:c r="F56" s="6" t="s">
-        <x:v>349</x:v>
-      </x:c>
-      <x:c r="G56" s="10" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H56" s="6" t="s">
-        <x:v>350</x:v>
-      </x:c>
-      <x:c r="I56" s="6" t="s">
-        <x:v>351</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="54" customHeight="1">
       <x:c r="A57" s="5" t="s">
+        <x:v>347</x:v>
+      </x:c>
+      <x:c r="B57" s="5" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="C57" s="5" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="D57" s="5" t="s">
+        <x:v>348</x:v>
+      </x:c>
+      <x:c r="E57" s="5" t="s">
+        <x:v>349</x:v>
+      </x:c>
+      <x:c r="F57" s="5" t="s">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="G57" s="9" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H57" s="5" t="s">
+        <x:v>351</x:v>
+      </x:c>
+      <x:c r="I57" s="5" t="s">
         <x:v>352</x:v>
-      </x:c>
-      <x:c r="B57" s="5" t="s">
-        <x:v>327</x:v>
-      </x:c>
-      <x:c r="C57" s="5" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="D57" s="5" t="s">
-        <x:v>353</x:v>
-      </x:c>
-      <x:c r="E57" s="5" t="s">
-        <x:v>354</x:v>
-      </x:c>
-      <x:c r="F57" s="5" t="s">
-        <x:v>355</x:v>
-      </x:c>
-      <x:c r="G57" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H57" s="5" t="s">
-        <x:v>356</x:v>
-      </x:c>
-      <x:c r="I57" s="5" t="s">
-        <x:v>357</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="54" customHeight="1">
       <x:c r="A58" s="6" t="s">
+        <x:v>353</x:v>
+      </x:c>
+      <x:c r="B58" s="6" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="C58" s="6" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="D58" s="6" t="s">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="E58" s="6" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="F58" s="6" t="s">
+        <x:v>356</x:v>
+      </x:c>
+      <x:c r="G58" s="9" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H58" s="6" t="s">
+        <x:v>357</x:v>
+      </x:c>
+      <x:c r="I58" s="6" t="s">
         <x:v>358</x:v>
-      </x:c>
-      <x:c r="B58" s="6" t="s">
-        <x:v>327</x:v>
-      </x:c>
-      <x:c r="C58" s="6" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="D58" s="6" t="s">
-        <x:v>359</x:v>
-      </x:c>
-      <x:c r="E58" s="6" t="s">
-        <x:v>360</x:v>
-      </x:c>
-      <x:c r="F58" s="6" t="s">
-        <x:v>361</x:v>
-      </x:c>
-      <x:c r="G58" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H58" s="6" t="s">
-        <x:v>362</x:v>
-      </x:c>
-      <x:c r="I58" s="6" t="s">
-        <x:v>363</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="54" customHeight="1">
       <x:c r="A59" s="5" t="s">
+        <x:v>359</x:v>
+      </x:c>
+      <x:c r="B59" s="5" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="C59" s="5" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="D59" s="5" t="s">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="E59" s="5" t="s">
+        <x:v>361</x:v>
+      </x:c>
+      <x:c r="F59" s="5" t="s">
+        <x:v>362</x:v>
+      </x:c>
+      <x:c r="G59" s="10" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H59" s="5" t="s">
+        <x:v>363</x:v>
+      </x:c>
+      <x:c r="I59" s="5" t="s">
         <x:v>364</x:v>
-      </x:c>
-      <x:c r="B59" s="5" t="s">
-        <x:v>327</x:v>
-      </x:c>
-      <x:c r="C59" s="5" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="D59" s="5" t="s">
-        <x:v>365</x:v>
-      </x:c>
-      <x:c r="E59" s="5" t="s">
-        <x:v>366</x:v>
-      </x:c>
-      <x:c r="F59" s="5" t="s">
-        <x:v>367</x:v>
-      </x:c>
-      <x:c r="G59" s="10" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H59" s="5" t="s">
-        <x:v>368</x:v>
-      </x:c>
-      <x:c r="I59" s="5" t="s">
-        <x:v>369</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="54" customHeight="1">
       <x:c r="A60" s="6" t="s">
+        <x:v>365</x:v>
+      </x:c>
+      <x:c r="B60" s="6" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="C60" s="6" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="D60" s="6" t="s">
+        <x:v>366</x:v>
+      </x:c>
+      <x:c r="E60" s="6" t="s">
+        <x:v>367</x:v>
+      </x:c>
+      <x:c r="F60" s="6" t="s">
+        <x:v>368</x:v>
+      </x:c>
+      <x:c r="G60" s="10" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H60" s="6" t="s">
+        <x:v>369</x:v>
+      </x:c>
+      <x:c r="I60" s="6" t="s">
         <x:v>370</x:v>
-      </x:c>
-      <x:c r="B60" s="6" t="s">
-        <x:v>327</x:v>
-      </x:c>
-      <x:c r="C60" s="6" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="D60" s="6" t="s">
-        <x:v>371</x:v>
-      </x:c>
-      <x:c r="E60" s="6" t="s">
-        <x:v>372</x:v>
-      </x:c>
-      <x:c r="F60" s="6" t="s">
-        <x:v>373</x:v>
-      </x:c>
-      <x:c r="G60" s="10" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H60" s="6" t="s">
-        <x:v>374</x:v>
-      </x:c>
-      <x:c r="I60" s="6" t="s">
-        <x:v>375</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="52" customHeight="1">
       <x:c r="A61" s="24" t="s">
+        <x:v>371</x:v>
+      </x:c>
+      <x:c r="B61" s="24" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="C61" s="24" t="s">
+        <x:v>372</x:v>
+      </x:c>
+      <x:c r="D61" s="24" t="s">
+        <x:v>373</x:v>
+      </x:c>
+      <x:c r="E61" s="24" t="s">
+        <x:v>374</x:v>
+      </x:c>
+      <x:c r="F61" s="24" t="s">
+        <x:v>375</x:v>
+      </x:c>
+      <x:c r="G61" s="31" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H61" s="24" t="s">
         <x:v>376</x:v>
       </x:c>
-      <x:c r="B61" s="24" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="C61" s="24" t="s">
+      <x:c r="I61" s="24" t="s">
         <x:v>377</x:v>
-      </x:c>
-      <x:c r="D61" s="24" t="s">
-        <x:v>378</x:v>
-      </x:c>
-      <x:c r="E61" s="24" t="s">
-        <x:v>379</x:v>
-      </x:c>
-      <x:c r="F61" s="24" t="s">
-        <x:v>380</x:v>
-      </x:c>
-      <x:c r="G61" s="31" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H61" s="24" t="s">
-        <x:v>381</x:v>
-      </x:c>
-      <x:c r="I61" s="24" t="s">
-        <x:v>382</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="52" customHeight="1">
       <x:c r="A62" s="24" t="s">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="B62" s="24" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="C62" s="24" t="s">
+        <x:v>372</x:v>
+      </x:c>
+      <x:c r="D62" s="24" t="s">
+        <x:v>379</x:v>
+      </x:c>
+      <x:c r="E62" s="24" t="s">
+        <x:v>380</x:v>
+      </x:c>
+      <x:c r="F62" s="24" t="s">
+        <x:v>381</x:v>
+      </x:c>
+      <x:c r="G62" s="32" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H62" s="24" t="s">
+        <x:v>382</x:v>
+      </x:c>
+      <x:c r="I62" s="24" t="s">
         <x:v>383</x:v>
-      </x:c>
-      <x:c r="B62" s="24" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="C62" s="24" t="s">
-        <x:v>377</x:v>
-      </x:c>
-      <x:c r="D62" s="24" t="s">
-        <x:v>384</x:v>
-      </x:c>
-      <x:c r="E62" s="24" t="s">
-        <x:v>385</x:v>
-      </x:c>
-      <x:c r="F62" s="24" t="s">
-        <x:v>386</x:v>
-      </x:c>
-      <x:c r="G62" s="32" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H62" s="24" t="s">
-        <x:v>387</x:v>
-      </x:c>
-      <x:c r="I62" s="24" t="s">
-        <x:v>388</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="52" customHeight="1">
       <x:c r="A63" s="24" t="s">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="B63" s="24" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="C63" s="24" t="s">
+        <x:v>372</x:v>
+      </x:c>
+      <x:c r="D63" s="24" t="s">
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="E63" s="24" t="s">
+        <x:v>386</x:v>
+      </x:c>
+      <x:c r="F63" s="24" t="s">
+        <x:v>387</x:v>
+      </x:c>
+      <x:c r="G63" s="32" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H63" s="24" t="s">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="I63" s="24" t="s">
         <x:v>389</x:v>
-      </x:c>
-      <x:c r="B63" s="24" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="C63" s="24" t="s">
-        <x:v>377</x:v>
-      </x:c>
-      <x:c r="D63" s="24" t="s">
-        <x:v>390</x:v>
-      </x:c>
-      <x:c r="E63" s="24" t="s">
-        <x:v>391</x:v>
-      </x:c>
-      <x:c r="F63" s="24" t="s">
-        <x:v>392</x:v>
-      </x:c>
-      <x:c r="G63" s="32" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H63" s="24" t="s">
-        <x:v>393</x:v>
-      </x:c>
-      <x:c r="I63" s="24" t="s">
-        <x:v>394</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="52" customHeight="1">
       <x:c r="A64" s="24" t="s">
-        <x:v>395</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="B64" s="24" t="s">
-        <x:v>289</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="C64" s="24" t="s">
-        <x:v>377</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="D64" s="24" t="s">
-        <x:v>396</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="E64" s="24" t="s">
-        <x:v>397</x:v>
+        <x:v>392</x:v>
       </x:c>
       <x:c r="F64" s="24" t="s">
-        <x:v>398</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="G64" s="26" t="s">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H64" s="24" t="str">
         <x:v>FT-014 e FT-015 concluídas. O balanço integrado permanece bloqueado enquanto FT-058 e FT-059 não tiverem modelos selecionados e validados.</x:v>
@@ -4269,89 +4254,89 @@
     </x:row>
     <x:row r="65" ht="52" customHeight="1">
       <x:c r="A65" s="24" t="s">
+        <x:v>394</x:v>
+      </x:c>
+      <x:c r="B65" s="24" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="C65" s="24" t="s">
+        <x:v>395</x:v>
+      </x:c>
+      <x:c r="D65" s="24" t="s">
+        <x:v>396</x:v>
+      </x:c>
+      <x:c r="E65" s="24" t="s">
+        <x:v>397</x:v>
+      </x:c>
+      <x:c r="F65" s="24" t="s">
+        <x:v>398</x:v>
+      </x:c>
+      <x:c r="G65" s="25" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H65" s="24" t="s">
         <x:v>399</x:v>
       </x:c>
-      <x:c r="B65" s="24" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="C65" s="24" t="s">
+      <x:c r="I65" s="24" t="s">
         <x:v>400</x:v>
-      </x:c>
-      <x:c r="D65" s="24" t="s">
-        <x:v>401</x:v>
-      </x:c>
-      <x:c r="E65" s="24" t="s">
-        <x:v>402</x:v>
-      </x:c>
-      <x:c r="F65" s="24" t="s">
-        <x:v>403</x:v>
-      </x:c>
-      <x:c r="G65" s="25" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H65" s="24" t="s">
-        <x:v>404</x:v>
-      </x:c>
-      <x:c r="I65" s="24" t="s">
-        <x:v>405</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="52" customHeight="1">
       <x:c r="A66" s="24" t="s">
+        <x:v>401</x:v>
+      </x:c>
+      <x:c r="B66" s="24" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="C66" s="24" t="s">
+        <x:v>395</x:v>
+      </x:c>
+      <x:c r="D66" s="24" t="s">
+        <x:v>402</x:v>
+      </x:c>
+      <x:c r="E66" s="24" t="s">
+        <x:v>403</x:v>
+      </x:c>
+      <x:c r="F66" s="24" t="s">
+        <x:v>404</x:v>
+      </x:c>
+      <x:c r="G66" s="26" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H66" s="24" t="s">
+        <x:v>405</x:v>
+      </x:c>
+      <x:c r="I66" s="24" t="s">
         <x:v>406</x:v>
-      </x:c>
-      <x:c r="B66" s="24" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="C66" s="24" t="s">
-        <x:v>400</x:v>
-      </x:c>
-      <x:c r="D66" s="24" t="s">
-        <x:v>407</x:v>
-      </x:c>
-      <x:c r="E66" s="24" t="s">
-        <x:v>408</x:v>
-      </x:c>
-      <x:c r="F66" s="24" t="s">
-        <x:v>409</x:v>
-      </x:c>
-      <x:c r="G66" s="26" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="H66" s="24" t="s">
-        <x:v>410</x:v>
-      </x:c>
-      <x:c r="I66" s="24" t="s">
-        <x:v>411</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="52" customHeight="1">
       <x:c r="A67" s="24" t="s">
+        <x:v>407</x:v>
+      </x:c>
+      <x:c r="B67" s="24" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="C67" s="24" t="s">
+        <x:v>408</x:v>
+      </x:c>
+      <x:c r="D67" s="24" t="s">
+        <x:v>409</x:v>
+      </x:c>
+      <x:c r="E67" s="24" t="s">
+        <x:v>410</x:v>
+      </x:c>
+      <x:c r="F67" s="24" t="s">
+        <x:v>411</x:v>
+      </x:c>
+      <x:c r="G67" s="26" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H67" s="24" t="s">
         <x:v>412</x:v>
       </x:c>
-      <x:c r="B67" s="24" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="C67" s="24" t="s">
+      <x:c r="I67" s="24" t="s">
         <x:v>413</x:v>
-      </x:c>
-      <x:c r="D67" s="24" t="s">
-        <x:v>414</x:v>
-      </x:c>
-      <x:c r="E67" s="24" t="s">
-        <x:v>415</x:v>
-      </x:c>
-      <x:c r="F67" s="24" t="s">
-        <x:v>416</x:v>
-      </x:c>
-      <x:c r="G67" s="26" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="H67" s="24" t="s">
-        <x:v>417</x:v>
-      </x:c>
-      <x:c r="I67" s="24" t="s">
-        <x:v>418</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -4488,7 +4473,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R259ec3809e634d7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bbcebbdef464ae5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: atualizar planilha de atividades FT-017 a FT-028
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rb5ef86c88fec4c12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R4e027cf4335f46d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rde2ffdd633ae4be5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rb5a1ca0f4bc04bd7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1647,7 +1647,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="48">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1772,6 +1772,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="14" fillId="18" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -3198,8 +3201,8 @@
       <x:c r="F28" s="6" t="s">
         <x:v>174</x:v>
       </x:c>
-      <x:c r="G28" s="8" t="s">
-        <x:v>6</x:v>
+      <x:c r="G28" s="8" t="str">
+        <x:v>GATE CONCLUÍDO/BLOQUEADO</x:v>
       </x:c>
       <x:c r="H28" s="6" t="s">
         <x:v>175</x:v>
@@ -3228,7 +3231,7 @@
         <x:v>180</x:v>
       </x:c>
       <x:c r="G29" s="9" t="str">
-        <x:v>Parcial</x:v>
+        <x:v>CONCLUÍDO</x:v>
       </x:c>
       <x:c r="H29" s="5" t="str">
         <x:v>Contrato ASF-medição v1, módulo asf_measurement.py, schema, CLI e exemplo sintético: alinham base de carbono, calculam resíduos por Cn/corte, MAE, RMSE, qui-quadrado, incertezas e diagnósticos C1/C2/cauda. A validação permanece bloqueada sem evidência aprovada.</x:v>
@@ -3256,8 +3259,8 @@
       <x:c r="F30" s="6" t="s">
         <x:v>184</x:v>
       </x:c>
-      <x:c r="G30" s="8" t="s">
-        <x:v>6</x:v>
+      <x:c r="G30" s="8" t="str">
+        <x:v>CONCLUÍDO</x:v>
       </x:c>
       <x:c r="H30" s="6" t="s">
         <x:v>185</x:v>
@@ -3286,7 +3289,7 @@
         <x:v>190</x:v>
       </x:c>
       <x:c r="G31" s="10" t="str">
-        <x:v>Concluído</x:v>
+        <x:v>CONCLUÍDO</x:v>
       </x:c>
       <x:c r="H31" s="5" t="str">
         <x:v>reporting.py gera JSON canônico, resumo CSV, faixas ASF CSV e manifesto com SHA-256, tipo e tamanho. A interface oferece os downloads e os testes confirmam determinismo, integridade, round-trip e leitura dos CSVs.</x:v>
@@ -3315,7 +3318,7 @@
         <x:v>194</x:v>
       </x:c>
       <x:c r="G32" s="10" t="str">
-        <x:v>Concluído</x:v>
+        <x:v>CONCLUÍDO — USO INTERNO</x:v>
       </x:c>
       <x:c r="H32" s="6" t="str">
         <x:v>reporting.py e a interface geram relatório científico Markdown v1 com fingerprint, premissas, resultados, fontes anexadas ou ausência explícita, prontidão, campos ausentes, limitações e bloqueio de recomendação.</x:v>
@@ -3343,8 +3346,8 @@
       <x:c r="F33" s="5" t="s">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="G33" s="11" t="s">
-        <x:v>9</x:v>
+      <x:c r="G33" s="11" t="str">
+        <x:v>CONCLUÍDO COM BLOQUEIO</x:v>
       </x:c>
       <x:c r="H33" s="5" t="s">
         <x:v>201</x:v>
@@ -3372,8 +3375,8 @@
       <x:c r="F34" s="6" t="s">
         <x:v>206</x:v>
       </x:c>
-      <x:c r="G34" s="10" t="s">
-        <x:v>7</x:v>
+      <x:c r="G34" s="10" t="str">
+        <x:v>CONCLUÍDO COM BLOQUEIO</x:v>
       </x:c>
       <x:c r="H34" s="6" t="s">
         <x:v>207</x:v>
@@ -3401,8 +3404,8 @@
       <x:c r="F35" s="5" t="s">
         <x:v>212</x:v>
       </x:c>
-      <x:c r="G35" s="9" t="s">
-        <x:v>8</x:v>
+      <x:c r="G35" s="9" t="str">
+        <x:v>PORTA IMPLEMENTADA/BLOQUEADA</x:v>
       </x:c>
       <x:c r="H35" s="5" t="s">
         <x:v>213</x:v>
@@ -3430,8 +3433,8 @@
       <x:c r="F36" s="6" t="s">
         <x:v>218</x:v>
       </x:c>
-      <x:c r="G36" s="11" t="s">
-        <x:v>9</x:v>
+      <x:c r="G36" s="11" t="str">
+        <x:v>CONCLUÍDO — INFRAESTRUTURA</x:v>
       </x:c>
       <x:c r="H36" s="6" t="s">
         <x:v>219</x:v>
@@ -3459,8 +3462,8 @@
       <x:c r="F37" s="5" t="s">
         <x:v>224</x:v>
       </x:c>
-      <x:c r="G37" s="9" t="s">
-        <x:v>8</x:v>
+      <x:c r="G37" s="9" t="str">
+        <x:v>CONCLUÍDO COM BLOQUEIO</x:v>
       </x:c>
       <x:c r="H37" s="5" t="s">
         <x:v>225</x:v>
@@ -3488,8 +3491,8 @@
       <x:c r="F38" s="6" t="s">
         <x:v>230</x:v>
       </x:c>
-      <x:c r="G38" s="10" t="s">
-        <x:v>7</x:v>
+      <x:c r="G38" s="10" t="str">
+        <x:v>CONTRATO IMPLEMENTADO/BLOQUEADO</x:v>
       </x:c>
       <x:c r="H38" s="6" t="s">
         <x:v>231</x:v>
@@ -3517,8 +3520,8 @@
       <x:c r="F39" s="5" t="s">
         <x:v>236</x:v>
       </x:c>
-      <x:c r="G39" s="11" t="s">
-        <x:v>9</x:v>
+      <x:c r="G39" s="11" t="str">
+        <x:v>CONCLUÍDO</x:v>
       </x:c>
       <x:c r="H39" s="5" t="s">
         <x:v>237</x:v>
@@ -4417,7 +4420,7 @@
         <x:v>Calcular Weisz–Prater, Mears de massa e Mears térmico com entradas/unidades/fontes explícitas e estados passed, failed ou not_assessable_missing_inputs.</x:v>
       </x:c>
       <x:c r="G70" s="45" t="str">
-        <x:v>Concluído</x:v>
+        <x:v>PREPARADA/BLOQUEADA</x:v>
       </x:c>
       <x:c r="H70" s="44" t="str">
         <x:v>transport_diagnostics.py, contrato JSON v1, exemplo sintético, CLI e testes implementam Weisz–Prater, Mears de massa e Mears térmico com unidades SI, proveniência por campo, sensibilidade e estado não avaliável por entradas ausentes.</x:v>
@@ -4453,12 +4456,42 @@
       </x:c>
       <x:c r="I71" s="44" t="str">
         <x:v>Aprovar dados em FT-021; então definir protocolo de ajuste, conjunto de avaliação, critérios AIC/BIC e revisão humana.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="B72" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="C72" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="D72" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="E72" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="F72" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="G72" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="H72" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="I72" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:I2"/>
     <x:mergeCell ref="A3:I3"/>
+    <x:mergeCell ref="A72:I72"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="G5:G52">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Concluído"/>
@@ -4473,7 +4506,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bbcebbdef464ae5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbe55bc1cf8e427e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: aprovar FT-016 para uso interno contextual
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rde2ffdd633ae4be5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rb5a1ca0f4bc04bd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rab73fee90ba042f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R50a562ef56f94333"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3173,7 +3173,7 @@
         <x:v>170</x:v>
       </x:c>
       <x:c r="G27" s="9" t="str">
-        <x:v>Concluído</x:v>
+        <x:v>CONCLUÍDO — APROVADO PARA USO INTERNO CONTEXTUAL</x:v>
       </x:c>
       <x:c r="H27" s="5" t="str">
         <x:v>Balanços H/O usam espécies e bases explícitas, propagam incertezas independentes e bloqueiam avaliação total em base seca; documentação e testes positivos/negativos incluídos.</x:v>
@@ -4484,6 +4484,35 @@
         <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
       </x:c>
       <x:c r="I72" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="B73" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="C73" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="D73" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="E73" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="F73" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="G73" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="H73" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="I73" s="47" t="str">
         <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
       </x:c>
     </x:row>
@@ -4492,6 +4521,7 @@
     <x:mergeCell ref="A2:I2"/>
     <x:mergeCell ref="A3:I3"/>
     <x:mergeCell ref="A72:I72"/>
+    <x:mergeCell ref="A73:I73"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="G5:G52">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Concluído"/>
@@ -4506,7 +4536,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbe55bc1cf8e427e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec47eb178a6d4bd2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: aprovar FT-023 para uso interno contextual
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rab73fee90ba042f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R50a562ef56f94333"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R920c83c4a1d84066"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rc977acedb6fe4bf1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3376,7 +3376,7 @@
         <x:v>206</x:v>
       </x:c>
       <x:c r="G34" s="10" t="str">
-        <x:v>CONCLUÍDO COM BLOQUEIO</x:v>
+        <x:v>CONCLUÍDO — APROVADO PARA USO INTERNO CONTEXTUAL</x:v>
       </x:c>
       <x:c r="H34" s="6" t="s">
         <x:v>207</x:v>
@@ -4513,6 +4513,35 @@
         <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
       </x:c>
       <x:c r="I73" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="B74" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="C74" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="D74" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="E74" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="F74" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="G74" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="H74" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="I74" s="47" t="str">
         <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
       </x:c>
     </x:row>
@@ -4522,6 +4551,7 @@
     <x:mergeCell ref="A3:I3"/>
     <x:mergeCell ref="A72:I72"/>
     <x:mergeCell ref="A73:I73"/>
+    <x:mergeCell ref="A74:I74"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="G5:G52">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Concluído"/>
@@ -4536,7 +4566,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec47eb178a6d4bd2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4824dd8ac4984614"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: aprovar FT-021 e FT-022 para uso interno
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R920c83c4a1d84066"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rc977acedb6fe4bf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R4bd6e3a1e7a54bf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R8a88bc719a6f43da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3318,7 +3318,7 @@
         <x:v>194</x:v>
       </x:c>
       <x:c r="G32" s="10" t="str">
-        <x:v>CONCLUÍDO — USO INTERNO</x:v>
+        <x:v>CONCLUÍDO — APROVADO PARA USO INTERNO CONTEXTUAL</x:v>
       </x:c>
       <x:c r="H32" s="6" t="str">
         <x:v>reporting.py e a interface geram relatório científico Markdown v1 com fingerprint, premissas, resultados, fontes anexadas ou ausência explícita, prontidão, campos ausentes, limitações e bloqueio de recomendação.</x:v>
@@ -3347,7 +3347,7 @@
         <x:v>200</x:v>
       </x:c>
       <x:c r="G33" s="11" t="str">
-        <x:v>CONCLUÍDO COM BLOQUEIO</x:v>
+        <x:v>CONCLUÍDO — APROVADO PARA USO INTERNO CONTEXTUAL</x:v>
       </x:c>
       <x:c r="H33" s="5" t="s">
         <x:v>201</x:v>
@@ -4542,6 +4542,35 @@
         <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
       </x:c>
       <x:c r="I74" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="B75" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="C75" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="D75" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="E75" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="F75" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="G75" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="H75" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="I75" s="47" t="str">
         <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
       </x:c>
     </x:row>
@@ -4552,6 +4581,7 @@
     <x:mergeCell ref="A72:I72"/>
     <x:mergeCell ref="A73:I73"/>
     <x:mergeCell ref="A74:I74"/>
+    <x:mergeCell ref="A75:I75"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="G5:G52">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Concluído"/>
@@ -4566,7 +4596,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4824dd8ac4984614"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fcb312b0ff64c4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: atualizar planilha de atividades FT-021 a FT-023
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R4bd6e3a1e7a54bf9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R8a88bc719a6f43da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R7672c9770a2d4680"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rde807367b30642e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4574,6 +4574,35 @@
         <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
       </x:c>
     </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="B76" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="C76" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="D76" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="E76" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="F76" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="G76" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="H76" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="I76" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:I2"/>
@@ -4582,6 +4611,7 @@
     <x:mergeCell ref="A73:I73"/>
     <x:mergeCell ref="A74:I74"/>
     <x:mergeCell ref="A75:I75"/>
+    <x:mergeCell ref="A76:I76"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="G5:G52">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Concluído"/>
@@ -4596,7 +4626,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fcb312b0ff64c4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8df87c02cdcb43cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: alinhar status das atividades na planilha
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R7672c9770a2d4680"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rde807367b30642e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R5baa31d6af0e4c5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Ra792bfd294a24e25"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4603,6 +4603,35 @@
         <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
       </x:c>
     </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="B77" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="C77" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="D77" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="E77" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="F77" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="G77" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="H77" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="I77" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:I2"/>
@@ -4612,6 +4641,7 @@
     <x:mergeCell ref="A74:I74"/>
     <x:mergeCell ref="A75:I75"/>
     <x:mergeCell ref="A76:I76"/>
+    <x:mergeCell ref="A77:I77"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="G5:G52">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Concluído"/>
@@ -4626,7 +4656,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8df87c02cdcb43cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re18735edaad34dfd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: corrigir status FT-023 na planilha
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R5baa31d6af0e4c5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Ra792bfd294a24e25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R999065731bbf46f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rc9f26cfdc9264a0a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3144,7 +3144,7 @@
         <x:v>166</x:v>
       </x:c>
       <x:c r="G26" s="10" t="str">
-        <x:v>Concluído</x:v>
+        <x:v>CONCLUÍDO — APROVADO PARA USO INTERNO CONTEXTUAL</x:v>
       </x:c>
       <x:c r="H26" s="6" t="str">
         <x:v>elemental_balance.py e contrato JSON v1 calculam C de entrada/saída, residual, fechamento, desvio e tolerância configurável; CLI e exemplo sintético auditável incluídos; suíte completa aprovada.</x:v>
@@ -3173,7 +3173,7 @@
         <x:v>170</x:v>
       </x:c>
       <x:c r="G27" s="9" t="str">
-        <x:v>CONCLUÍDO — APROVADO PARA USO INTERNO CONTEXTUAL</x:v>
+        <x:v>GATE CONCLUÍDO/BLOQUEADO</x:v>
       </x:c>
       <x:c r="H27" s="5" t="str">
         <x:v>Balanços H/O usam espécies e bases explícitas, propagam incertezas independentes e bloqueiam avaliação total em base seca; documentação e testes positivos/negativos incluídos.</x:v>
@@ -3202,7 +3202,7 @@
         <x:v>174</x:v>
       </x:c>
       <x:c r="G28" s="8" t="str">
-        <x:v>GATE CONCLUÍDO/BLOQUEADO</x:v>
+        <x:v>CONCLUÍDO</x:v>
       </x:c>
       <x:c r="H28" s="6" t="s">
         <x:v>175</x:v>
@@ -3289,7 +3289,7 @@
         <x:v>190</x:v>
       </x:c>
       <x:c r="G31" s="10" t="str">
-        <x:v>CONCLUÍDO</x:v>
+        <x:v>CONCLUÍDO — APROVADO PARA USO INTERNO CONTEXTUAL</x:v>
       </x:c>
       <x:c r="H31" s="5" t="str">
         <x:v>reporting.py gera JSON canônico, resumo CSV, faixas ASF CSV e manifesto com SHA-256, tipo e tamanho. A interface oferece os downloads e os testes confirmam determinismo, integridade, round-trip e leitura dos CSVs.</x:v>
@@ -3376,7 +3376,7 @@
         <x:v>206</x:v>
       </x:c>
       <x:c r="G34" s="10" t="str">
-        <x:v>CONCLUÍDO — APROVADO PARA USO INTERNO CONTEXTUAL</x:v>
+        <x:v>PORTA IMPLEMENTADA/BLOQUEADA</x:v>
       </x:c>
       <x:c r="H34" s="6" t="s">
         <x:v>207</x:v>
@@ -3405,7 +3405,7 @@
         <x:v>212</x:v>
       </x:c>
       <x:c r="G35" s="9" t="str">
-        <x:v>PORTA IMPLEMENTADA/BLOQUEADA</x:v>
+        <x:v>CONCLUÍDO — INFRAESTRUTURA</x:v>
       </x:c>
       <x:c r="H35" s="5" t="s">
         <x:v>213</x:v>
@@ -3434,7 +3434,7 @@
         <x:v>218</x:v>
       </x:c>
       <x:c r="G36" s="11" t="str">
-        <x:v>CONCLUÍDO — INFRAESTRUTURA</x:v>
+        <x:v>CONCLUÍDO COM BLOQUEIO</x:v>
       </x:c>
       <x:c r="H36" s="6" t="s">
         <x:v>219</x:v>
@@ -3463,7 +3463,7 @@
         <x:v>224</x:v>
       </x:c>
       <x:c r="G37" s="9" t="str">
-        <x:v>CONCLUÍDO COM BLOQUEIO</x:v>
+        <x:v>CONTRATO IMPLEMENTADO/BLOQUEADO</x:v>
       </x:c>
       <x:c r="H37" s="5" t="s">
         <x:v>225</x:v>
@@ -3492,7 +3492,7 @@
         <x:v>230</x:v>
       </x:c>
       <x:c r="G38" s="10" t="str">
-        <x:v>CONTRATO IMPLEMENTADO/BLOQUEADO</x:v>
+        <x:v>CONCLUÍDO</x:v>
       </x:c>
       <x:c r="H38" s="6" t="s">
         <x:v>231</x:v>
@@ -4391,7 +4391,7 @@
         <x:v>Adicionar diluente, razão e partículas; geometria/porosidade; ativação completa; detectores, faixas, calibração, limites e recuperação da fração pesada.</x:v>
       </x:c>
       <x:c r="G69" s="46" t="str">
-        <x:v>Concluído</x:v>
+        <x:v>PREPARADA/BLOQUEADA</x:v>
       </x:c>
       <x:c r="H69" s="44" t="str">
         <x:v>experimental_protocol.py, schema v2, migração, template e exemplo sintético completo cobrem diluição, partículas, geometria, ativação, analytics e fontes por campo sem inventar valores ausentes.</x:v>
@@ -4629,6 +4629,35 @@
         <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
       </x:c>
       <x:c r="I77" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="B78" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="C78" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="D78" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="E78" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="F78" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="G78" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="H78" s="47" t="str">
+        <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
+      </x:c>
+      <x:c r="I78" s="47" t="str">
         <x:v>Atualizado em 2026-10-16: FT-017 a FT-028 revisadas. FT-017/017A e FT-024/027 permanecem bloqueadas por dados experimentais, calibração ou execução real.</x:v>
       </x:c>
     </x:row>
@@ -4642,6 +4671,7 @@
     <x:mergeCell ref="A75:I75"/>
     <x:mergeCell ref="A76:I76"/>
     <x:mergeCell ref="A77:I77"/>
+    <x:mergeCell ref="A78:I78"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="G5:G52">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Concluído"/>
@@ -4656,7 +4686,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re18735edaad34dfd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R637cd0ff8b8d4583"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: auditar e normalizar status do backlog
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2477,7 +2477,7 @@
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>CONCLUÍDO — APROVADO PARA USO INTERNO CONTEXTUAL</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>CONCLUÍDO</t>
+          <t>CONCLUÍDO — APROVADO PARA USO INTERNO CONTEXTUAL</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
@@ -2618,7 +2618,7 @@
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>CONCLUÍDO</t>
+          <t>GATE CONCLUÍDO/BLOQUEADO</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>CONTRATO IMPLEMENTADO/BLOQUEADO</t>
+          <t>CONCLUÍDO — INFRAESTRUTURA</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>CONCLUÍDO</t>
+          <t>CONCLUÍDO COM BLOQUEIO</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="G39" s="11" t="inlineStr">
         <is>
-          <t>CONCLUÍDO</t>
+          <t>CONTRATO IMPLEMENTADO/BLOQUEADO</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat: auditar validacao externa da FT-024
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rba77a31681d44b62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rc82247b263c74abf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Re7d16e8a75b64a2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R721f94fcc09b4299"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2951,13 +2951,13 @@
         </x:is>
       </x:c>
       <x:c r="G36" s="51" t="str">
-        <x:v>MODELO EXPLORATÓRIO / VALIDAÇÃO EXTERNA PENDENTE</x:v>
+        <x:v>MODELO EXPLORATÓRIO / VALIDAÇÃO EXTERNA COMPATÍVEL PENDENTE</x:v>
       </x:c>
       <x:c r="H36" s="52" t="str">
-        <x:v>FT024_FT027_EVIDENCIAS.md: 22 registros publicados, 14 LTFT; ajuste em 10 e avaliação em 4. MAE 0,013757 e RMSE 0,015509 mmol CO/(g cat min); intervalos preditivos.</x:v>
+        <x:v>FT024_FT027_EVIDENCIAS.md: 22 registros Co–Ce e 15 candidatos externos Co–Mn. A porta rejeitou o candidato por incompatibilidade de catalisador e alimentação; holdout interno documentado.</x:v>
       </x:c>
       <x:c r="I36" s="52" t="str">
-        <x:v>Obter campanha independente compatível e critérios de aceitação; manter recomendação bloqueada.</x:v>
+        <x:v>Obter campanha independente do mesmo sistema Co–Ce e domínio; definir critérios de aceitação; manter recomendação bloqueada.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="54" customHeight="1">
@@ -4673,7 +4673,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d7973b407754ce9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b3b92c8fc374ad9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: concluir caso e contrato HTFT FT-028 FT-029
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Re7d16e8a75b64a2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R721f94fcc09b4299"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R28cb7b1507f94307"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R66ea1ca6969f4247"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -439,7 +439,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="54">
+  <x:cellXfs count="55">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -581,6 +581,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -3126,20 +3129,14 @@
           <x:t xml:space="preserve">Escolher produto, base de seletividade, alimentação, reator, família e critérios de sucesso.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G40" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Parcial</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H40" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Planejamento e exemplo HTFT existem, mas o alvo inicial não foi formalmente aprovado.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I40" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Aprovar olefinas leves, gasolina ou outro alvo e registrar responsáveis.</x:t>
-        </x:is>
+      <x:c r="G40" s="54" t="str">
+        <x:v>CONCLUÍDO</x:v>
+      </x:c>
+      <x:c r="H40" s="52" t="str">
+        <x:v>ACEITE_FT_028_029.md e htft_light_olefins_v1.json: alvo C2–C4, condições de referência, respostas, estabilidade, fechamento e replicatas definidos.</x:v>
+      </x:c>
+      <x:c r="I40" s="52" t="str">
+        <x:v>Usar o caso como contrato diagnóstico; revisar limiares antes de execução e manter recomendação bloqueada.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="54" customHeight="1">
@@ -3173,20 +3170,14 @@
           <x:t xml:space="preserve">Modelar Fe/promotores, fases, O/P por Cn, coque, gradientes, WGS e reações secundárias.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G41" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Parcial</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H41" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Contrato v2 identifica HTFT e restringe a Fe, mas ainda não contém toda a taxonomia específica.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I41" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Criar schema HTFT dedicado e exemplos positivos/negativos.</x:t>
-        </x:is>
+      <x:c r="G41" s="54" t="str">
+        <x:v>CONCLUÍDO</x:v>
+      </x:c>
+      <x:c r="H41" s="53" t="str">
+        <x:v>htft-case-v1.schema.json cobre Fe/promotores/fases, O/P C2–C4, oxigenados, coque, gradiente e reações secundárias; exemplos positivo e negativo validados na CI.</x:v>
+      </x:c>
+      <x:c r="I41" s="53" t="str">
+        <x:v>Versionar o schema se o escopo mudar; avançar corpus e balanços HTFT em atividades próprias.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="54" customHeight="1">
@@ -4673,7 +4664,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b3b92c8fc374ad9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4741052228904de5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: concluir atividades HTFT FT-030 a FT-033
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R28cb7b1507f94307"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R66ea1ca6969f4247"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Re1076021ee934f4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rec196c74506f4b78"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -439,7 +439,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="55">
+  <x:cellXfs count="57">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -583,6 +583,12 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -3211,20 +3217,14 @@
           <x:t xml:space="preserve">Validar regime, temperatura e família; rejeitar combinações incompatíveis e manter recomendação bloqueada.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G42" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Concluído</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H42" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">domain.py, contrato v2 e testes rejeitam família LTFT no escopo HTFT e exigem regime consistente.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I42" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Estender o bloqueio a futuros modelos e datasets por identificador de regime.</x:t>
-        </x:is>
+      <x:c r="G42" s="55" t="str">
+        <x:v>CONCLUÍDO</x:v>
+      </x:c>
+      <x:c r="H42" s="52" t="str">
+        <x:v>Roteamento do caso e da evidência impede execução LTFT, calibração automática e transferência entre famílias incompatíveis.</x:v>
+      </x:c>
+      <x:c r="I42" s="52" t="str">
+        <x:v>Manter testes de não regressão ao adicionar novos modelos ou datasets.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="54" customHeight="1">
@@ -3258,20 +3258,14 @@
           <x:t xml:space="preserve">Curar estudos HTFT compatíveis, licenças, condições, produtos, fases e reações secundárias.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G43" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Bloqueado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H43" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Não existe corpus HTFT aprovado no repositório.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I43" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Definir protocolo de busca/extração após aprovação de FT-028/FT-029.</x:t>
-        </x:is>
+      <x:c r="G43" s="51" t="str">
+        <x:v>CONCLUÍDO — USO INTERNO CONTEXTUAL</x:v>
+      </x:c>
+      <x:c r="H43" s="53" t="str">
+        <x:v>Corpus HTFT separado com 8 registros Fe a 350 °C; auditor verifica manifesto, hash, envelope e fechamento. Calibração e ranking permanecem proibidos.</x:v>
+      </x:c>
+      <x:c r="I43" s="53" t="str">
+        <x:v>Confirmar licença antes de redistribuição externa; ampliar com estudos compatíveis revisados.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="54" customHeight="1">
@@ -3305,20 +3299,14 @@
           <x:t xml:space="preserve">Implementar balanços com WGS, carbono/coque e espécies secundárias.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G44" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Planejado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H44" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Não há contrato analítico nem módulo de balanços HTFT.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I44" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Executar após schema e corpus HTFT.</x:t>
-        </x:is>
+      <x:c r="G44" s="56" t="str">
+        <x:v>CONCLUÍDO — INFRAESTRUTURA</x:v>
+      </x:c>
+      <x:c r="H44" s="52" t="str">
+        <x:v>Contrato e módulo fecham C/H/O com CO₂, água, hidrocarbonetos, oxigenados, coque e não identificados; exemplo sintético e testes aprovados.</x:v>
+      </x:c>
+      <x:c r="I44" s="52" t="str">
+        <x:v>Aplicar a dados medidos quando houver ensaio HTFT completo.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="54" customHeight="1">
@@ -3352,20 +3340,14 @@
           <x:t xml:space="preserve">Oferecer seletor HTFT, valores iniciais compatíveis e avisos/bloqueio explícitos.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G45" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Concluído</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H45" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Streamlit contém regime HTFT, família Fe, temperatura inicial 320 °C e aviso de preparação; teste de interface cobre o estado.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I45" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Adicionar campos específicos HTFT quando FT-029 estiver concluída.</x:t>
-        </x:is>
+      <x:c r="G45" s="55" t="str">
+        <x:v>CONCLUÍDO</x:v>
+      </x:c>
+      <x:c r="H45" s="53" t="str">
+        <x:v>Interface HTFT mostra alvo C2–C4, 8 registros contextuais, requisitos analíticos e bloqueio; ASF é rotulada como referência matemática.</x:v>
+      </x:c>
+      <x:c r="I45" s="53" t="str">
+        <x:v>Manter recomendação bloqueada até validação HTFT independente na FT-034.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="54" customHeight="1">
@@ -4664,7 +4646,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4741052228904de5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74d21ef56c7b4b53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Implementa FT-034 a FT-037
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Re1076021ee934f4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="Rec196c74506f4b78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rabd0d2e5da5b47ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R5796366c0dfb42c2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3381,20 +3381,14 @@
           <x:t xml:space="preserve">Avaliar resíduos, incerteza, domínio, estabilidade, coque e transformação de fase.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G46" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Bloqueado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H46" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Faltam corpus, balanços e modelo HTFT.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I46" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Concluir FT-028 a FT-033 antes de iniciar validação.</x:t>
-        </x:is>
+      <x:c r="G46" s="51" t="str">
+        <x:v>PORTA IMPLEMENTADA / BLOQUEADA</x:v>
+      </x:c>
+      <x:c r="H46" s="52" t="str">
+        <x:v>ACEITE_FT_034_037.md: contrato e testes exigem modelo congelado, dataset externo compatível, métricas, incerteza, resíduos e parecer independente.</x:v>
+      </x:c>
+      <x:c r="I46" s="52" t="str">
+        <x:v>Implementar e congelar modelo HTFT; selecionar conjunto externo compatível; executar avaliação e obter revisão independente.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="54" customHeight="1">
@@ -3428,20 +3422,14 @@
           <x:t xml:space="preserve">Definir estrutura, proveniência, simetria, ocupação, carga, spin e estado de validação.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G47" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Planejado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H47" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DFT está documentado apenas como requisito; não há schema estrutural.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I47" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Criar schema e exemplos válidos/inválidos antes de qualquer gerador.</x:t>
-        </x:is>
+      <x:c r="G47" s="56" t="str">
+        <x:v>CONCLUÍDO COMO CONTRATO</x:v>
+      </x:c>
+      <x:c r="H47" s="53" t="str">
+        <x:v>Schema estrutural v1 exige célula, sítios, periodicidade, carga, spin, arquivo, SHA-256 e proveniência; exemplo identificado como sintético.</x:v>
+      </x:c>
+      <x:c r="I47" s="53" t="str">
+        <x:v>Na FT-038, consumir somente estruturas reais revisadas; não tratar o exemplo sintético como evidência científica.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="54" customHeight="1">
@@ -3475,20 +3463,14 @@
           <x:t xml:space="preserve">Definir faceta, terminação, slab, vácuo, supercélula, cobertura e sítios.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G48" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Planejado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H48" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Não há protocolo executável de superfície.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I48" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Aprovar protocolos separados para Co, Fe e carbetos relevantes.</x:t>
-        </x:is>
+      <x:c r="G48" s="56" t="str">
+        <x:v>CONCLUÍDO COMO PROTOCOLO</x:v>
+      </x:c>
+      <x:c r="H48" s="52" t="str">
+        <x:v>Protocolo v1 registra faceta, terminação, slab, vácuo, supercélula, camadas fixas, cobertura, método e testes de convergência.</x:v>
+      </x:c>
+      <x:c r="I48" s="52" t="str">
+        <x:v>Gerar slabs reais e fechar convergência de espessura, vácuo, malha k e cutoff antes de produção.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="54" customHeight="1">
@@ -3522,20 +3504,14 @@
           <x:t xml:space="preserve">Executar superfície limpa, adsorbato isolado e sistema adsorvido com parâmetros comparáveis.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G49" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Planejado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H49" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">A fórmula e requisitos estão no planejamento, mas não há implementação.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I49" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Definir adsorbatos, convenções e testes de consistência energética.</x:t>
-        </x:is>
+      <x:c r="G49" s="56" t="str">
+        <x:v>CONCLUÍDO COMO INFRAESTRUTURA</x:v>
+      </x:c>
+      <x:c r="H49" s="53" t="str">
+        <x:v>Cálculo aceita apenas superfície limpa, adsorbato isolado e sistema adsorvido convergidos sob a mesma impressão digital metodológica.</x:v>
+      </x:c>
+      <x:c r="I49" s="53" t="str">
+        <x:v>Integrar à engine na FT-038; substituir energias sintéticas por saídas reais e submetê-las à revisão científica.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="54" customHeight="1">
@@ -4646,7 +4622,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74d21ef56c7b4b53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd69b58ece3e2455f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Amplia base experimental da FT-024
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rabd0d2e5da5b47ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R5796366c0dfb42c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R0aadc94ce454421d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R4fea2227f4ea4ccd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2960,13 +2960,13 @@
         </x:is>
       </x:c>
       <x:c r="G36" s="51" t="str">
-        <x:v>MODELO EXPLORATÓRIO / VALIDAÇÃO EXTERNA COMPATÍVEL PENDENTE</x:v>
+        <x:v>BANCO AMPLIADO / VALIDAÇÃO EXTERNA COMPATÍVEL PENDENTE</x:v>
       </x:c>
       <x:c r="H36" s="52" t="str">
-        <x:v>FT024_FT027_EVIDENCIAS.md: 22 registros Co–Ce e 15 candidatos externos Co–Mn. A porta rejeitou o candidato por incompatibilidade de catalisador e alimentação; holdout interno documentado.</x:v>
+        <x:v>FT024_REFERENCIAS_E_CRITERIOS.md: 374 medições em 52 ensaios; critérios MAE, MSE/RMSE, resíduos e incerteza implementados. Apenas 22 ensaios usam o catalisador exato e são do estudo de calibração.</x:v>
       </x:c>
       <x:c r="I36" s="52" t="str">
-        <x:v>Obter campanha independente do mesmo sistema Co–Ce e domínio; definir critérios de aceitação; manter recomendação bloqueada.</x:v>
+        <x:v>Obter campanha independente do mesmo Co–Ce/SiO2, preparação e domínio; aplicar critérios congelados; manter recomendação bloqueada.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="54" customHeight="1">
@@ -4622,7 +4622,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd69b58ece3e2455f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75b55e5d5b4c41e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Implementa adaptador DFT FT-038 com pymatgen
</commit_message>
<xml_diff>
--- a/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
+++ b/docs/Planilha_Atividades_Plataforma_Fischer_Tropsch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R0aadc94ce454421d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R4fea2227f4ea4ccd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R7d15027fb2114e3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atividades" sheetId="2" r:id="R3c62aff0f29b43af"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="164" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="19">
+  <x:fonts count="20">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -145,8 +145,15 @@
       <x:name val="Arial"/>
       <x:family val="2"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF375623"/>
+      <x:name val="Arial"/>
+      <x:family val="2"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="27">
+  <x:fills count="29">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -276,6 +283,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFDCEFD8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -439,7 +456,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="57">
+  <x:cellXfs count="60">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -589,6 +606,15 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="28" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -958,10 +984,8 @@
       <x:c r="H2" s="13" t="n"/>
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
-      <x:c r="A3" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Situação verificada no repositório principal em 2026-10-14</x:t>
-        </x:is>
+      <x:c r="A3" s="14" t="str">
+        <x:v>Situação verificada no repositório principal em 2026-10-17</x:v>
       </x:c>
       <x:c r="B3" s="14" t="n"/>
       <x:c r="C3" s="14" t="n"/>
@@ -997,7 +1021,7 @@
         </x:is>
       </x:c>
       <x:c r="E5" s="16" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F5" s="12" t="n"/>
       <x:c r="G5" s="15" t="inlineStr">
@@ -1006,7 +1030,8 @@
         </x:is>
       </x:c>
       <x:c r="H5" s="17" t="n">
-        <x:v>0.4925373134328358</x:v>
+        <x:f>E5/B5</x:f>
+        <x:v>0.5074626865671642</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -1054,7 +1079,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" s="20" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C9" s="12" t="n"/>
       <x:c r="D9" s="12" t="n"/>
@@ -1086,7 +1111,7 @@
         </x:is>
       </x:c>
       <x:c r="B11" s="20" t="n">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C11" s="12" t="n"/>
       <x:c r="D11" s="12" t="n"/>
@@ -1304,15 +1329,11 @@
       <x:c r="H25" s="12" t="n"/>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
-      <x:c r="A26" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Validação</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B26" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">tests/ — 123 testes e 15 subtestes; 15 schemas, 14 exemplos e 6 notebooks aprovados na conclusão de FT-019/FT-020 em 2026-10-14</x:t>
-        </x:is>
+      <x:c r="A26" s="21" t="str">
+        <x:v>Validação</x:v>
+      </x:c>
+      <x:c r="B26" s="21" t="str">
+        <x:v>tests/ — 164 testes e 15 subtestes; 22 schemas, 23 exemplos e 6 notebooks aprovados em 2026-10-17</x:v>
       </x:c>
       <x:c r="C26" s="12" t="n"/>
       <x:c r="D26" s="12" t="n"/>
@@ -1340,15 +1361,11 @@
       <x:c r="H27" s="12" t="n"/>
     </x:row>
     <x:row r="28" ht="20" customHeight="1">
-      <x:c r="A28" s="27" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Expansão planejada</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B28" s="27" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Próximo: qualificar e aprovar dados em FT-021; FT-017/FT-017A permanecem limitadas enquanto não houver distribuição experimental aprovada</x:t>
-        </x:is>
+      <x:c r="A28" s="27" t="str">
+        <x:v>Expansão planejada</x:v>
+      </x:c>
+      <x:c r="B28" s="27" t="str">
+        <x:v>Próximo: FT-039, parser de saída DFT; FT-024 e FT-027 continuam dependentes de execução experimental independente.</x:v>
       </x:c>
       <x:c r="C28" s="12" t="n"/>
       <x:c r="D28" s="12" t="n"/>
@@ -3545,20 +3562,14 @@
           <x:t xml:space="preserve">Mapear contrato para engine, validar sintaxe e registrar versão/pseudopotenciais/bases.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G50" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Planejado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H50" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Nenhum engine ou adaptador foi aprovado/implementado.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I50" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Escolher engine e criar adaptador somente após FT-035 a FT-037.</x:t>
-        </x:is>
+      <x:c r="G50" s="59" t="str">
+        <x:v>CONCLUÍDO COMO INFRAESTRUTURA</x:v>
+      </x:c>
+      <x:c r="H50" s="52" t="str">
+        <x:v>dft_engine.py e schema ft-dft-engine-input-v1: adaptador VASP via pymatgen gera POSCAR, INCAR e KPOINTS determinísticos, manifesto versionado, hashes e bloqueio explícito; 5 testes dedicados.</x:v>
+      </x:c>
+      <x:c r="I50" s="52" t="str">
+        <x:v>Implementar FT-039 para interpretar convergência e erros; antes de execução real, anexar e auditar POTCAR licenciado, potenciais e hashes.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="54" customHeight="1">
@@ -4622,7 +4633,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75b55e5d5b4c41e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaeed40b30ad4320"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>